<commit_message>
chore: Update song list to Aug.28, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,56 +413,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J889"/>
+  <dimension ref="A1:J899"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>歌名</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>歌名翻译</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>原唱</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>语言</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>次数</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>歌切</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>标签</t>
         </is>
@@ -539,7 +527,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/09，2025/11/14，2025/12/24，2025/12/26，2026/01/16，2026/01/24，2026/01/28，2026/01/30，2026/02/10，2026/02/14，2026/03/09，2026/03/27，2026/04/01，2026/04/14，2026/04/24，2026/06/12，2026/07/22，2026/08/11</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/02，2025/09/07，2025/09/17，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/09，2025/11/14，2025/12/24，2025/12/26，2026/01/16，2026/01/24，2026/01/28，2026/01/30，2026/02/10，2026/02/14，2026/03/09，2026/03/27，2026/04/01，2026/04/14，2026/04/24，2026/06/12，2026/07/22，2026/08/11</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -583,7 +571,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/07，2026/01/14，2026/01/24，2026/02/19，2026/03/07，2026/03/15，2026/06/06，2026/06/23，2026/08/05，2026/08/05</t>
+          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/07，2026/01/14，2026/01/24，2026/02/19，2026/03/07，2026/03/15，2026/06/06，2026/06/23，2026/08/05，2026/08/05，2026/08/19</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -594,7 +582,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -631,7 +619,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/01/19，2026/01/21，2026/03/04，2026/04/16，2026/06/06，2026/06/18，2026/06/23</t>
+          <t>2025/03/02，2025/03/25，2025/03/28，2025/04/17，2025/05/03，2025/05/09，2025/05/16，2025/05/30，2025/06/14，2025/06/19，2025/07/05，2025/07/18，2025/08/21，2025/08/25，2025/09/05，2025/09/22，2025/09/26，2026/01/19，2026/01/21，2026/03/04，2026/04/16，2026/06/06，2026/06/18，2026/06/23，2026/08/25</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -642,7 +630,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -675,7 +663,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/09，2025/12/11，2026/01/15，2026/02/12，2026/04/19，2026/08/08</t>
+          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/09，2025/12/11，2026/01/15，2026/02/12，2026/04/19，2026/08/08，2026/8/28</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -686,7 +674,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -839,7 +827,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/04/04，2025/04/14，2025/04/20，2025/04/24，2025/05/09，2025/05/18，2025/05/29，2025/06/06，2025/08/01，2025/09/21，2025/10/10，2025/11/28，2025/12/08，2025/12/30，2026/04/26，2026/07/09，2026/07/31</t>
+          <t>2025/03/03，2025/04/04，2025/04/14，2025/04/20，2025/04/24，2025/05/09，2025/05/18，2025/05/29，2025/06/06，2025/08/01，2025/09/21，2025/10/10，2025/11/28，2025/12/08，2025/12/30，2026/04/26，2026/07/09，2026/07/31，2026/08/25</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -850,7 +838,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -963,7 +951,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/04，2026/01/24，2026/01/24，2026/02/19，2026/02/25，2026/03/13，2026/04/08，2026/06/10，2026/07/27</t>
+          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/04，2026/01/24，2026/01/24，2026/02/19，2026/02/25，2026/03/13，2026/04/08，2026/06/10，2026/07/27，2026/08/18</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -974,7 +962,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1003,7 +991,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/07，2025/12/17，2026/01/19，2026/01/29，2026/02/10，2026/02/12，2026/03/22，2026/04/18，2026/05/10，2026/06/06，2026/06/25，2026/07/17</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/07，2025/12/17，2026/01/19，2026/01/29，2026/02/10，2026/02/12，2026/03/22，2026/04/18，2026/05/10，2026/06/06，2026/06/25，2026/07/17，2026/8/28</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1014,7 +1002,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1283,7 +1271,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/09，2025/12/16，2026/02/14，2026/03/07，2026/03/17，2026/03/21，2026/05/01，2026/07/04，2026/07/26</t>
+          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/09，2025/12/16，2026/02/14，2026/03/07，2026/03/17，2026/03/21，2026/05/01，2026/07/04，2026/07/26，2026/8/28</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1294,7 +1282,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1323,7 +1311,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/09，2025/05/29，2025/06/28，2025/08/08，2025/08/21，2025/09/15，2025/10/24，2025/12/17，2026/01/15，2026/02/14，2026/03/04，2026/04/09</t>
+          <t>2025/03/04，2025/05/09，2025/05/29，2025/06/28，2025/08/08，2025/08/21，2025/09/15，2025/10/24，2025/12/17，2026/01/15，2026/02/14，2026/03/04，2026/04/09，2026/08/25</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1334,7 +1322,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1363,7 +1351,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/09，2025/11/12，2025/11/27，2025/12/04，2025/12/28，2026/01/22，2026/02/02，2026/02/23，2026/03/25，2026/04/16，2026/05/06，2026/05/21，2026/07/10，2026/07/15</t>
+          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/09，2025/11/12，2025/11/27，2025/12/04，2025/12/28，2026/01/22，2026/02/02，2026/02/23，2026/03/25，2026/04/16，2026/05/06，2026/05/21，2026/07/10，2026/07/15，2026/08/21，2026/8/28，2026/8/28</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1374,7 +1362,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1443,7 +1431,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/01/03，2026/03/25，2026/05/10，2026/06/20，2026/8/16</t>
+          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/01/03，2026/03/25，2026/05/10，2026/06/20，2026/08/16</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1523,7 +1511,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/09，2025/12/30，2026/02/20，2026/02/23，2026/03/04，2026/04/11，2026/04/16，2026/04/23，2026/06/14，2026/07/04，2026/07/31</t>
+          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/09，2025/12/30，2026/02/20，2026/02/23，2026/03/04，2026/04/11，2026/04/16，2026/04/23，2026/06/14，2026/07/04，2026/07/31，2026/08/25</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1534,7 +1522,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1563,7 +1551,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/01，2025/11/09，2025/11/21，2025/12/08，2026/01/15，2026/01/24，2026/03/04，2026/03/14，2026/05/06，2026/05/16，2026/05/20，2026/06/12，2026/07/16，2026/07/26，2026/07/31</t>
+          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/01，2025/11/09，2025/11/21，2025/12/08，2026/01/15，2026/01/24，2026/03/04，2026/03/14，2026/05/06，2026/05/16，2026/05/20，2026/06/12，2026/07/16，2026/07/26，2026/07/31，2026/8/28</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1574,7 +1562,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1643,7 +1631,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/12，2025/09/17，2025/09/02，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/05，2025/11/14，2025/11/21，2025/11/28，2025/12/08，2025/12/17，2026/01/10，2026/01/22，2026/02/10，2026/02/14，2026/02/14，2026/02/27，2026/03/28，2026/04/09，2026/04/14，2026/05/06，2026/05/23，2026/06/06，2026/06/25，2026/07/09，2026/07/16，2026/07/27</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/02，2025/09/12，2025/09/17，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/05，2025/11/14，2025/11/21，2025/11/28，2025/12/08，2025/12/17，2026/01/10，2026/01/22，2026/02/10，2026/02/14，2026/02/14，2026/02/27，2026/03/28，2026/04/09，2026/04/14，2026/05/06，2026/05/23，2026/06/06，2026/06/25，2026/07/09，2026/07/16，2026/07/27，2026/08/21</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1654,7 +1642,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1683,7 +1671,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/01，2025/11/28，2025/12/12，2026/01/05，2026/01/22，2026/03/04，2026/03/08，2026/03/22，2026/04/22，2026/04/24，2026/05/10，2026/05/23，2026/06/10，2026/06/15，2026/07/31，2026/08/11</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/01，2025/11/28，2025/12/12，2026/01/05，2026/01/22，2026/03/04，2026/03/08，2026/03/22，2026/04/22，2026/04/24，2026/05/10，2026/05/23，2026/06/10，2026/06/15，2026/07/31，2026/08/11，2026/08/25</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1694,7 +1682,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2255,7 +2243,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/07，2025/11/09，2025/12/02，2026/01/21，2026/03/05，2026/04/16，2026/06/23，2026/07/05，2026/08/05，2026/08/05</t>
+          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/07，2025/11/09，2025/12/02，2026/01/21，2026/03/05，2026/04/16，2026/06/23，2026/07/05，2026/08/05，2026/08/05，2026/08/19</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2266,7 +2254,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2635,7 +2623,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/05/04，2025/05/18，2025/06/09，2025/08/04，2025/08/16，2025/09/18，2025/10/17，2025/11/21，2025/11/28，2026/05/10</t>
+          <t>2025/03/07，2025/03/28，2025/05/04，2025/05/18，2025/06/09，2025/08/04，2025/08/16，2025/09/18，2025/10/17，2025/11/21，2025/11/28，2026/05/10，2026/8/27</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2646,7 +2634,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2755,7 +2743,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/07，2025/11/19，2025/11/26，2025/12/30，2026/01/28，2026/02/14，2026/03/13，2026/04/10，2026/05/23，2026/06/18，2026/06/29，2026/07/25</t>
+          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/07，2025/11/19，2025/11/26，2025/12/30，2026/01/28，2026/02/14，2026/03/13，2026/04/10，2026/05/23，2026/06/18，2026/06/29，2026/07/25，2026/08/25</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -2766,7 +2754,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2883,7 +2871,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/04，2025/12/24，2026/01/15，2026/02/23，2026/03/08，2026/04/14，2026/05/04，2026/05/23，2026/06/14，2026/07/27</t>
+          <t>2025/03/07，2025/03/17，2025/03/28，2025/03/29，2025/04/13，2025/04/15，2025/04/18，2025/04/28，2025/05/22，2025/06/02，2025/06/03，2025/06/10，2025/06/12，2025/06/20，2025/06/20，2025/06/27，2025/07/05，2025/07/09，2025/07/13，2025/08/04，2025/08/08，2025/08/12，2025/08/24，2025/09/06，2025/10/07，2025/10/24，2025/11/24，2025/12/04，2025/12/24，2026/01/15，2026/02/23，2026/03/08，2026/04/14，2026/05/04，2026/05/23，2026/06/14，2026/07/27，2026/08/18</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -2894,7 +2882,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -2923,7 +2911,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/04，2025/04/12，2025/04/18，2025/04/24，2025/06/17，2025/06/19，2025/07/11，2025/07/18，2025/08/28，2025/09/05，2025/09/08，2025/09/27，2025/10/03，2025/12/11，2025/12/30，2026/01/21，2026/01/25，2026/02/10，2026/02/23，2026/03/06，2026/03/22，2026/04/24</t>
+          <t>2025/03/07，2025/04/04，2025/04/12，2025/04/18，2025/04/24，2025/06/17，2025/06/19，2025/07/11，2025/07/18，2025/08/28，2025/09/05，2025/09/08，2025/09/27，2025/10/03，2025/12/11，2025/12/30，2026/01/21，2026/01/25，2026/02/10，2026/02/23，2026/03/06，2026/03/22，2026/04/24，2026/08/19</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -2934,7 +2922,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -2963,7 +2951,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/01，2025/11/09，2025/12/04，2025/12/16，2025/12/31，2026/01/09，2026/01/15，2026/01/21，2026/01/23，2026/01/29，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/02/24，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/05，2026/03/07，2026/03/08，2026/03/09，2026/03/12，2026/03/13，2026/03/14，2026/03/15，2026/03/17，2026/03/18，2026/03/19，2026/03/22，2026/03/24，2026/03/27，2026/03/28，2026/03/31，2026/04/08，2026/04/14，2026/04/18，2026/04/25，2026/05/01，2026/05/15，2026/05/25，2026/06/12，2026/06/23，2026/06/26，2026/07/04，2026/07/20，2026/07/30，2026/08/09</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/01，2025/11/09，2025/12/04，2025/12/16，2025/12/31，2026/01/09，2026/01/15，2026/01/21，2026/01/23，2026/01/29，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/02/24，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/05，2026/03/07，2026/03/08，2026/03/09，2026/03/12，2026/03/13，2026/03/14，2026/03/15，2026/03/17，2026/03/18，2026/03/19，2026/03/22，2026/03/24，2026/03/27，2026/03/28，2026/03/31，2026/04/08，2026/04/14，2026/04/18，2026/04/25，2026/05/01，2026/05/15，2026/05/25，2026/06/12，2026/06/23，2026/06/26，2026/07/04，2026/07/20，2026/07/30，2026/08/09，2026/8/28</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2962,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>73</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3091,7 +3079,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/05/01，2025/05/09，2025/05/26，2025/06/17，2025/06/20，2025/07/13，2025/09/12，2025/09/26，2025/10/11，2025/12/08，2026/01/12，2026/01/30，2026/02/07，2026/04/18，2026/05/23，2026/07/18</t>
+          <t>2025/03/07，2025/05/01，2025/05/09，2025/05/26，2025/06/17，2025/06/20，2025/07/13，2025/09/12，2025/09/26，2025/10/11，2025/12/08，2026/01/12，2026/01/30，2026/02/07，2026/04/18，2026/05/23，2026/07/18，2026/08/21，2026/8/28</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -3102,7 +3090,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3171,7 +3159,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/04/09，2026/05/10，2026/06/12，2026/07/27</t>
+          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/04/09，2026/05/10，2026/06/12，2026/07/27，2026/8/28</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3182,7 +3170,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3211,7 +3199,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/02/02，2026/02/12，2026/04/14，2026/04/22，2026/06/10</t>
+          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/02/02，2026/02/12，2026/04/14，2026/04/22，2026/06/10，2026/8/28</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3222,7 +3210,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3339,7 +3327,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/01，2026/01/16，2026/02/02，2026/02/23，2026/03/08，2026/03/19，2026/03/21，2026/04/16，2026/05/10，2026/06/14，2026/07/25，2026/08/07</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/01，2026/01/16，2026/02/02，2026/02/23，2026/03/08，2026/03/19，2026/03/21，2026/04/16，2026/05/10，2026/06/14，2026/07/25，2026/08/07，2026/08/25</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3350,7 +3338,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3503,7 +3491,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/04，2025/04/28，2025/07/08，2025/07/21，2025/08/18，2026/02/09，2026/04/08</t>
+          <t>2025/03/09，2025/04/04，2025/04/28，2025/07/08，2025/07/21，2025/08/18，2026/02/09，2026/04/08，2026/08/21</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3514,7 +3502,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3631,7 +3619,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/05/05，2025/05/13，2025/05/24，2025/08/12，2025/08/30，2025/11/26</t>
+          <t>2025/03/10，2025/05/05，2025/05/13，2025/05/24，2025/08/12，2025/08/30，2025/11/26，2026/08/21</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3642,7 +3630,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -3671,7 +3659,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/05/03，2025/06/19，2026/01/19，2026/06/23</t>
+          <t>2025/03/12，2025/05/03，2025/06/19，2026/01/19，2026/06/23，2026/08/21</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -3682,7 +3670,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -3875,7 +3863,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/04，2025/11/07，2025/11/09，2025/12/04，2026/01/09，2026/01/19，2026/01/21，2026/01/25，2026/03/04，2026/03/07，2026/03/14，2026/06/06，2026/06/19，2026/08/05，2026/08/05</t>
+          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/04，2025/11/07，2025/11/09，2025/12/04，2026/01/09，2026/01/19，2026/01/21，2026/01/25，2026/03/04，2026/03/07，2026/03/14，2026/06/06，2026/06/19，2026/08/05，2026/08/05，2026/08/19</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -3886,7 +3874,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -3967,7 +3955,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/13，2025/05/01，2025/05/06，2025/05/24，2025/06/09，2025/06/24，2025/07/08，2025/08/19，2025/08/16，2025/09/08，2025/10/07，2025/10/28，2025/11/18，2025/12/11，2026/01/14，2026/02/04，2026/05/20，2026/07/09</t>
+          <t>2025/03/12，2025/04/13，2025/05/01，2025/05/06，2025/05/24，2025/06/09，2025/06/24，2025/07/08，2025/08/16，2025/08/19，2025/09/08，2025/10/07，2025/10/28，2025/11/18，2025/12/11，2026/01/14，2026/02/04，2026/05/20，2026/07/09</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4287,7 +4275,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/09，2026/01/23，2026/02/18，2026/04/09，2026/06/15，2026/07/22</t>
+          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/09，2026/01/23，2026/02/18，2026/04/09，2026/06/15，2026/07/22，2026/8/28</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4298,7 +4286,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4407,7 +4395,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/02/10，2026/02/24，2026/03/18，2026/05/20，2026/06/19</t>
+          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/02/10，2026/02/24，2026/03/18，2026/05/20，2026/06/19，2026/08/25</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4418,7 +4406,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -4607,7 +4595,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/09，2026/03/25，2026/04/26，2026/06/15</t>
+          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/09，2026/03/25，2026/04/26，2026/06/15，2026/08/25</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4618,7 +4606,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -4767,7 +4755,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/01/12，2026/02/07，2026/03/15，2026/04/19，2026/06/26</t>
+          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/01/12，2026/02/07，2026/03/15，2026/04/19，2026/06/26，2026/08/25</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -4778,7 +4766,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5099,7 +5087,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/09，2026/01/15，2026/02/19，2026/03/13，2026/03/15，2026/03/21，2026/06/14，2026/06/17，2026/07/20，2026/07/31</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/09，2026/01/15，2026/02/19，2026/03/13，2026/03/15，2026/03/21，2026/06/14，2026/06/17，2026/07/20，2026/07/31，2026/08/21，2026/8/28</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5110,7 +5098,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5139,7 +5127,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/01/19，2026/04/18，2026/05/01，2026/05/23，2026/07/17</t>
+          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/01/19，2026/04/18，2026/05/01，2026/05/23，2026/07/17，2026/08/25</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5150,7 +5138,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5219,7 +5207,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/28，2025/04/18，2025/09/20，2025/10/12，2025/10/22，2026/01/02，2026/01/30，2026/04/09，2026/07/31</t>
+          <t>2025/03/14，2025/03/28，2025/04/18，2025/09/20，2025/10/12，2025/10/22，2026/01/02，2026/01/30，2026/04/09，2026/07/31，2026/8/27</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5230,7 +5218,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -5259,7 +5247,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/03，2025/11/24，2026/04/09，2026/04/14，2026/04/24，2026/05/23，2026/08/02</t>
+          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/03，2025/11/24，2026/04/09，2026/04/14，2026/04/24，2026/05/23，2026/08/02，2026/8/27</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5270,7 +5258,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5619,7 +5607,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/08，2025/12/12，2026/02/14，2026/03/12，2026/04/09，2026/05/10，2026/05/23，2026/06/06，2026/06/25，2026/07/18</t>
+          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/08，2025/12/12，2026/02/14，2026/03/12，2026/04/09，2026/05/10，2026/05/23，2026/06/06，2026/06/25，2026/07/18，2026/08/25，2026/8/28</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -5630,7 +5618,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -5659,7 +5647,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/05/12，2025/06/23，2025/09/04，2025/12/23，2026/05/05，2026/07/16</t>
+          <t>2025/03/15，2025/05/12，2025/06/23，2025/09/04，2025/12/23，2026/05/05，2026/07/16，2026/08/25</t>
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -5670,7 +5658,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -5699,7 +5687,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2025/03/16，2025/04/17，2025/05/08，2025/09/11，2025/10/03，2025/10/16，2025/11/19，2026/02/07，2026/06/23</t>
+          <t>2025/03/16，2025/04/17，2025/05/08，2025/09/11，2025/10/03，2025/10/16，2025/11/19，2026/02/07，2026/06/23，2026/08/18</t>
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -5710,7 +5698,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -5739,7 +5727,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/07，2025/12/23，2026/01/05，2026/01/21，2026/01/29，2026/02/09，2026/02/20，2026/02/23，2026/03/04，2026/03/06，2026/03/07，2026/04/11，2026/04/14，2026/04/29，2026/05/23，2026/07/03，2026/07/21，2026/08/11</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/07，2025/12/23，2026/01/05，2026/01/21，2026/01/29，2026/02/09，2026/02/20，2026/02/23，2026/03/04，2026/03/06，2026/03/07，2026/04/11，2026/04/14，2026/04/29，2026/05/23，2026/07/03，2026/07/21，2026/08/11，2026/08/25</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5750,7 +5738,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -6059,7 +6047,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/12，2025/09/02，2025/11/09，2025/12/04，2026/01/01，2026/01/29，2026/04/09，2026/06/15，2026/08/05</t>
+          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/02，2025/09/12，2025/11/09，2025/12/04，2026/01/01，2026/01/29，2026/04/09，2026/06/15，2026/08/05</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -6099,7 +6087,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08，2026/08/23</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6110,7 +6098,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6139,7 +6127,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/05/22，2025/07/10，2025/09/08，2025/10/09，2025/11/01，2026/01/15，2026/04/08，2026/8/16</t>
+          <t>2025/03/18，2025/03/25，2025/05/22，2025/07/10，2025/09/08，2025/10/09，2025/11/01，2026/01/15，2026/04/08，2026/08/16</t>
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
@@ -6259,7 +6247,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/05，2025/04/24，2025/05/12，2025/06/19，2025/07/11，2025/07/31，2025/09/03，2025/09/20，2025/10/17，2025/11/09，2025/11/21，2026/01/15</t>
+          <t>2025/03/19，2025/04/05，2025/04/24，2025/05/12，2025/06/19，2025/07/11，2025/07/31，2025/09/03，2025/09/20，2025/10/17，2025/11/09，2025/11/21，2026/01/15，2026/8/27</t>
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -6270,7 +6258,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -6419,7 +6407,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/04，2026/01/03，2026/02/10，2026/03/13，2026/03/22，2026/04/14，2026/06/17</t>
+          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/04，2026/01/03，2026/02/10，2026/03/13，2026/03/22，2026/04/14，2026/06/17，2026/08/25</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -6430,7 +6418,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6499,7 +6487,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/01/01，2026/01/09，2026/03/22，2026/04/09，2026/04/20，2026/05/25，2026/06/10，2026/06/19，2026/08/11</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/01/01，2026/01/09，2026/03/22，2026/04/09，2026/04/20，2026/05/25，2026/06/10，2026/06/19，2026/08/11，2026/8/28，2026/8/28</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6510,7 +6498,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -6539,7 +6527,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/17，2025/05/20，2025/05/31，2025/09/15，2025/10/13，2025/10/22，2025/12/24，2026/04/26，2026/06/19，2026/06/20</t>
+          <t>2025/03/19，2025/04/17，2025/05/20，2025/05/31，2025/09/15，2025/10/13，2025/10/22，2025/12/24，2026/04/26，2026/06/19，2026/06/20，2026/8/28</t>
         </is>
       </c>
       <c r="F150" t="inlineStr"/>
@@ -6550,7 +6538,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -6579,7 +6567,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/06/03，2026/8/16</t>
+          <t>2025/03/20，2025/06/03，2026/08/16</t>
         </is>
       </c>
       <c r="F151" t="inlineStr"/>
@@ -6663,7 +6651,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/02，2026/01/16，2026/02/02，2026/02/23，2026/02/25，2026/03/17，2026/04/08，2026/05/06，2026/05/21，2026/06/25，2026/07/18</t>
+          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/02，2026/01/16，2026/02/02，2026/02/23，2026/02/25，2026/03/17，2026/04/08，2026/05/06，2026/05/21，2026/06/25，2026/07/18，2026/08/25</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -6674,7 +6662,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -6743,7 +6731,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/23，2025/07/21，2025/08/08，2025/09/05，2026/01/29</t>
+          <t>2025/03/20，2025/05/23，2025/07/21，2025/08/08，2025/09/05，2026/01/29，2026/08/25</t>
         </is>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -6754,7 +6742,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -6823,7 +6811,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/08，2026/01/23，2026/01/26，2026/02/07，2026/02/10，2026/02/23，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/13，2026/03/24，2026/03/28，2026/03/29，2026/04/27，2026/05/02，2026/06/18，2026/07/04，2026/07/31</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/16，2025/08/26，2025/09/21，2025/10/03，2025/11/12，2025/12/08，2026/01/23，2026/01/26，2026/02/07，2026/02/10，2026/02/23，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/13，2026/03/24，2026/03/28，2026/03/29，2026/04/27，2026/05/02，2026/06/18，2026/07/04，2026/07/31，2026/08/25，2026/8/28</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6834,7 +6822,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -6987,7 +6975,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/17，2025/05/01，2025/05/03，2025/05/18，2025/05/22，2025/05/29，2025/06/06，2025/06/13，2025/06/30，2025/07/09，2025/07/27，2025/08/23，2025/09/03，2025/09/11，2025/10/11，2025/10/17，2025/12/24，2026/01/16，2026/02/07，2026/03/28，2026/8/16</t>
+          <t>2025/03/20，2025/04/17，2025/05/01，2025/05/03，2025/05/18，2025/05/22，2025/05/29，2025/06/06，2025/06/13，2025/06/30，2025/07/09，2025/07/27，2025/08/23，2025/09/03，2025/09/11，2025/10/11，2025/10/17，2025/12/24，2026/01/16，2026/02/07，2026/03/28，2026/08/16</t>
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -7027,7 +7015,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/08，2025/12/26，2026/01/05，2026/01/24，2026/02/05，2026/02/14，2026/03/09，2026/03/28，2026/04/26，2026/05/05，2026/05/23，2026/06/12</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/08，2025/12/26，2026/01/05，2026/01/24，2026/02/05，2026/02/14，2026/03/09，2026/03/28，2026/04/26，2026/05/05，2026/05/23，2026/06/12，2026/8/27</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -7038,7 +7026,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -7223,7 +7211,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/19，2025/06/13，2025/07/22，2025/07/23，2025/08/25，2025/09/12，2025/10/26，2025/12/17，2026/02/09，2026/03/04，2026/03/25，2026/03/29，2026/05/23</t>
+          <t>2025/03/21，2025/05/19，2025/06/13，2025/07/22，2025/07/23，2025/08/25，2025/09/12，2025/10/26，2025/12/17，2026/02/09，2026/03/04，2026/03/25，2026/03/29，2026/05/23，2026/08/25</t>
         </is>
       </c>
       <c r="F167" t="inlineStr"/>
@@ -7234,7 +7222,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -7423,7 +7411,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/03/29，2025/04/25，2025/05/30，2025/06/22，2025/07/18，2025/09/03，2025/09/13，2026/04/16</t>
+          <t>2025/03/21，2025/03/29，2025/04/25，2025/05/30，2025/06/22，2025/07/18，2025/09/03，2025/09/13，2026/04/16，2026/08/23</t>
         </is>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -7434,7 +7422,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -7499,7 +7487,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/09/28</t>
+          <t>2025/03/21，2025/09/28，2026/8/27</t>
         </is>
       </c>
       <c r="F174" t="inlineStr"/>
@@ -7510,7 +7498,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -7539,7 +7527,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11，2026/8/28</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7550,7 +7538,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -7623,7 +7611,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/08，2026/02/18，2026/03/06，2026/03/13，2026/03/14，2026/03/31，2026/05/01，2026/06/28，2026/07/17，2026/08/02</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/08，2026/02/18，2026/03/06，2026/03/13，2026/03/14，2026/03/31，2026/05/01，2026/06/28，2026/07/17，2026/08/02，2026/08/21</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7634,7 +7622,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -7747,7 +7735,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/01/19，2026/03/09，2026/04/18，2026/04/20，2026/05/10，2026/06/19，2026/06/26，2026/07/27</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/01/19，2026/03/09，2026/04/18，2026/04/20，2026/05/10，2026/06/19，2026/06/26，2026/07/27，2026/8/28</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7758,7 +7746,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -7867,7 +7855,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/05，2025/05/18，2025/06/12，2025/07/14，2025/07/15，2025/08/02，2025/08/30，2025/10/03，2025/11/01，2025/11/26，2025/12/02，2026/02/14，2026/07/09</t>
+          <t>2025/03/21，2025/04/05，2025/05/18，2025/06/12，2025/07/14，2025/07/15，2025/08/02，2025/08/30，2025/10/03，2025/11/01，2025/11/26，2025/12/02，2026/02/14，2026/07/09，2026/08/25</t>
         </is>
       </c>
       <c r="F183" t="inlineStr"/>
@@ -7878,7 +7866,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -7907,7 +7895,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/02，2025/12/05，2025/12/30，2026/01/23，2026/01/29，2026/02/23，2026/03/17，2026/03/22，2026/04/19，2026/05/10，2026/06/12，2026/07/22，2026/08/08</t>
+          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/02，2025/12/05，2025/12/30，2026/01/23，2026/01/29，2026/02/23，2026/03/17，2026/03/22，2026/04/19，2026/05/10，2026/06/12，2026/07/22，2026/08/08，2026/8/28，2026/8/28</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -7918,7 +7906,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>39</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -8147,7 +8135,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/04/10，2025/05/01，2025/05/19，2025/06/08，2025/07/14，2025/09/12，2025/09/11，2025/10/31，2026/01/09，2026/07/05</t>
+          <t>2025/03/23，2025/04/10，2025/05/01，2025/05/19，2025/06/08，2025/07/14，2025/09/11，2025/09/12，2025/10/31，2026/01/09，2026/07/05</t>
         </is>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -8587,7 +8575,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/03/25，2026/06/23</t>
+          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/03/25，2026/06/23，2026/08/21</t>
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -8598,7 +8586,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -8867,7 +8855,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/24，2025/05/13，2025/06/02，2025/06/27，2025/07/14，2025/08/26，2025/09/02，2025/10/03，2025/10/17，2025/11/21，2026/02/14，2026/02/23，2026/02/25，2026/03/09，2026/03/15</t>
+          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/24，2025/05/13，2025/06/02，2025/06/27，2025/07/14，2025/08/26，2025/09/02，2025/10/03，2025/10/17，2025/11/21，2026/02/14，2026/02/23，2026/02/25，2026/03/09，2026/03/15，2026/8/28</t>
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
@@ -8878,7 +8866,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -8907,7 +8895,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/17，2025/05/15，2025/05/27，2025/11/27，2025/12/24，2026/01/14，2026/06/28</t>
+          <t>2025/03/27，2025/04/17，2025/05/15，2025/05/27，2025/11/27，2025/12/24，2026/01/14，2026/06/28，2026/08/18</t>
         </is>
       </c>
       <c r="F209" t="inlineStr"/>
@@ -8918,7 +8906,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -9034,12 +9022,12 @@
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Connie Talbot</t>
+          <t>Bruno Mars</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/22，2025/04/28，2025/06/30，2026/03/06</t>
+          <t>2025/03/27，2025/04/22，2025/04/28，2025/06/30，2026/03/06，2026/08/25</t>
         </is>
       </c>
       <c r="F212" t="inlineStr"/>
@@ -9050,7 +9038,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -9435,7 +9423,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/03，2025/07/24，2025/09/28，2025/10/31，2025/11/13，2026/01/14</t>
+          <t>2025/03/28，2025/05/03，2025/07/24，2025/09/28，2025/10/31，2025/11/13，2026/01/14，2026/08/18</t>
         </is>
       </c>
       <c r="F222" t="inlineStr"/>
@@ -9446,7 +9434,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -9475,7 +9463,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/09，2026/01/09，2026/02/19，2026/05/10，2026/07/10，2026/07/15，2026/07/31</t>
+          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/09，2026/01/09，2026/02/19，2026/05/10，2026/07/10，2026/07/15，2026/07/31，2026/8/28</t>
         </is>
       </c>
       <c r="F223" t="inlineStr"/>
@@ -9486,7 +9474,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -9671,7 +9659,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/8/16</t>
+          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/08/16</t>
         </is>
       </c>
       <c r="F228" t="inlineStr"/>
@@ -9751,7 +9739,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/24，2025/06/02，2025/06/27，2025/09/21，2025/10/07，2025/11/13，2025/12/02，2026/08/01</t>
+          <t>2025/03/28，2025/04/24，2025/06/02，2025/06/27，2025/09/21，2025/10/07，2025/11/13，2025/12/02，2026/08/01，2026/8/28</t>
         </is>
       </c>
       <c r="F230" t="inlineStr"/>
@@ -9762,7 +9750,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -9831,7 +9819,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/05/08，2025/05/20，2025/05/26，2025/06/05，2025/06/22，2025/07/10，2025/07/11，2025/07/22，2025/08/07，2025/09/17，2025/09/24，2025/10/23，2025/11/01，2025/11/13，2026/07/16，2026/07/25</t>
+          <t>2025/03/29，2025/05/08，2025/05/20，2025/05/26，2025/06/05，2025/06/22，2025/07/10，2025/07/11，2025/07/22，2025/08/07，2025/09/17，2025/09/24，2025/10/23，2025/11/01，2025/11/13，2026/07/16，2026/07/25，2026/08/25</t>
         </is>
       </c>
       <c r="F232" t="inlineStr"/>
@@ -9842,7 +9830,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -9955,7 +9943,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/03，2025/11/09，2025/12/23，2026/04/08，2026/04/24，2026/05/21，2026/06/10，2026/08/02</t>
+          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/03，2025/11/09，2025/12/23，2026/04/08，2026/04/24，2026/05/21，2026/06/10，2026/08/02，2026/8/28</t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
@@ -9966,7 +9954,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -9995,7 +9983,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/07，2025/11/13，2025/12/02，2026/01/14，2026/01/24，2026/03/07，2026/03/15，2026/04/24，2026/06/06，2026/06/23，2026/08/05，2026/08/05</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/07，2025/11/13，2025/12/02，2026/01/14，2026/01/24，2026/03/07，2026/03/15，2026/04/24，2026/06/06，2026/06/23，2026/08/05，2026/08/05，2026/08/19</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
@@ -10006,7 +9994,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -10035,7 +10023,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/25，2025/05/03，2025/06/23，2025/09/28，2025/11/28，2025/12/26，2026/06/28</t>
+          <t>2025/03/29，2025/04/25，2025/05/03，2025/06/23，2025/09/28，2025/11/28，2025/12/26，2026/06/28，2026/8/27</t>
         </is>
       </c>
       <c r="F237" t="inlineStr"/>
@@ -10046,7 +10034,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -10163,7 +10151,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/07/13，2025/10/20，2026/8/16</t>
+          <t>2025/03/30，2025/07/13，2025/10/20，2026/08/16</t>
         </is>
       </c>
       <c r="F240" t="inlineStr"/>
@@ -10203,7 +10191,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/06/17，2025/09/28，2025/10/20，2025/10/31，2026/01/16，2026/06/14，2026/06/17</t>
+          <t>2025/03/30，2025/06/17，2025/09/28，2025/10/20，2025/10/31，2026/01/16，2026/06/14，2026/06/17，2026/08/21</t>
         </is>
       </c>
       <c r="F241" t="inlineStr"/>
@@ -10214,7 +10202,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -10243,7 +10231,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/14，2025/05/26，2025/06/15，2025/07/09，2025/10/25，2025/11/24，2025/12/30，2026/01/16，2026/03/25，2026/05/23，2026/07/17</t>
+          <t>2025/03/30，2025/04/14，2025/05/26，2025/06/15，2025/07/09，2025/10/25，2025/11/24，2025/12/30，2026/01/16，2026/03/25，2026/05/23，2026/07/17，2026/08/25</t>
         </is>
       </c>
       <c r="F242" t="inlineStr"/>
@@ -10254,7 +10242,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -10283,7 +10271,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/22，2025/06/29，2025/09/30，2025/10/23，2026/01/19</t>
+          <t>2025/03/30，2025/05/22，2025/06/29，2025/09/30，2025/10/23，2026/01/19，2026/08/18</t>
         </is>
       </c>
       <c r="F243" t="inlineStr"/>
@@ -10294,7 +10282,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -10363,7 +10351,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/01/09，2026/03/07，2026/04/19，2026/05/23，2026/07/16</t>
+          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/01/09，2026/03/07，2026/04/19，2026/05/23，2026/07/16，2026/8/27</t>
         </is>
       </c>
       <c r="F245" t="inlineStr"/>
@@ -10374,7 +10362,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -10403,7 +10391,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/27，2025/05/19，2025/05/31，2025/08/30，2025/09/02，2025/11/18，2026/04/22，2026/07/31</t>
+          <t>2025/03/30，2025/04/27，2025/05/19，2025/05/31，2025/08/30，2025/09/02，2025/11/18，2026/04/22，2026/07/31，2026/8/28</t>
         </is>
       </c>
       <c r="F246" t="inlineStr"/>
@@ -10414,7 +10402,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -10483,7 +10471,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/01/01，2026/01/25，2026/03/08，2026/04/27，2026/06/13，2026/07/28</t>
+          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/01/01，2026/01/25，2026/03/08，2026/04/27，2026/06/13，2026/07/28，2026/8/28</t>
         </is>
       </c>
       <c r="F248" t="inlineStr"/>
@@ -10494,7 +10482,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -10559,7 +10547,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/19，2025/06/23，2025/07/08，2025/09/21，2025/10/23，2025/11/14，2025/12/17，2026/02/07</t>
+          <t>2025/03/30，2025/04/19，2025/06/23，2025/07/08，2025/09/21，2025/10/23，2025/11/14，2025/12/17，2026/02/07，2026/08/18</t>
         </is>
       </c>
       <c r="F250" t="inlineStr"/>
@@ -10570,7 +10558,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -10639,7 +10627,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/02/12，2026/04/16，2026/05/20，2026/06/20</t>
+          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/02/12，2026/04/16，2026/05/20，2026/06/20，2026/8/27</t>
         </is>
       </c>
       <c r="F252" t="inlineStr"/>
@@ -10650,7 +10638,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -10759,7 +10747,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/06/23，2025/07/08，2025/09/30，2025/10/23，2026/02/07，2026/06/28</t>
+          <t>2025/04/01，2025/06/23，2025/07/08，2025/09/30，2025/10/23，2026/02/07，2026/06/28，2026/08/18</t>
         </is>
       </c>
       <c r="F255" t="inlineStr"/>
@@ -10770,7 +10758,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -10799,7 +10787,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/01/21，2026/02/25，2026/02/27，2026/03/01，2026/03/08，2026/03/13，2026/03/25，2026/04/01，2026/05/01，2026/05/07，2026/05/08，2026/05/23，2026/06/13</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/01/21，2026/02/25，2026/02/27，2026/03/01，2026/03/08，2026/03/13，2026/03/25，2026/04/01，2026/05/01，2026/05/07，2026/05/08，2026/05/23，2026/06/13，2026/08/21</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10810,7 +10798,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -10839,7 +10827,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/02，2026/04/08，2026/05/01，2026/06/10，2026/06/20，2026/08/02</t>
+          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/02，2026/04/08，2026/05/01，2026/06/10，2026/06/20，2026/08/02，2026/08/21</t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
@@ -10850,7 +10838,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -10879,7 +10867,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/05/10，2025/09/04，2025/09/10，2025/09/28，2025/11/26，2026/01/19，2026/05/10</t>
+          <t>2025/04/01，2025/05/10，2025/09/04，2025/09/10，2025/09/28，2025/11/26，2026/01/19，2026/05/10，2026/08/18</t>
         </is>
       </c>
       <c r="F258" t="inlineStr"/>
@@ -10890,7 +10878,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -10919,7 +10907,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/02/08，2026/03/17，2026/05/05，2026/05/21，2026/06/25，2026/07/16</t>
+          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/02/08，2026/03/17，2026/05/05，2026/05/21，2026/06/25，2026/07/16，2026/08/23，2026/8/28</t>
         </is>
       </c>
       <c r="F259" t="inlineStr"/>
@@ -10930,7 +10918,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -10959,7 +10947,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/01/02，2026/01/05，2026/02/02，2026/02/09，2026/02/19，2026/03/25，2026/05/10，2026/05/21，2026/07/16</t>
+          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/01/02，2026/01/05，2026/02/02，2026/02/09，2026/02/19，2026/03/25，2026/05/10，2026/05/21，2026/07/16，2026/8/27，2026/8/27</t>
         </is>
       </c>
       <c r="F260" t="inlineStr"/>
@@ -10970,7 +10958,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -10999,7 +10987,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/12，2025/05/26，2025/08/26，2025/08/16，2025/10/05，2026/05/04</t>
+          <t>2025/04/02，2025/05/12，2025/05/26，2025/08/16，2025/08/26，2025/10/05，2026/05/04，2026/08/25</t>
         </is>
       </c>
       <c r="F261" t="inlineStr"/>
@@ -11010,7 +10998,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -11039,7 +11027,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/18，2025/05/26，2025/09/21，2025/10/07，2026/01/15</t>
+          <t>2025/04/02，2025/04/18，2025/05/26，2025/09/21，2025/10/07，2026/01/15，2026/08/25</t>
         </is>
       </c>
       <c r="F262" t="inlineStr"/>
@@ -11050,7 +11038,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -11239,7 +11227,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/13，2025/05/29，2025/09/04，2025/09/21，2025/10/22，2026/01/01，2026/01/15，2026/05/05，2026/8/16</t>
+          <t>2025/04/02，2025/05/13，2025/05/29，2025/09/04，2025/09/21，2025/10/22，2026/01/01，2026/01/15，2026/05/05，2026/08/16</t>
         </is>
       </c>
       <c r="F267" t="inlineStr"/>
@@ -11479,7 +11467,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08</t>
+          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08，2026/8/28</t>
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
@@ -11490,7 +11478,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -11683,7 +11671,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/06，2026/01/09，2026/01/29，2026/03/25，2026/04/24，2026/05/23，2026/06/15，2026/07/09，2026/07/22</t>
+          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/06，2026/01/09，2026/01/29，2026/03/25，2026/04/24，2026/05/23，2026/06/15，2026/07/09，2026/07/22，2026/08/25，2026/8/28</t>
         </is>
       </c>
       <c r="F278" t="inlineStr"/>
@@ -11694,7 +11682,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -11723,7 +11711,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/27，2026/8/16</t>
+          <t>2025/04/03，2025/04/27，2026/08/16</t>
         </is>
       </c>
       <c r="F279" t="inlineStr"/>
@@ -12195,7 +12183,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/07/13，2025/07/18，2025/11/03，2025/11/28，2026/8/16</t>
+          <t>2025/04/04，2025/07/13，2025/07/18，2025/11/03，2025/11/28，2026/08/16</t>
         </is>
       </c>
       <c r="F291" t="inlineStr"/>
@@ -12315,7 +12303,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/02/14，2026/03/05，2026/04/02，2026/05/20</t>
+          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/02/14，2026/03/05，2026/04/02，2026/05/20，2026/8/28</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -12326,7 +12314,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -12759,7 +12747,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09</t>
+          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23</t>
         </is>
       </c>
       <c r="F305" t="inlineStr"/>
@@ -12770,7 +12758,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -12799,7 +12787,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/05/19，2025/10/01，2025/10/31，2026/01/05，2026/03/25，2026/03/25，2026/08/02</t>
+          <t>2025/04/07，2025/05/19，2025/10/01，2025/10/31，2026/01/05，2026/03/25，2026/03/25，2026/08/02，2026/08/21</t>
         </is>
       </c>
       <c r="F306" t="inlineStr"/>
@@ -12810,7 +12798,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -12839,7 +12827,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/01/03，2026/01/22，2026/02/14，2026/05/20，2026/08/08</t>
+          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/01/03，2026/01/22，2026/02/14，2026/05/20，2026/08/08，2026/08/19，2026/08/25</t>
         </is>
       </c>
       <c r="F307" t="inlineStr"/>
@@ -12850,7 +12838,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -12879,7 +12867,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/05/08，2025/05/20，2025/05/30，2025/06/16，2025/08/29，2025/09/12，2025/10/09，2025/10/16，2025/11/18，2026/02/04，2026/02/14，2026/04/15，2026/06/13，2026/07/07，2026/07/28</t>
+          <t>2025/04/07，2025/04/17，2025/05/08，2025/05/20，2025/05/30，2025/06/16，2025/08/29，2025/09/12，2025/10/09，2025/10/16，2025/11/18，2026/02/04，2026/02/14，2026/04/15，2026/06/13，2026/07/07，2026/07/28，2026/8/28</t>
         </is>
       </c>
       <c r="F308" t="inlineStr"/>
@@ -12890,7 +12878,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
@@ -12919,7 +12907,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/03，2025/11/09，2025/11/26，2025/12/09，2026/01/23，2026/03/13，2026/03/25，2026/04/08，2026/05/23，2026/06/20，2026/08/02</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/03，2025/11/09，2025/11/26，2025/12/09，2026/01/23，2026/03/13，2026/03/25，2026/04/08，2026/05/23，2026/06/20，2026/08/02，2026/8/28</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12930,7 +12918,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -13079,7 +13067,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/09，2025/12/05，2025/12/19，2025/12/26，2026/01/10，2026/01/19，2026/02/10，2026/03/24，2026/04/18，2026/06/06，2026/08/07</t>
+          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/09，2025/12/05，2025/12/19，2025/12/26，2026/01/10，2026/01/19，2026/02/10，2026/03/24，2026/04/18，2026/06/06，2026/08/07，2026/08/23</t>
         </is>
       </c>
       <c r="F313" t="inlineStr"/>
@@ -13090,7 +13078,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -13239,7 +13227,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/06/29，2025/08/01，2025/09/04，2025/09/21，2025/10/17，2025/11/09，2025/11/13，2025/12/04，2025/12/13，2026/03/04，2026/05/07，2026/06/20</t>
+          <t>2025/04/11，2025/06/29，2025/08/01，2025/09/04，2025/09/21，2025/10/17，2025/11/09，2025/11/13，2025/12/04，2025/12/13，2026/03/04，2026/05/07，2026/06/20，2026/8/28</t>
         </is>
       </c>
       <c r="F317" t="inlineStr"/>
@@ -13250,7 +13238,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -13315,7 +13303,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/18，2025/06/09，2025/07/07，2025/08/26，2025/09/03，2025/09/13，2025/10/17，2025/10/30，2025/11/21，2025/12/17，2026/04/19</t>
+          <t>2025/04/11，2025/05/18，2025/06/09，2025/07/07，2025/08/26，2025/09/03，2025/09/13，2025/10/17，2025/10/30，2025/11/21，2025/12/17，2026/04/19，2026/8/27</t>
         </is>
       </c>
       <c r="F319" t="inlineStr"/>
@@ -13326,7 +13314,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
@@ -13399,7 +13387,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/09，2025/12/08，2026/01/05，2026/02/14，2026/05/23，2026/06/20，2026/07/18</t>
+          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/09，2025/12/08，2026/01/05，2026/02/14，2026/05/23，2026/06/20，2026/07/18，2026/08/25</t>
         </is>
       </c>
       <c r="F321" t="inlineStr"/>
@@ -13410,7 +13398,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -13475,7 +13463,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/01/29，2026/02/10，2026/03/09，2026/03/24，2026/04/19，2026/05/21，2026/06/15，2026/08/02</t>
+          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/11，2025/09/12，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/01/29，2026/02/10，2026/03/09，2026/03/24，2026/04/19，2026/05/21，2026/06/15，2026/08/02</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -13831,7 +13819,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/06/02，2025/06/12，2025/09/27，2025/11/09，2025/12/19，2026/01/01，2026/02/17，2026/07/09，2026/07/27</t>
+          <t>2025/04/11，2025/06/02，2025/06/12，2025/09/27，2025/11/09，2025/12/19，2026/01/01，2026/02/17，2026/07/09，2026/07/27，2026/08/21</t>
         </is>
       </c>
       <c r="F332" t="inlineStr"/>
@@ -13842,7 +13830,7 @@
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I332" t="inlineStr">
@@ -13911,7 +13899,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>2025/04/12，2025/04/28，2025/07/10，2025/09/08，2025/09/07</t>
+          <t>2025/04/12，2025/04/28，2025/07/10，2025/09/07，2025/09/08</t>
         </is>
       </c>
       <c r="F334" t="inlineStr"/>
@@ -13987,7 +13975,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/01/09，2026/02/08，2026/03/01，2026/03/09，2026/03/24，2026/04/17，2026/05/01，2026/05/21，2026/06/10，2026/06/25，2026/07/27</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/01/09，2026/02/08，2026/03/01，2026/03/09，2026/03/24，2026/04/17，2026/05/01，2026/05/21，2026/06/10，2026/06/25，2026/07/27，2026/08/23，2026/8/28</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13998,7 +13986,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -14327,7 +14315,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>2025/04/14，2025/05/24，2025/06/15，2025/06/19，2025/07/21，2025/08/22，2025/09/20，2025/10/09，2025/10/28，2025/12/22，2026/06/20</t>
+          <t>2025/04/14，2025/05/24，2025/06/15，2025/06/19，2025/07/21，2025/08/22，2025/09/20，2025/10/09，2025/10/28，2025/12/22，2026/06/20，2026/8/27</t>
         </is>
       </c>
       <c r="F344" t="inlineStr"/>
@@ -14338,7 +14326,7 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
@@ -14447,7 +14435,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/01/16，2026/03/25，2026/04/24，2026/05/23，2026/07/17</t>
+          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/01/16，2026/03/25，2026/04/24，2026/05/23，2026/07/17，2026/08/21</t>
         </is>
       </c>
       <c r="F347" t="inlineStr"/>
@@ -14458,7 +14446,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -14775,7 +14763,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/05/01，2025/05/26，2025/07/03，2025/07/27，2025/09/18，2025/10/17，2025/11/21，2026/01/12，2026/01/24，2026/02/19，2026/02/23，2026/03/24，2026/05/04，2026/07/07</t>
+          <t>2025/04/17，2025/05/01，2025/05/26，2025/07/03，2025/07/27，2025/09/18，2025/10/17，2025/11/21，2026/01/12，2026/01/24，2026/02/19，2026/02/23，2026/03/24，2026/05/04，2026/07/07，2026/08/25</t>
         </is>
       </c>
       <c r="F355" t="inlineStr"/>
@@ -14786,7 +14774,7 @@
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
@@ -14895,7 +14883,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/05/31，2025/06/03，2025/06/14，2025/09/10，2026/03/28</t>
+          <t>2025/04/17，2025/05/31，2025/06/03，2025/06/14，2025/09/10，2026/03/28，2026/8/28</t>
         </is>
       </c>
       <c r="F358" t="inlineStr"/>
@@ -14906,7 +14894,7 @@
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
@@ -15255,7 +15243,7 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/01/10，2026/03/22，2026/04/24，2026/05/25，2026/08/11</t>
+          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/01/10，2026/03/22，2026/04/24，2026/05/25，2026/08/11，2026/08/25</t>
         </is>
       </c>
       <c r="F367" t="inlineStr"/>
@@ -15266,7 +15254,7 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
@@ -15663,7 +15651,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>2025/04/21，2025/05/19，2025/07/25，2025/08/07，2025/09/15，2025/09/29，2026/01/05，2026/02/14，2026/04/09，2026/06/20</t>
+          <t>2025/04/21，2025/05/19，2025/07/25，2025/08/07，2025/09/15，2025/09/29，2026/01/05，2026/02/14，2026/04/09，2026/06/20，2026/08/23</t>
         </is>
       </c>
       <c r="F377" t="inlineStr"/>
@@ -15674,7 +15662,7 @@
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I377" t="inlineStr">
@@ -15855,7 +15843,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>2025/04/24，2025/09/22，2026/03/29，2026/06/10</t>
+          <t>2025/04/24，2025/09/22，2026/03/29，2026/06/10，2026/8/28</t>
         </is>
       </c>
       <c r="F382" t="inlineStr"/>
@@ -15866,7 +15854,7 @@
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I382" t="inlineStr">
@@ -16355,7 +16343,7 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/19，2025/06/23，2025/08/12，2025/10/09，2025/11/03，2025/12/30，2026/01/09，2026/04/01，2026/05/23，2026/07/31</t>
+          <t>2025/04/25，2025/06/19，2025/06/23，2025/08/12，2025/10/09，2025/11/03，2025/12/30，2026/01/09，2026/04/01，2026/05/23，2026/07/31，2026/08/25</t>
         </is>
       </c>
       <c r="F395" t="inlineStr"/>
@@ -16366,7 +16354,7 @@
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I395" t="inlineStr">
@@ -17195,7 +17183,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/08/28，2025/09/11，2025/10/20，2025/12/09，2026/8/16</t>
+          <t>2025/05/03，2025/08/28，2025/09/11，2025/10/20，2025/12/09，2026/08/16</t>
         </is>
       </c>
       <c r="F416" t="inlineStr"/>
@@ -17235,7 +17223,7 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/07/18，2025/08/02，2025/10/16，2026/05/01</t>
+          <t>2025/05/03，2025/07/18，2025/08/02，2025/10/16，2026/05/01，2026/8/27</t>
         </is>
       </c>
       <c r="F417" t="inlineStr"/>
@@ -17246,7 +17234,7 @@
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I417" t="inlineStr">
@@ -17355,7 +17343,7 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>2025/05/03</t>
+          <t>2025/05/03，2026/8/27</t>
         </is>
       </c>
       <c r="F420" t="inlineStr"/>
@@ -17366,7 +17354,7 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
@@ -17555,7 +17543,7 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/04/20，2026/05/23</t>
+          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/04/20，2026/05/23，2026/8/28</t>
         </is>
       </c>
       <c r="F425" t="inlineStr"/>
@@ -17566,7 +17554,7 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
@@ -18191,7 +18179,7 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/01/01，2026/02/10，2026/02/22，2026/03/12，2026/04/05，2026/05/03，2026/05/24，2026/07/03，2026/08/07</t>
+          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/01/01，2026/02/10，2026/02/22，2026/03/12，2026/04/05，2026/05/03，2026/05/24，2026/07/03，2026/08/07，2026/08/23</t>
         </is>
       </c>
       <c r="F441" t="inlineStr"/>
@@ -18202,7 +18190,7 @@
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
@@ -18231,7 +18219,7 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/27，2025/07/10，2026/03/09，2026/04/09，2026/06/10</t>
+          <t>2025/05/18，2025/06/27，2025/07/10，2026/03/09，2026/04/09，2026/06/10，2026/8/28，2026/8/28</t>
         </is>
       </c>
       <c r="F442" t="inlineStr"/>
@@ -18242,7 +18230,7 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
@@ -18431,7 +18419,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/01/02，2026/03/17，2026/04/29，2026/05/10，2026/07/09，2026/07/31，2026/08/11</t>
+          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/01/02，2026/03/17，2026/04/29，2026/05/10，2026/07/09，2026/07/31，2026/08/11，2026/08/25</t>
         </is>
       </c>
       <c r="F447" t="inlineStr"/>
@@ -18442,7 +18430,7 @@
       </c>
       <c r="H447" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I447" t="inlineStr">
@@ -18511,7 +18499,7 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/12/16，2025/12/24，2026/8/16</t>
+          <t>2025/05/19，2025/12/16，2025/12/24，2026/08/16</t>
         </is>
       </c>
       <c r="F449" t="inlineStr"/>
@@ -18675,7 +18663,7 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/31，2025/06/07，2025/06/10，2025/08/02，2025/10/07，2025/12/06，2026/03/22，2026/05/01，2026/8/16</t>
+          <t>2025/05/22，2025/05/31，2025/06/07，2025/06/10，2025/08/02，2025/10/07，2025/12/06，2026/03/22，2026/05/01，2026/08/16</t>
         </is>
       </c>
       <c r="F453" t="inlineStr"/>
@@ -18755,7 +18743,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/09/12，2025/09/02，2025/12/05，2026/04/09，2026/05/10</t>
+          <t>2025/05/22，2025/09/02，2025/09/12，2025/12/05，2026/04/09，2026/05/10</t>
         </is>
       </c>
       <c r="F455" t="inlineStr"/>
@@ -19047,7 +19035,7 @@
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>2025/05/23，2025/05/29，2025/09/17，2025/09/02，2025/09/26，2025/10/09，2025/10/24，2026/04/29，2026/05/23，2026/07/07</t>
+          <t>2025/05/23，2025/05/29，2025/09/02，2025/09/17，2025/09/26，2025/10/09，2025/10/24，2026/04/29，2026/05/23，2026/07/07，2026/08/25</t>
         </is>
       </c>
       <c r="F462" t="inlineStr"/>
@@ -19058,7 +19046,7 @@
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I462" t="inlineStr">
@@ -19247,7 +19235,7 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>2025/05/24，2025/07/13，2025/08/23，2025/09/29，2025/12/24，2025/12/30，2026/01/28，2026/04/08，2026/8/16</t>
+          <t>2025/05/24，2025/07/13，2025/08/23，2025/09/29，2025/12/24，2025/12/30，2026/01/28，2026/04/08，2026/08/16</t>
         </is>
       </c>
       <c r="F467" t="inlineStr"/>
@@ -19447,7 +19435,7 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/07，2025/12/07，2025/12/23，2026/01/09，2026/01/24，2026/02/09，2026/02/25，2026/03/13，2026/03/21，2026/04/18，2026/05/04，2026/05/23，2026/06/14，2026/06/19，2026/07/16</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/07，2025/12/07，2025/12/23，2026/01/09，2026/01/24，2026/02/09，2026/02/25，2026/03/13，2026/03/21，2026/04/18，2026/05/04，2026/05/23，2026/06/14，2026/06/19，2026/07/16，2026/08/23</t>
         </is>
       </c>
       <c r="F472" t="inlineStr"/>
@@ -19458,7 +19446,7 @@
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I472" t="inlineStr">
@@ -19527,7 +19515,7 @@
       </c>
       <c r="E474" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/08/21</t>
+          <t>2025/05/30，2025/08/21，2026/08/18</t>
         </is>
       </c>
       <c r="F474" t="inlineStr"/>
@@ -19538,7 +19526,7 @@
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I474" t="inlineStr">
@@ -19567,7 +19555,7 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/08/23，2025/10/11，2026/8/16</t>
+          <t>2025/05/30，2025/08/23，2025/10/11，2026/08/16</t>
         </is>
       </c>
       <c r="F475" t="inlineStr"/>
@@ -19767,7 +19755,7 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/05/31，2025/05/31，2025/06/02，2025/06/03，2025/06/05，2025/06/19，2025/06/26，2025/07/03，2025/07/14，2025/08/02，2025/08/24，2025/09/03，2025/09/18，2025/10/07，2025/11/19，2025/12/11，2026/01/10，2026/01/22，2026/03/25，2026/06/28，2026/08/03</t>
+          <t>2025/05/30，2025/05/31，2025/05/31，2025/06/02，2025/06/03，2025/06/05，2025/06/19，2025/06/26，2025/07/03，2025/07/14，2025/08/02，2025/08/24，2025/09/03，2025/09/18，2025/10/07，2025/11/19，2025/12/11，2026/01/10，2026/01/22，2026/03/25，2026/06/28，2026/08/03，2026/08/23</t>
         </is>
       </c>
       <c r="F480" t="inlineStr"/>
@@ -19778,7 +19766,7 @@
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I480" t="inlineStr">
@@ -19807,7 +19795,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>2025/05/31，2025/06/02，2025/06/23，2025/09/15，2025/09/27，2025/10/17，2026/8/16</t>
+          <t>2025/05/31，2025/06/02，2025/06/23，2025/09/15，2025/09/27，2025/10/17，2026/08/16</t>
         </is>
       </c>
       <c r="F481" t="inlineStr"/>
@@ -20611,7 +20599,7 @@
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>2025/06/02，2025/06/07，2025/06/12，2025/06/28，2025/08/13，2025/09/11，2025/09/30，2025/11/27</t>
+          <t>2025/06/02，2025/06/07，2025/06/12，2025/06/28，2025/08/13，2025/09/11，2025/09/30，2025/11/27，2026/8/27</t>
         </is>
       </c>
       <c r="F501" t="inlineStr"/>
@@ -20622,7 +20610,7 @@
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I501" t="inlineStr">
@@ -20651,7 +20639,7 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>2025/06/02，2025/10/20，2025/11/01，2026/03/05，2026/04/14</t>
+          <t>2025/06/02，2025/10/20，2025/11/01，2026/03/05，2026/04/14，2026/08/23</t>
         </is>
       </c>
       <c r="F502" t="inlineStr"/>
@@ -20662,7 +20650,7 @@
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I502" t="inlineStr">
@@ -20887,7 +20875,7 @@
       </c>
       <c r="E508" t="inlineStr">
         <is>
-          <t>2025/06/07，2025/11/24</t>
+          <t>2025/06/07，2025/11/24，2026/08/18</t>
         </is>
       </c>
       <c r="F508" t="inlineStr"/>
@@ -20898,7 +20886,7 @@
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I508" t="inlineStr">
@@ -21211,7 +21199,7 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>2025/06/13，2025/07/25，2026/05/05</t>
+          <t>2025/06/13，2025/07/25，2026/05/05，2026/08/25</t>
         </is>
       </c>
       <c r="F516" t="inlineStr"/>
@@ -21222,7 +21210,7 @@
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I516" t="inlineStr">
@@ -21291,7 +21279,7 @@
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/02，2025/12/09，2025/12/16，2025/12/26，2026/01/05，2026/01/15，2026/01/28，2026/03/06，2026/04/22，2026/05/10，2026/05/15，2026/06/19，2026/07/09，2026/07/31</t>
+          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/02，2025/12/09，2025/12/16，2025/12/26，2026/01/05，2026/01/15，2026/01/28，2026/03/06，2026/04/22，2026/05/10，2026/05/15，2026/06/19，2026/07/09，2026/07/31，2026/08/21</t>
         </is>
       </c>
       <c r="F518" t="inlineStr"/>
@@ -21302,7 +21290,7 @@
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I518" t="inlineStr">
@@ -21411,7 +21399,7 @@
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>2025/06/17，2026/06/26</t>
+          <t>2025/06/17，2026/06/26，2026/08/21</t>
         </is>
       </c>
       <c r="F521" t="inlineStr"/>
@@ -21422,7 +21410,7 @@
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I521" t="inlineStr">
@@ -22175,7 +22163,7 @@
       </c>
       <c r="E540" t="inlineStr">
         <is>
-          <t>2025/06/23，2025/10/19，2026/01/19，2026/8/16</t>
+          <t>2025/06/23，2025/10/19，2026/01/19，2026/08/16</t>
         </is>
       </c>
       <c r="F540" t="inlineStr"/>
@@ -22375,7 +22363,7 @@
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/01/14，2026/01/22，2026/02/19，2026/03/13，2026/04/12，2026/05/10，2026/06/17，2026/08/08</t>
+          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/01/14，2026/01/22，2026/02/19，2026/03/13，2026/04/12，2026/05/10，2026/06/17，2026/08/08，2026/08/18</t>
         </is>
       </c>
       <c r="F545" t="inlineStr"/>
@@ -22386,7 +22374,7 @@
       </c>
       <c r="H545" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I545" t="inlineStr">
@@ -22419,7 +22407,7 @@
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/03/08，2026/05/01，2026/05/23，2026/07/17</t>
+          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/03/08，2026/05/01，2026/05/23，2026/07/17，2026/08/25</t>
         </is>
       </c>
       <c r="F546" t="inlineStr"/>
@@ -22430,7 +22418,7 @@
       </c>
       <c r="H546" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I546" t="inlineStr">
@@ -22711,7 +22699,7 @@
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/8/16</t>
+          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/08/16</t>
         </is>
       </c>
       <c r="F553" t="inlineStr"/>
@@ -22751,7 +22739,7 @@
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>2025/06/29，2026/08/11</t>
+          <t>2025/06/29，2026/08/11，2026/08/21</t>
         </is>
       </c>
       <c r="F554" t="inlineStr"/>
@@ -22762,7 +22750,7 @@
       </c>
       <c r="H554" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I554" t="inlineStr">
@@ -23423,7 +23411,7 @@
       </c>
       <c r="E571" t="inlineStr">
         <is>
-          <t>2025/07/07，2025/07/31，2025/09/11，2025/10/11，2025/11/07，2025/11/12，2025/12/09，2026/01/14，2026/01/30，2026/04/09</t>
+          <t>2025/07/07，2025/07/31，2025/09/11，2025/10/11，2025/11/07，2025/11/12，2025/12/09，2026/01/14，2026/01/30，2026/04/09，2026/8/28</t>
         </is>
       </c>
       <c r="F571" t="inlineStr"/>
@@ -23434,7 +23422,7 @@
       </c>
       <c r="H571" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I571" t="inlineStr">
@@ -23703,7 +23691,7 @@
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/01/09，2026/03/07，2026/03/08，2026/06/14</t>
+          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/01/09，2026/03/07，2026/03/08，2026/06/14，2026/8/27</t>
         </is>
       </c>
       <c r="F578" t="inlineStr"/>
@@ -23714,7 +23702,7 @@
       </c>
       <c r="H578" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I578" t="inlineStr">
@@ -23903,7 +23891,7 @@
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>2025/07/14，2025/07/18，2025/07/28，2025/08/07，2025/08/10，2025/09/04，2025/09/18，2025/10/16，2025/10/22，2026/06/03，2026/07/26</t>
+          <t>2025/07/14，2025/07/18，2025/07/28，2025/08/07，2025/08/10，2025/09/04，2025/09/18，2025/10/16，2025/10/22，2026/06/03，2026/07/26，2026/8/27</t>
         </is>
       </c>
       <c r="F583" t="inlineStr"/>
@@ -23914,7 +23902,7 @@
       </c>
       <c r="H583" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I583" t="inlineStr">
@@ -23983,7 +23971,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/03，2025/11/22，2026/01/05，2026/02/18，2026/02/23，2026/04/19，2026/06/06，2026/06/19，2026/07/28</t>
+          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/03，2025/11/22，2026/01/05，2026/02/18，2026/02/23，2026/04/19，2026/06/06，2026/06/19，2026/07/28，2026/8/28</t>
         </is>
       </c>
       <c r="F585" t="inlineStr"/>
@@ -23994,7 +23982,7 @@
       </c>
       <c r="H585" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I585" t="inlineStr">
@@ -24063,7 +24051,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>2025/07/15，2026/01/05，2026/01/10，2026/01/25，2026/02/10，2026/02/27，2026/03/07，2026/03/15，2026/03/29，2026/06/23</t>
+          <t>2025/07/15，2026/01/05，2026/01/10，2026/01/25，2026/02/10，2026/02/27，2026/03/07，2026/03/15，2026/03/29，2026/06/23，2026/8/28</t>
         </is>
       </c>
       <c r="F587" t="inlineStr"/>
@@ -24074,7 +24062,7 @@
       </c>
       <c r="H587" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I587" t="inlineStr">
@@ -24451,7 +24439,7 @@
       </c>
       <c r="E597" t="inlineStr">
         <is>
-          <t>2025/07/24，2025/07/26，2025/07/28，2025/07/31，2025/08/04，2025/08/07，2025/08/12，2025/08/22，2025/09/17，2025/09/11，2025/10/07，2025/11/12，2026/01/14，2026/02/07，2026/06/03，2026/07/26</t>
+          <t>2025/07/24，2025/07/26，2025/07/28，2025/07/31，2025/08/04，2025/08/07，2025/08/12，2025/08/22，2025/09/11，2025/09/17，2025/10/07，2025/11/12，2026/01/14，2026/02/07，2026/06/03，2026/07/26</t>
         </is>
       </c>
       <c r="F597" t="inlineStr"/>
@@ -24575,7 +24563,7 @@
       </c>
       <c r="E600" t="inlineStr">
         <is>
-          <t>2025/07/26，2025/09/24，2025/10/28，2025/11/12，2025/12/16，2026/01/14，2026/01/30，2026/06/10，2026/07/26</t>
+          <t>2025/07/26，2025/09/24，2025/10/28，2025/11/12，2025/12/16，2026/01/14，2026/01/30，2026/06/10，2026/07/26，2026/08/21</t>
         </is>
       </c>
       <c r="F600" t="inlineStr"/>
@@ -24586,7 +24574,7 @@
       </c>
       <c r="H600" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I600" t="inlineStr">
@@ -24735,7 +24723,7 @@
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/01/19，2026/02/12，2026/02/14，2026/04/08，2026/04/19，2026/05/20，2026/06/06，2026/07/22</t>
+          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/01/19，2026/02/12，2026/02/14，2026/04/08，2026/04/19，2026/05/20，2026/06/06，2026/07/22，2026/8/27</t>
         </is>
       </c>
       <c r="F604" t="inlineStr"/>
@@ -24746,7 +24734,7 @@
       </c>
       <c r="H604" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I604" t="inlineStr">
@@ -25007,7 +24995,7 @@
       </c>
       <c r="E611" t="inlineStr">
         <is>
-          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/02，2025/12/17，2026/01/14，2026/02/02，2026/03/22，2026/04/01，2026/04/08，2026/05/15，2026/06/10，2026/07/31</t>
+          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/02，2025/12/17，2026/01/14，2026/02/02，2026/03/22，2026/04/01，2026/04/08，2026/05/15，2026/06/10，2026/07/31，2026/08/25</t>
         </is>
       </c>
       <c r="F611" t="inlineStr"/>
@@ -25018,7 +25006,7 @@
       </c>
       <c r="H611" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I611" t="inlineStr">
@@ -25371,7 +25359,7 @@
       </c>
       <c r="E620" t="inlineStr">
         <is>
-          <t>2025/08/26，2025/08/16，2025/11/13，2025/12/09，2026/01/29，2026/02/19，2026/03/31</t>
+          <t>2025/08/16，2025/08/26，2025/11/13，2025/12/09，2026/01/29，2026/02/19，2026/03/31</t>
         </is>
       </c>
       <c r="F620" t="inlineStr"/>
@@ -26311,7 +26299,7 @@
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/03，2025/11/13，2025/11/24，2025/12/05，2025/12/12，2025/12/17，2026/01/06，2026/01/15，2026/01/24，2026/02/27，2026/04/19，2026/06/06，2026/07/17，2026/07/28</t>
+          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/03，2025/11/13，2025/11/24，2025/12/05，2025/12/12，2025/12/17，2026/01/06，2026/01/15，2026/01/24，2026/02/27，2026/04/19，2026/06/06，2026/07/17，2026/07/28，2026/8/28</t>
         </is>
       </c>
       <c r="F644" t="inlineStr"/>
@@ -26322,7 +26310,7 @@
       </c>
       <c r="H644" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I644" t="inlineStr">
@@ -26387,7 +26375,7 @@
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>2025/09/17，2025/09/15，2025/09/22，2025/09/29，2025/09/29，2025/10/10，2025/10/28，2025/12/02，2026/01/05，2026/03/13，2026/06/23</t>
+          <t>2025/09/15，2025/09/17，2025/09/22，2025/09/29，2025/09/29，2025/10/10，2025/10/28，2025/12/02，2026/01/05，2026/03/13，2026/06/23</t>
         </is>
       </c>
       <c r="F646" t="inlineStr"/>
@@ -26427,7 +26415,7 @@
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/02/23，2026/03/17，2026/03/25，2026/05/23</t>
+          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/02/23，2026/03/17，2026/03/25，2026/05/23，2026/8/27</t>
         </is>
       </c>
       <c r="F647" t="inlineStr"/>
@@ -26438,7 +26426,7 @@
       </c>
       <c r="H647" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I647" t="inlineStr">
@@ -26895,7 +26883,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31，2026/08/23</t>
         </is>
       </c>
       <c r="F659" t="inlineStr"/>
@@ -26906,7 +26894,7 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
@@ -26975,7 +26963,7 @@
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>2025/09/22</t>
+          <t>2025/09/22，2026/08/19</t>
         </is>
       </c>
       <c r="F661" t="inlineStr"/>
@@ -26986,7 +26974,7 @@
       </c>
       <c r="H661" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I661" t="inlineStr">
@@ -27087,7 +27075,7 @@
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>2025/09/22，2025/10/09，2025/12/05，2026/8/16</t>
+          <t>2025/09/22，2025/10/09，2025/12/05，2026/08/16</t>
         </is>
       </c>
       <c r="F664" t="inlineStr"/>
@@ -27275,7 +27263,7 @@
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/26，2025/09/28，2025/09/29，2025/10/01，2025/10/07，2025/10/10，2025/10/11，2025/10/17，2025/10/23，2025/10/28，2025/12/26，2026/02/05，2026/07/16，2026/07/31</t>
+          <t>2025/09/24，2025/09/26，2025/09/28，2025/09/29，2025/10/01，2025/10/07，2025/10/10，2025/10/11，2025/10/17，2025/10/23，2025/10/28，2025/12/26，2026/02/05，2026/07/16，2026/07/31，2026/08/19</t>
         </is>
       </c>
       <c r="F669" t="inlineStr"/>
@@ -27286,7 +27274,7 @@
       </c>
       <c r="H669" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I669" t="inlineStr">
@@ -27667,7 +27655,7 @@
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>2025/09/30，2025/10/01，2025/10/11，2025/10/17，2025/10/26，2026/8/16</t>
+          <t>2025/09/30，2025/10/01，2025/10/11，2025/10/17，2025/10/26，2026/08/16</t>
         </is>
       </c>
       <c r="F679" t="inlineStr"/>
@@ -28475,7 +28463,7 @@
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>2025/10/18</t>
+          <t>2025/10/18，2026/08/25</t>
         </is>
       </c>
       <c r="F699" t="inlineStr"/>
@@ -28486,7 +28474,7 @@
       </c>
       <c r="H699" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I699" t="inlineStr">
@@ -28591,7 +28579,7 @@
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>2025/10/23，2026/8/16</t>
+          <t>2025/10/23，2026/08/16，2026/08/21</t>
         </is>
       </c>
       <c r="F702" t="inlineStr"/>
@@ -28602,12 +28590,12 @@
       </c>
       <c r="H702" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I702" t="inlineStr">
         <is>
-          <t>BV1gabm6ZEH1</t>
+          <t>BV1GHb16oEuk，BV1gabm6ZEH1</t>
         </is>
       </c>
       <c r="J702" t="inlineStr"/>
@@ -28631,7 +28619,7 @@
       </c>
       <c r="E703" t="inlineStr">
         <is>
-          <t>2025/10/23，2025/10/25，2025/12/12，2026/01/19，2026/03/28</t>
+          <t>2025/10/23，2025/10/25，2025/12/12，2026/01/19，2026/03/28，2026/08/21</t>
         </is>
       </c>
       <c r="F703" t="inlineStr"/>
@@ -28642,7 +28630,7 @@
       </c>
       <c r="H703" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I703" t="inlineStr">
@@ -29059,7 +29047,7 @@
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>2025/10/28，2025/11/01，2025/11/12，2025/12/19，2026/02/08，2026/02/10，2026/05/10，2026/8/16</t>
+          <t>2025/10/28，2025/11/01，2025/11/12，2025/12/19，2026/02/08，2026/02/10，2026/05/10，2026/08/16</t>
         </is>
       </c>
       <c r="F714" t="inlineStr"/>
@@ -30411,7 +30399,7 @@
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>2025/12/09，2025/12/17，2026/01/14，2026/01/23，2026/02/05，2026/02/10，2026/02/25，2026/04/08，2026/05/01，2026/06/16，2026/8/16</t>
+          <t>2025/12/09，2025/12/17，2026/01/14，2026/01/23，2026/02/05，2026/02/10，2026/02/25，2026/04/08，2026/05/01，2026/06/16，2026/08/16</t>
         </is>
       </c>
       <c r="F749" t="inlineStr"/>
@@ -30875,7 +30863,7 @@
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/01/02，2026/01/05，2026/01/11，2026/01/25，2026/02/09，2026/02/23，2026/03/20，2026/04/02，2026/04/16，2026/04/29，2026/05/10，2026/06/06，2026/06/14，2026/06/20，2026/07/16，2026/08/02，2026/08/07</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/01/02，2026/01/05，2026/01/11，2026/01/25，2026/02/09，2026/02/23，2026/03/20，2026/04/02，2026/04/16，2026/04/29，2026/05/10，2026/06/06，2026/06/14，2026/06/20，2026/07/16，2026/08/02，2026/08/07，2026/08/23，2026/8/28</t>
         </is>
       </c>
       <c r="F761" t="inlineStr"/>
@@ -30886,7 +30874,7 @@
       </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I761" t="inlineStr">
@@ -30915,7 +30903,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08</t>
+          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08，2026/08/19</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -30926,7 +30914,7 @@
       </c>
       <c r="H762" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I762" t="inlineStr">
@@ -30955,7 +30943,7 @@
       </c>
       <c r="E763" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/01/05，2026/01/19，2026/01/21，2026/01/22，2026/01/24，2026/02/07，2026/02/19，2026/02/24，2026/02/24，2026/02/25，2026/03/06，2026/03/25，2026/04/11，2026/04/20，2026/05/15，2026/06/19，2026/07/18</t>
+          <t>2025/12/26，2026/01/05，2026/01/19，2026/01/21，2026/01/22，2026/01/24，2026/02/07，2026/02/19，2026/02/24，2026/02/24，2026/02/25，2026/03/06，2026/03/25，2026/04/11，2026/04/20，2026/05/15，2026/06/19，2026/07/18，2026/08/21，2026/8/28</t>
         </is>
       </c>
       <c r="F763" t="inlineStr"/>
@@ -30966,7 +30954,7 @@
       </c>
       <c r="H763" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I763" t="inlineStr">
@@ -31039,7 +31027,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/01/10，2026/01/22，2026/01/23，2026/01/31，2026/02/10，2026/02/23，2026/03/09，2026/03/12，2026/03/14，2026/03/17，2026/03/27，2026/04/24，2026/05/01，2026/06/14，2026/08/01</t>
+          <t>2025/12/26，2026/01/10，2026/01/22，2026/01/23，2026/01/31，2026/02/10，2026/02/23，2026/03/09，2026/03/12，2026/03/14，2026/03/17，2026/03/27，2026/04/24，2026/05/01，2026/06/14，2026/08/01，2026/8/28</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -31050,7 +31038,7 @@
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I765" t="inlineStr">
@@ -31463,7 +31451,7 @@
       </c>
       <c r="E776" t="inlineStr">
         <is>
-          <t>2026/01/24，2026/01/25，2026/01/26，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/03/04，2026/03/12，2026/03/31，2026/04/01，2026/04/14，2026/04/18，2026/05/10，2026/05/23，2026/06/12，2026/07/03，2026/07/21，2026/08/07</t>
+          <t>2026/01/24，2026/01/25，2026/01/26，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/03/04，2026/03/12，2026/03/31，2026/04/01，2026/04/14，2026/04/18，2026/05/10，2026/05/23，2026/06/12，2026/07/03，2026/07/21，2026/08/07，2026/08/23</t>
         </is>
       </c>
       <c r="F776" t="inlineStr"/>
@@ -31474,7 +31462,7 @@
       </c>
       <c r="H776" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I776" t="inlineStr">
@@ -31547,7 +31535,7 @@
       </c>
       <c r="E778" t="inlineStr">
         <is>
-          <t>2026/01/25</t>
+          <t>2026/01/25，2026/08/19</t>
         </is>
       </c>
       <c r="F778" t="inlineStr"/>
@@ -31558,10 +31546,14 @@
       </c>
       <c r="H778" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I778" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>BV18u8n6QEXN</t>
+        </is>
+      </c>
       <c r="J778" t="inlineStr">
         <is>
           <t>游戏</t>
@@ -31907,7 +31899,7 @@
       </c>
       <c r="E787" t="inlineStr">
         <is>
-          <t>2026/02/08，2026/02/09，2026/02/14，2026/02/20，2026/02/28，2026/05/25，2026/06/13，2026/07/05，2026/07/18，2026/08/08</t>
+          <t>2026/02/08，2026/02/09，2026/02/14，2026/02/20，2026/02/28，2026/05/25，2026/06/13，2026/07/05，2026/07/18，2026/08/08，2026/08/23</t>
         </is>
       </c>
       <c r="F787" t="inlineStr"/>
@@ -31918,7 +31910,7 @@
       </c>
       <c r="H787" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I787" t="inlineStr">
@@ -32075,7 +32067,7 @@
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>2026/02/14，2026/02/24，2026/03/07，2026/03/13，2026/05/26，2026/06/19</t>
+          <t>2026/02/14，2026/02/24，2026/03/07，2026/03/13，2026/05/26，2026/06/19，2026/08/25</t>
         </is>
       </c>
       <c r="F791" t="inlineStr"/>
@@ -32086,7 +32078,7 @@
       </c>
       <c r="H791" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I791" t="inlineStr">
@@ -32355,7 +32347,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>2026/02/22，2026/02/23，2026/02/24，2026/02/25，2026/03/14，2026/04/20，2026/06/16，2026/08/01</t>
+          <t>2026/02/22，2026/02/23，2026/02/24，2026/02/25，2026/03/14，2026/04/20，2026/06/16，2026/08/01，2026/8/27</t>
         </is>
       </c>
       <c r="F798" t="inlineStr"/>
@@ -32366,7 +32358,7 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I798" t="inlineStr">
@@ -33379,7 +33371,7 @@
       </c>
       <c r="E823" t="inlineStr">
         <is>
-          <t>2026/03/17，2026/03/17，2026/03/25，2026/03/27，2026/03/29，2026/04/02，2026/04/08，2026/04/16，2026/04/20，2026/05/02，2026/05/06，2026/05/26，2026/06/14，2026/07/18，2026/08/08</t>
+          <t>2026/03/17，2026/03/17，2026/03/25，2026/03/27，2026/03/29，2026/04/02，2026/04/08，2026/04/16，2026/04/20，2026/05/02，2026/05/06，2026/05/26，2026/06/14，2026/07/18，2026/08/08，2026/08/21</t>
         </is>
       </c>
       <c r="F823" t="inlineStr"/>
@@ -33390,7 +33382,7 @@
       </c>
       <c r="H823" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I823" t="inlineStr">
@@ -33475,7 +33467,7 @@
       </c>
       <c r="E825" t="inlineStr">
         <is>
-          <t>2026/03/25，2026/04/14，2026/05/25，2026/05/25，2026/06/25，2026/06/25，2026/06/25，2026/06/26，2026/07/07，2026/08/09</t>
+          <t>2026/03/25，2026/04/14，2026/05/25，2026/05/25，2026/06/25，2026/06/25，2026/06/25，2026/06/26，2026/07/07，2026/08/09，2026/08/25</t>
         </is>
       </c>
       <c r="F825" t="inlineStr"/>
@@ -33486,7 +33478,7 @@
       </c>
       <c r="H825" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I825" t="inlineStr">
@@ -34583,7 +34575,7 @@
       </c>
       <c r="E852" t="inlineStr">
         <is>
-          <t>2026/05/01，2026/07/31，2026/08/01，2026/08/08，2026/08/11</t>
+          <t>2026/05/01，2026/07/31，2026/08/01，2026/08/08，2026/08/11，2026/08/25</t>
         </is>
       </c>
       <c r="F852" t="inlineStr"/>
@@ -34594,7 +34586,7 @@
       </c>
       <c r="H852" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I852" t="inlineStr">
@@ -34879,7 +34871,7 @@
       </c>
       <c r="E859" t="inlineStr">
         <is>
-          <t>2026/05/25，2026/05/25，2026/05/25，2026/05/26，2026/05/26，2026/06/25，2026/06/26，2026/07/09，2026/07/16</t>
+          <t>2026/05/25，2026/05/25，2026/05/25，2026/05/26，2026/05/26，2026/06/25，2026/06/26，2026/07/09，2026/07/16，2026/08/23，2026/08/23</t>
         </is>
       </c>
       <c r="F859" t="inlineStr"/>
@@ -34890,7 +34882,7 @@
       </c>
       <c r="H859" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I859" t="inlineStr">
@@ -35327,7 +35319,7 @@
       </c>
       <c r="E870" t="inlineStr">
         <is>
-          <t>2026/06/20</t>
+          <t>2026/06/20，2026/08/23</t>
         </is>
       </c>
       <c r="F870" t="inlineStr"/>
@@ -35338,7 +35330,7 @@
       </c>
       <c r="H870" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I870" t="inlineStr">
@@ -35451,7 +35443,7 @@
       </c>
       <c r="E873" t="inlineStr">
         <is>
-          <t>2026/06/25，2026/07/09，2026/07/18，2026/07/31</t>
+          <t>2026/06/25，2026/07/09，2026/07/18，2026/07/31，2026/08/25</t>
         </is>
       </c>
       <c r="F873" t="inlineStr"/>
@@ -35462,7 +35454,7 @@
       </c>
       <c r="H873" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I873" t="inlineStr">
@@ -35615,7 +35607,7 @@
       </c>
       <c r="E877" t="inlineStr">
         <is>
-          <t>2026/07/07，2026/07/09，2026/07/10，2026/07/15，2026/07/16，2026/07/18，2026/07/25，2026/07/27，2026/08/01，2026/08/08，2026/08/11</t>
+          <t>2026/07/07，2026/07/09，2026/07/10，2026/07/15，2026/07/16，2026/07/18，2026/07/25，2026/07/27，2026/08/01，2026/08/08，2026/08/11，2026/08/18，2026/08/23，2026/08/25，2026/8/28</t>
         </is>
       </c>
       <c r="F877" t="inlineStr"/>
@@ -35626,7 +35618,7 @@
       </c>
       <c r="H877" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I877" t="inlineStr">
@@ -35735,7 +35727,7 @@
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08</t>
+          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08，2026/8/28</t>
         </is>
       </c>
       <c r="F880" t="inlineStr"/>
@@ -35746,7 +35738,7 @@
       </c>
       <c r="H880" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I880" t="inlineStr">
@@ -35935,7 +35927,7 @@
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>2026/08/03，2026/08/08，2026/08/09，2026/08/11</t>
+          <t>2026/08/03，2026/08/08，2026/08/09，2026/08/11，2026/08/18，2026/08/25</t>
         </is>
       </c>
       <c r="F885" t="inlineStr"/>
@@ -35946,7 +35938,7 @@
       </c>
       <c r="H885" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I885" t="inlineStr">
@@ -36015,7 +36007,7 @@
       </c>
       <c r="E887" t="inlineStr">
         <is>
-          <t>2026/08/05，2025/05/03</t>
+          <t>2025/05/03，2026/08/05</t>
         </is>
       </c>
       <c r="F887" t="inlineStr"/>
@@ -36055,7 +36047,7 @@
       </c>
       <c r="E888" t="inlineStr">
         <is>
-          <t>2026/08/11，2026/08/11</t>
+          <t>2026/08/11，2026/08/11，2026/08/18，2026/08/25</t>
         </is>
       </c>
       <c r="F888" t="inlineStr"/>
@@ -36066,10 +36058,14 @@
       </c>
       <c r="H888" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I888" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>BV1oBui6sEzT</t>
+        </is>
+      </c>
       <c r="J888" t="inlineStr"/>
     </row>
     <row r="889">
@@ -36105,8 +36101,412 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I889" t="inlineStr"/>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>BV1DQui61EPb</t>
+        </is>
+      </c>
       <c r="J889" t="inlineStr"/>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>889</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>迷宫</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr"/>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>step.jad依加</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>2026/08/18，2026/08/19，2026/08/23</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr"/>
+      <c r="G890" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>BV1UL836dEFE</t>
+        </is>
+      </c>
+      <c r="J890" t="inlineStr"/>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>890</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>爱你但说不出口</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr"/>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Karencici</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>2026/08/18</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr"/>
+      <c r="G891" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>BV1e1836KEbJ</t>
+        </is>
+      </c>
+      <c r="J891" t="inlineStr"/>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>891</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>写一首歌April 5,1969</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr"/>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>顺子</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>2026/08/18</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr"/>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>BV1xw8G6sEvA</t>
+        </is>
+      </c>
+      <c r="J892" t="inlineStr"/>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>892</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Black Sheep</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr"/>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Gin Wigmore</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>2026/08/18</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr"/>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>BV1Ps836DEGr</t>
+        </is>
+      </c>
+      <c r="J893" t="inlineStr"/>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>893</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Get Jinxed</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr"/>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Agnete Kjolsund</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>2026/08/19</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr"/>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>BV1t58n6EEBo</t>
+        </is>
+      </c>
+      <c r="J894" t="inlineStr"/>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>894</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>涅槃</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>英雄联盟/Cailin Russo/Chrissy Costanza</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>2026/08/19，2026/08/21</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr"/>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>BV1zA8B6SEvE</t>
+        </is>
+      </c>
+      <c r="J895" t="inlineStr"/>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>895</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>才二十三</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr"/>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>方大同</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>2026/08/23，2026/08/25</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr"/>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>BV1Ko886rE7j</t>
+        </is>
+      </c>
+      <c r="J896" t="inlineStr"/>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>896</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>入秋的第一场雨真让人矫情</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr"/>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>ChiliChill</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>2026/08/23</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr"/>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>BV1cs886YEQS</t>
+        </is>
+      </c>
+      <c r="J897" t="inlineStr"/>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>897</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>芭蕉夜雨</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr"/>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>ChiliChill</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>2026/08/23</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr"/>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>BV1ns886YEqh</t>
+        </is>
+      </c>
+      <c r="J898" t="inlineStr"/>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>898</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>summer vibe</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr"/>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Walk off the Earth</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>2026/08/25</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr"/>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr"/>
+      <c r="J899" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Aug.30, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J899"/>
+  <dimension ref="A1:J904"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/03/15，2026/06/23</t>
+          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/03/15，2026/06/23，2026/8/30</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/07，2025/12/16，2025/12/28，2026/01/10，2026/01/15，2026/02/19，2026/03/07，2026/03/17，2026/03/21，2026/05/06，2026/07/05，2026/07/20</t>
+          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/07，2025/12/16，2025/12/28，2026/01/10，2026/01/15，2026/02/19，2026/03/07，2026/03/17，2026/03/21，2026/05/06，2026/07/05，2026/07/20，2026/8/30</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2025/03/08，2025/04/06，2025/05/15，2025/05/26，2025/07/22，2025/09/17，2025/12/30，2026/02/14，2026/05/04</t>
+          <t>2025/03/08，2025/04/06，2025/05/15，2025/05/26，2025/07/22，2025/09/17，2025/12/30，2026/02/14，2026/05/04，2026/8/30</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/05/05，2025/05/13，2025/05/24，2025/08/12，2025/08/30，2025/11/26，2026/08/21</t>
+          <t>2025/03/10，2025/05/05，2025/05/13，2025/05/24，2025/08/12，2025/08/30，2025/11/26，2026/08/21，2026/8/30</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3630,7 +3630,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/17，2025/05/04，2025/05/13，2025/07/22，2025/09/05，2025/09/28，2026/06/03</t>
+          <t>2025/03/13，2025/04/17，2025/05/04，2025/05/13，2025/07/22，2025/09/05，2025/09/28，2026/06/03，2026/8/30</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/02/10，2026/02/24，2026/03/18，2026/05/20，2026/06/19，2026/08/25</t>
+          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/02/10，2026/02/24，2026/03/18，2026/05/20，2026/06/19，2026/08/25，2026/8/30</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/01/12，2026/02/07，2026/03/15，2026/04/19，2026/06/26，2026/08/25</t>
+          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/01/12，2026/02/07，2026/03/15，2026/04/19，2026/06/26，2026/08/25，2026/8/30</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/10/11，2025/11/14</t>
+          <t>2025/03/14，2025/10/11，2025/11/14，2026/8/30</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/01/19，2026/04/18，2026/05/01，2026/05/23，2026/07/17，2026/08/25</t>
+          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/01/19，2026/04/18，2026/05/01，2026/05/23，2026/07/17，2026/08/25，2026/8/30</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/06/26，2025/08/04，2025/09/18，2025/10/25，2026/03/05，2026/07/28</t>
+          <t>2025/03/15，2025/06/26，2025/08/04，2025/09/18，2025/10/25，2026/03/05，2026/07/28，2026/8/30</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/29，2025/06/03，2025/07/24，2025/08/01，2025/08/03，2025/10/10，2025/11/09，2026/04/26，2026/08/02</t>
+          <t>2025/03/17，2025/04/29，2025/06/03，2025/07/24，2025/08/01，2025/08/03，2025/10/10，2025/11/09，2026/04/26，2026/08/02，2026/8/30</t>
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
@@ -6018,7 +6018,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/02，2025/09/12，2025/11/09，2025/12/04，2026/01/01，2026/01/29，2026/04/09，2026/06/15，2026/08/05</t>
+          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/02，2025/09/12，2025/11/09，2025/12/04，2026/01/01，2026/01/29，2026/04/09，2026/06/15，2026/08/05，2026/8/30</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -6058,7 +6058,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08，2026/08/23</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08，2026/08/23，2026/8/30</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/02，2026/01/16，2026/02/02，2026/02/23，2026/02/25，2026/03/17，2026/04/08，2026/05/06，2026/05/21，2026/06/25，2026/07/18，2026/08/25</t>
+          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/02，2026/01/16，2026/02/02，2026/02/23，2026/02/25，2026/03/17，2026/04/08，2026/05/06，2026/05/21，2026/06/25，2026/07/18，2026/08/25，2026/8/30</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/06/28，2025/08/04，2026/01/19，2026/04/08</t>
+          <t>2025/03/21，2025/06/28，2025/08/04，2026/01/19，2026/04/08，2026/8/30</t>
         </is>
       </c>
       <c r="F163" t="inlineStr"/>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/12，2025/12/07，2026/04/24</t>
+          <t>2025/03/21，2025/05/12，2025/12/07，2026/04/24，2026/8/30</t>
         </is>
       </c>
       <c r="F164" t="inlineStr"/>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -8615,7 +8615,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/09/24，2025/11/27，2026/04/14，2026/06/10</t>
+          <t>2025/03/25，2025/09/24，2025/11/27，2026/04/14，2026/06/10，2026/8/30</t>
         </is>
       </c>
       <c r="F202" t="inlineStr"/>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/03/25，2026/04/09，2026/05/10，2026/06/10</t>
+          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/03/25，2026/04/09，2026/05/10，2026/06/10，2026/8/30</t>
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
@@ -9118,7 +9118,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/23，2025/06/13，2025/06/26，2025/07/11，2025/09/18，2025/11/03，2025/12/23，2025/12/26，2026/01/24，2026/06/03，2026/07/18</t>
+          <t>2025/03/28，2025/05/23，2025/06/13，2025/06/26，2025/07/11，2025/09/18，2025/11/03，2025/12/23，2025/12/26，2026/01/24，2026/06/03，2026/07/18，2026/8/30，2026/8/30</t>
         </is>
       </c>
       <c r="F220" t="inlineStr"/>
@@ -9354,7 +9354,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/03，2025/11/09，2025/12/23，2026/04/08，2026/04/24，2026/05/21，2026/06/10，2026/08/02，2026/8/28</t>
+          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/03，2025/11/09，2025/12/23，2026/04/08，2026/04/24，2026/05/21，2026/06/10，2026/08/02，2026/8/28，2026/8/30</t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
@@ -9954,7 +9954,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/22，2025/06/29，2025/09/30，2025/10/23，2026/01/19，2026/08/18</t>
+          <t>2025/03/30，2025/05/22，2025/06/29，2025/09/30，2025/10/23，2026/01/19，2026/08/18，2026/8/30</t>
         </is>
       </c>
       <c r="F243" t="inlineStr"/>
@@ -10282,7 +10282,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>2025/03/30</t>
+          <t>2025/03/30，2026/8/30</t>
         </is>
       </c>
       <c r="F249" t="inlineStr"/>
@@ -10522,7 +10522,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I249" t="inlineStr"/>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/27，2025/07/24，2026/01/01，2026/06/14</t>
+          <t>2025/04/02，2025/05/27，2025/07/24，2026/01/01，2026/06/14，2026/8/30</t>
         </is>
       </c>
       <c r="F265" t="inlineStr"/>
@@ -11158,7 +11158,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/13，2025/05/10，2025/05/26，2025/06/02，2025/06/05，2025/06/17，2025/08/04，2025/09/10，2025/09/30，2025/10/16，2025/11/17，2025/12/06，2025/12/31，2026/04/26，2026/07/22</t>
+          <t>2025/04/02，2025/04/13，2025/05/10，2025/05/26，2025/06/02，2025/06/05，2025/06/17，2025/08/04，2025/09/10，2025/09/30，2025/10/16，2025/11/17，2025/12/06，2025/12/31，2026/04/26，2026/07/22，2026/8/30</t>
         </is>
       </c>
       <c r="F269" t="inlineStr"/>
@@ -11318,7 +11318,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/03/09，2026/03/13，2026/03/17，2026/05/01，2026/06/18</t>
+          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/03/09，2026/03/13，2026/03/17，2026/05/01，2026/06/18，2026/8/30</t>
         </is>
       </c>
       <c r="F274" t="inlineStr"/>
@@ -11522,7 +11522,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/14，2025/04/24，2025/06/01，2025/07/06，2025/09/21，2025/11/03，2025/12/12，2025/12/26，2026/04/08，2026/07/20</t>
+          <t>2025/04/03，2025/04/14，2025/04/24，2025/06/01，2025/07/06，2025/09/21，2025/11/03，2025/12/12，2025/12/26，2026/04/08，2026/07/20，2026/8/30</t>
         </is>
       </c>
       <c r="F277" t="inlineStr"/>
@@ -11642,7 +11642,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -11831,7 +11831,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/05/12，2025/05/18，2025/06/20，2025/07/05，2025/07/14，2025/12/23，2026/01/30，2026/04/09</t>
+          <t>2025/04/04，2025/05/12，2025/05/18，2025/06/20，2025/07/05，2025/07/14，2025/12/23，2026/01/30，2026/04/09，2026/8/30</t>
         </is>
       </c>
       <c r="F282" t="inlineStr"/>
@@ -11842,7 +11842,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -12183,7 +12183,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/07/13，2025/07/18，2025/11/03，2025/11/28，2026/08/16</t>
+          <t>2025/04/04，2025/07/13，2025/07/18，2025/11/03，2025/11/28，2026/08/16，2026/8/30</t>
         </is>
       </c>
       <c r="F291" t="inlineStr"/>
@@ -12194,7 +12194,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -12667,7 +12667,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/05/09，2025/06/19，2025/07/22，2026/03/09</t>
+          <t>2025/04/07，2025/05/09，2025/06/19，2025/07/22，2026/03/09，2026/8/30</t>
         </is>
       </c>
       <c r="F303" t="inlineStr"/>
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -12747,7 +12747,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23</t>
+          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23，2026/8/30</t>
         </is>
       </c>
       <c r="F305" t="inlineStr"/>
@@ -12758,7 +12758,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -13939,7 +13939,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>2025/04/12</t>
+          <t>2025/04/12，2026/8/30</t>
         </is>
       </c>
       <c r="F335" t="inlineStr"/>
@@ -13950,7 +13950,7 @@
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I335" t="inlineStr"/>
@@ -14111,7 +14111,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/18，2025/08/28，2026/01/16，2026/05/01</t>
+          <t>2025/04/13，2025/04/18，2025/08/28，2026/01/16，2026/05/01，2026/8/30</t>
         </is>
       </c>
       <c r="F339" t="inlineStr"/>
@@ -14122,7 +14122,7 @@
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I339" t="inlineStr">
@@ -15283,7 +15283,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/06/17，2025/08/28</t>
+          <t>2025/04/19，2025/06/17，2025/08/28，2026/8/30</t>
         </is>
       </c>
       <c r="F368" t="inlineStr"/>
@@ -15294,7 +15294,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -17063,7 +17063,7 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>2025/05/01，2025/08/12，2025/08/26，2025/11/24，2026/06/20</t>
+          <t>2025/05/01，2025/08/12，2025/08/26，2025/11/24，2026/06/20，2026/8/30</t>
         </is>
       </c>
       <c r="F413" t="inlineStr"/>
@@ -17074,7 +17074,7 @@
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
@@ -17263,7 +17263,7 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/06/13，2025/09/08，2026/04/25</t>
+          <t>2025/05/03，2025/06/13，2025/09/08，2026/04/25，2026/8/30</t>
         </is>
       </c>
       <c r="F418" t="inlineStr"/>
@@ -17274,7 +17274,7 @@
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
@@ -18499,7 +18499,7 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/12/16，2025/12/24，2026/08/16</t>
+          <t>2025/05/19，2025/12/16，2025/12/24，2026/08/16，2026/8/30</t>
         </is>
       </c>
       <c r="F449" t="inlineStr"/>
@@ -18510,7 +18510,7 @@
       </c>
       <c r="H449" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I449" t="inlineStr">
@@ -18743,7 +18743,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/09/02，2025/09/12，2025/12/05，2026/04/09，2026/05/10</t>
+          <t>2025/05/22，2025/09/02，2025/09/12，2025/12/05，2026/04/09，2026/05/10，2026/8/30</t>
         </is>
       </c>
       <c r="F455" t="inlineStr"/>
@@ -18754,7 +18754,7 @@
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I455" t="inlineStr">
@@ -19075,7 +19075,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>2025/05/23</t>
+          <t>2025/05/23，2026/8/30</t>
         </is>
       </c>
       <c r="F463" t="inlineStr"/>
@@ -19086,7 +19086,7 @@
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I463" t="inlineStr">
@@ -19675,7 +19675,7 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/09/03，2025/09/11，2025/09/29，2025/11/09，2026/01/01，2026/04/20</t>
+          <t>2025/05/30，2025/09/03，2025/09/11，2025/09/29，2025/11/09，2026/01/01，2026/04/20，2026/8/30</t>
         </is>
       </c>
       <c r="F478" t="inlineStr"/>
@@ -19686,7 +19686,7 @@
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I478" t="inlineStr">
@@ -21759,7 +21759,7 @@
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/07，2025/11/21，2025/12/02，2025/12/17，2026/01/01，2026/01/05，2026/01/14，2026/01/22，2026/01/24，2026/02/02，2026/03/05，2026/03/15，2026/04/01，2026/05/04，2026/05/25，2026/06/20，2026/07/05，2026/07/18，2026/07/28，2026/08/11</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/07，2025/11/21，2025/12/02，2025/12/17，2026/01/01，2026/01/05，2026/01/14，2026/01/22，2026/01/24，2026/02/02，2026/03/05，2026/03/15，2026/04/01，2026/05/04，2026/05/25，2026/06/20，2026/07/05，2026/07/18，2026/07/28，2026/08/11，2026/8/30</t>
         </is>
       </c>
       <c r="F530" t="inlineStr"/>
@@ -21770,7 +21770,7 @@
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I530" t="inlineStr">
@@ -22083,7 +22083,7 @@
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>2025/06/23</t>
+          <t>2025/06/23，2026/8/30</t>
         </is>
       </c>
       <c r="F538" t="inlineStr"/>
@@ -22094,7 +22094,7 @@
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I538" t="inlineStr">
@@ -22699,7 +22699,7 @@
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/08/16</t>
+          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/08/16，2026/8/30</t>
         </is>
       </c>
       <c r="F553" t="inlineStr"/>
@@ -22710,7 +22710,7 @@
       </c>
       <c r="H553" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I553" t="inlineStr">
@@ -22739,7 +22739,7 @@
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>2025/06/29，2026/08/11，2026/08/21</t>
+          <t>2025/06/29，2026/08/11，2026/08/21，2026/8/30</t>
         </is>
       </c>
       <c r="F554" t="inlineStr"/>
@@ -22750,7 +22750,7 @@
       </c>
       <c r="H554" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I554" t="inlineStr">
@@ -22819,7 +22819,7 @@
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>2025/06/29</t>
+          <t>2025/06/29，2026/8/30</t>
         </is>
       </c>
       <c r="F556" t="inlineStr"/>
@@ -22830,7 +22830,7 @@
       </c>
       <c r="H556" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I556" t="inlineStr">
@@ -22859,7 +22859,7 @@
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>2025/06/29</t>
+          <t>2025/06/29，2026/8/30</t>
         </is>
       </c>
       <c r="F557" t="inlineStr"/>
@@ -22870,7 +22870,7 @@
       </c>
       <c r="H557" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I557" t="inlineStr">
@@ -26299,7 +26299,7 @@
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/03，2025/11/13，2025/11/24，2025/12/05，2025/12/12，2025/12/17，2026/01/06，2026/01/15，2026/01/24，2026/02/27，2026/04/19，2026/06/06，2026/07/17，2026/07/28，2026/8/28</t>
+          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/03，2025/11/13，2025/11/24，2025/12/05，2025/12/12，2025/12/17，2026/01/06，2026/01/15，2026/01/24，2026/02/27，2026/04/19，2026/06/06，2026/07/17，2026/07/28，2026/8/28，2026/8/30</t>
         </is>
       </c>
       <c r="F644" t="inlineStr"/>
@@ -26310,7 +26310,7 @@
       </c>
       <c r="H644" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I644" t="inlineStr">
@@ -27263,7 +27263,7 @@
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/26，2025/09/28，2025/09/29，2025/10/01，2025/10/07，2025/10/10，2025/10/11，2025/10/17，2025/10/23，2025/10/28，2025/12/26，2026/02/05，2026/07/16，2026/07/31，2026/08/19</t>
+          <t>2025/09/24，2025/09/26，2025/09/28，2025/09/29，2025/10/01，2025/10/07，2025/10/10，2025/10/11，2025/10/17，2025/10/23，2025/10/28，2025/12/26，2026/02/05，2026/07/16，2026/07/31，2026/08/19，2026/8/30</t>
         </is>
       </c>
       <c r="F669" t="inlineStr"/>
@@ -27274,7 +27274,7 @@
       </c>
       <c r="H669" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I669" t="inlineStr">
@@ -34655,7 +34655,7 @@
       </c>
       <c r="E854" t="inlineStr">
         <is>
-          <t>2026/05/01，2026/08/02</t>
+          <t>2026/05/01，2026/08/02，2026/8/30</t>
         </is>
       </c>
       <c r="F854" t="inlineStr"/>
@@ -34666,7 +34666,7 @@
       </c>
       <c r="H854" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I854" t="inlineStr">
@@ -36127,7 +36127,7 @@
       </c>
       <c r="E890" t="inlineStr">
         <is>
-          <t>2026/08/18，2026/08/19，2026/08/23</t>
+          <t>2026/08/18，2026/08/19，2026/08/23，2026/8/30</t>
         </is>
       </c>
       <c r="F890" t="inlineStr"/>
@@ -36138,7 +36138,7 @@
       </c>
       <c r="H890" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I890" t="inlineStr">
@@ -36480,7 +36480,7 @@
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>summer vibe</t>
+          <t>Summer Vibe</t>
         </is>
       </c>
       <c r="C899" t="inlineStr"/>
@@ -36505,8 +36505,212 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I899" t="inlineStr"/>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>BV1mY496eEud</t>
+        </is>
+      </c>
       <c r="J899" t="inlineStr"/>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>899</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>All About That Bass</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr"/>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Meghan Trainor</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>2026/8/30</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr"/>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>BV1y4th6AEz2</t>
+        </is>
+      </c>
+      <c r="J900" t="inlineStr"/>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Last Friday Night</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr"/>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Katy Perry</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>2026/8/30</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr"/>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>BV12Hth6iEup</t>
+        </is>
+      </c>
+      <c r="J901" t="inlineStr"/>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>901</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Tik Tok</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr"/>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Kesha</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>2026/8/30，2026/8/30</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr"/>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>BV1w8th6wERB</t>
+        </is>
+      </c>
+      <c r="J902" t="inlineStr"/>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Honeymoon Avenue</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr"/>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>Ariana Grande</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>2026/8/30</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr"/>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>BV1k8th6cEpk</t>
+        </is>
+      </c>
+      <c r="J903" t="inlineStr"/>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>903</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Love Me Like You Do</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr"/>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>Ellie Goulding</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>2026/8/30</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr"/>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>BV12wta6uEUK</t>
+        </is>
+      </c>
+      <c r="J904" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Sep.2, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J904"/>
+  <dimension ref="A1:J905"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -703,7 +703,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/01，2025/11/17，2025/12/02，2025/12/31，2026/02/02，2026/02/14，2026/03/06，2026/04/01，2026/04/20，2026/05/15，2026/06/10，2026/07/22，2026/08/09</t>
+          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/01，2025/11/17，2025/12/02，2025/12/31，2026/02/02，2026/02/14，2026/03/06，2026/04/01，2026/04/20，2026/05/15，2026/06/10，2026/07/22，2026/08/09，2026/9/2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -714,7 +714,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/09，2025/11/19，2025/12/16，2026/01/16，2026/01/28，2026/02/07，2026/02/10，2026/03/17，2026/04/19，2026/05/23，2026/06/19，2026/07/22，2026/08/08</t>
+          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/09，2025/11/19，2025/12/16，2026/01/16，2026/01/28，2026/02/07，2026/02/10，2026/03/17，2026/04/19，2026/05/23，2026/06/19，2026/07/22，2026/08/08，2026/9/2</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -758,7 +758,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/07，2025/12/24，2026/01/01，2026/01/16，2026/03/14，2026/05/01，2026/05/20，2026/08/01</t>
+          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/07，2025/12/24，2026/01/01，2026/01/16，2026/03/14，2026/05/01，2026/05/20，2026/08/01，2026/9/2</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1722,7 +1722,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/18，2025/05/03，2025/05/08，2025/06/05，2025/06/19，2025/07/15，2025/09/08，2025/10/07，2025/10/17，2025/10/23，2025/12/24</t>
+          <t>2025/03/04，2025/04/18，2025/05/03，2025/05/08，2025/06/05，2025/06/19，2025/07/15，2025/09/08，2025/10/07，2025/10/17，2025/10/23，2025/12/24，2026/9/2</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2002,7 +2002,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/18，2025/07/26，2025/08/12，2025/11/28，2026/02/19，2026/03/04，2026/07/17</t>
+          <t>2025/03/04，2025/05/18，2025/07/26，2025/08/12，2025/11/28，2026/02/19，2026/03/04，2026/07/17，2026/9/2</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/01/09，2026/01/28，2026/02/25，2026/03/12，2026/03/21，2026/04/26，2026/05/10，2026/06/26</t>
+          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/01/09，2026/01/28，2026/02/25，2026/03/12，2026/03/21，2026/04/26，2026/05/10，2026/06/26，2026/9/2</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/01，2025/11/09，2025/12/04，2025/12/16，2025/12/31，2026/01/09，2026/01/15，2026/01/21，2026/01/23，2026/01/29，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/02/24，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/05，2026/03/07，2026/03/08，2026/03/09，2026/03/12，2026/03/13，2026/03/14，2026/03/15，2026/03/17，2026/03/18，2026/03/19，2026/03/22，2026/03/24，2026/03/27，2026/03/28，2026/03/31，2026/04/08，2026/04/14，2026/04/18，2026/04/25，2026/05/01，2026/05/15，2026/05/25，2026/06/12，2026/06/23，2026/06/26，2026/07/04，2026/07/20，2026/07/30，2026/08/09，2026/8/28</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/01，2025/11/09，2025/12/04，2025/12/16，2025/12/31，2026/01/09，2026/01/15，2026/01/21，2026/01/23，2026/01/29，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/02/24，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/05，2026/03/07，2026/03/08，2026/03/09，2026/03/12，2026/03/13，2026/03/14，2026/03/15，2026/03/17，2026/03/18，2026/03/19，2026/03/22，2026/03/24，2026/03/27，2026/03/28，2026/03/31，2026/04/08，2026/04/14，2026/04/18，2026/04/25，2026/05/01，2026/05/15，2026/05/25，2026/06/12，2026/06/23，2026/06/26，2026/07/04，2026/07/20，2026/07/30，2026/08/09，2026/8/28，2026/9/2</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>74</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/30，2025/04/10，2025/04/20，2025/05/04，2025/05/13，2025/05/22，2025/06/05，2025/06/07，2025/08/29，2025/09/07，2025/09/11，2025/10/10，2025/11/09，2026/01/01，2026/06/20，2026/07/30</t>
+          <t>2025/03/09，2025/03/30，2025/04/10，2025/04/20，2025/05/04，2025/05/13，2025/05/22，2025/06/05，2025/06/07，2025/08/29，2025/09/07，2025/09/11，2025/10/10，2025/11/09，2026/01/01，2026/06/20，2026/07/30，2026/9/2</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/05/12，2025/06/12，2025/07/21，2025/12/11，2026/01/15，2026/03/01，2026/05/05，2026/07/16</t>
+          <t>2025/03/09，2025/05/12，2025/06/12，2025/07/21，2025/12/11，2026/01/15，2026/03/01，2026/05/05，2026/07/16，2026/9/2</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/03/27，2026/04/01，2026/06/23，2026/07/31</t>
+          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/03/27，2026/04/01，2026/06/23，2026/07/31，2026/9/2</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3542,7 +3542,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/01/01，2026/02/14，2026/05/06，2026/05/23，2026/07/07，2026/08/02</t>
+          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/01/01，2026/02/14，2026/05/06，2026/05/23，2026/07/07，2026/08/02，2026/9/2</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/03，2025/12/02，2025/12/04，2025/12/12，2026/01/05，2026/01/14，2026/02/19，2026/03/04，2026/03/31，2026/04/12，2026/04/29，2026/05/15，2026/06/12，2026/06/23，2026/07/09，2026/08/11</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/03，2025/12/02，2025/12/04，2025/12/12，2026/01/05，2026/01/14，2026/02/19，2026/03/04，2026/03/31，2026/04/12，2026/04/29，2026/05/15，2026/06/12，2026/06/23，2026/07/09，2026/08/11，2026/9/2</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/08，2025/04/18，2025/05/12，2025/05/23，2025/06/27，2025/07/24，2025/08/28，2025/10/11，2025/10/31，2025/11/24，2025/12/19，2026/02/02，2026/04/19，2026/07/25</t>
+          <t>2025/03/19，2025/04/08，2025/04/18，2025/05/12，2025/05/23，2025/06/27，2025/07/24，2025/08/28，2025/10/11，2025/10/31，2025/11/24，2025/12/19，2026/02/02，2026/04/19，2026/07/25，2026/9/2</t>
         </is>
       </c>
       <c r="F145" t="inlineStr"/>
@@ -6338,7 +6338,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -7331,7 +7331,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/06，2026/02/07，2026/03/24，2026/04/26，2026/05/04，2026/05/23，2026/07/09，2026/07/27</t>
+          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/06，2026/02/07，2026/03/24，2026/04/26，2026/05/04，2026/05/23，2026/07/09，2026/07/27，2026/9/2</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -7342,7 +7342,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -9263,7 +9263,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/01/16，2026/06/06，2026/07/09，2026/08/08</t>
+          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/01/16，2026/06/06，2026/07/09，2026/08/08，2026/9/2</t>
         </is>
       </c>
       <c r="F218" t="inlineStr"/>
@@ -9274,7 +9274,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/08/16</t>
+          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/08/16，2026/9/2</t>
         </is>
       </c>
       <c r="F228" t="inlineStr"/>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -11267,7 +11267,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/12，2025/05/23，2025/06/08，2025/07/29，2025/08/13，2025/08/28，2025/09/28，2025/09/29，2025/11/09，2025/12/06，2025/12/24，2026/04/13，2026/05/04，2026/07/27</t>
+          <t>2025/04/02，2025/04/12，2025/05/23，2025/06/08，2025/07/29，2025/08/13，2025/08/28，2025/09/28，2025/09/29，2025/11/09，2025/12/06，2025/12/24，2026/04/13，2026/05/04，2026/07/27，2026/9/2</t>
         </is>
       </c>
       <c r="F268" t="inlineStr"/>
@@ -11278,7 +11278,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/06/02，2025/06/29，2025/07/24，2025/07/26，2025/08/21，2025/11/09，2025/12/16</t>
+          <t>2025/04/04，2025/06/02，2025/06/29，2025/07/24，2025/07/26，2025/08/21，2025/11/09，2025/12/16，2026/9/2</t>
         </is>
       </c>
       <c r="F283" t="inlineStr"/>
@@ -11882,7 +11882,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -12947,7 +12947,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/09，2026/01/24，2026/03/31，2026/04/02，2026/06/15，2026/07/27</t>
+          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/09，2026/01/24，2026/03/31，2026/04/02，2026/06/15，2026/07/27，2026/9/2</t>
         </is>
       </c>
       <c r="F310" t="inlineStr"/>
@@ -12958,7 +12958,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -14019,7 +14019,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/21，2025/04/22，2025/04/25，2025/04/26，2025/04/29，2025/05/08，2025/05/12，2025/05/22，2025/05/30，2025/06/06，2025/06/08，2025/06/28，2025/07/13，2025/08/12，2025/08/24，2025/09/07，2025/09/30，2025/10/05，2025/11/21，2025/12/17，2026/01/14，2026/01/23，2026/02/12，2026/03/31，2026/06/18，2026/07/17</t>
+          <t>2025/04/13，2025/04/21，2025/04/22，2025/04/25，2025/04/26，2025/04/29，2025/05/08，2025/05/12，2025/05/22，2025/05/30，2025/06/06，2025/06/08，2025/06/28，2025/07/13，2025/08/12，2025/08/24，2025/09/07，2025/09/30，2025/10/05，2025/11/21，2025/12/17，2026/01/14，2026/01/23，2026/02/12，2026/03/31，2026/06/18，2026/07/17，2026/9/2</t>
         </is>
       </c>
       <c r="F337" t="inlineStr"/>
@@ -14030,7 +14030,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/05/13，2025/07/14，2025/09/18，2026/01/01，2026/01/09，2026/02/20，2026/04/18，2026/05/10，2026/07/16</t>
+          <t>2025/04/15，2025/05/13，2025/07/14，2025/09/18，2026/01/01，2026/01/09，2026/02/20，2026/04/18，2026/05/10，2026/07/16，2026/9/2</t>
         </is>
       </c>
       <c r="F346" t="inlineStr"/>
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
@@ -15611,7 +15611,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>2025/04/21，2025/05/23，2025/06/29，2025/07/26，2025/09/28，2025/12/02，2025/12/17，2026/05/06</t>
+          <t>2025/04/21，2025/05/23，2025/06/29，2025/07/26，2025/09/28，2025/12/02，2025/12/17，2026/05/06，2026/9/2</t>
         </is>
       </c>
       <c r="F376" t="inlineStr"/>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">
@@ -16867,7 +16867,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/05/12，2025/05/23，2025/07/20，2025/10/18，2026/01/19，2026/07/27</t>
+          <t>2025/04/28，2025/05/12，2025/05/23，2025/07/20，2025/10/18，2026/01/19，2026/07/27，2026/9/2</t>
         </is>
       </c>
       <c r="F408" t="inlineStr"/>
@@ -16878,7 +16878,7 @@
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I408" t="inlineStr">
@@ -17819,7 +17819,7 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/04/29，2026/08/07</t>
+          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/04/29，2026/08/07，2026/9/2</t>
         </is>
       </c>
       <c r="F432" t="inlineStr"/>
@@ -17830,7 +17830,7 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I432" t="inlineStr">
@@ -18911,7 +18911,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/01/05，2026/02/02，2026/03/17，2026/05/10，2026/06/14，2026/06/15，2026/07/31</t>
+          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/01/05，2026/02/02，2026/03/17，2026/05/10，2026/06/14，2026/06/15，2026/07/31，2026/9/2</t>
         </is>
       </c>
       <c r="F459" t="inlineStr"/>
@@ -18922,7 +18922,7 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
@@ -19395,7 +19395,7 @@
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>2025/05/26，2025/07/03，2025/09/15</t>
+          <t>2025/05/26，2025/07/03，2025/09/15，2026/9/2</t>
         </is>
       </c>
       <c r="F471" t="inlineStr"/>
@@ -19406,7 +19406,7 @@
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I471" t="inlineStr">
@@ -21479,7 +21479,7 @@
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>2025/06/17，2025/09/24</t>
+          <t>2025/06/17，2025/09/24，2026/9/2</t>
         </is>
       </c>
       <c r="F523" t="inlineStr"/>
@@ -21490,7 +21490,7 @@
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I523" t="inlineStr">
@@ -22043,7 +22043,7 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>2025/06/23，2025/10/23，2026/07/09</t>
+          <t>2025/06/23，2025/10/23，2026/07/09，2026/9/2</t>
         </is>
       </c>
       <c r="F537" t="inlineStr"/>
@@ -22054,7 +22054,7 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
@@ -22659,7 +22659,7 @@
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>2025/06/29，2025/09/19，2025/11/22，2026/07/22</t>
+          <t>2025/06/29，2025/09/19，2025/11/22，2026/07/22，2026/9/2</t>
         </is>
       </c>
       <c r="F552" t="inlineStr"/>
@@ -22670,7 +22670,7 @@
       </c>
       <c r="H552" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I552" t="inlineStr">
@@ -23175,7 +23175,7 @@
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/09，2026/01/09，2026/01/23，2026/02/12，2026/02/25，2026/03/09，2026/03/28，2026/05/10，2026/06/06</t>
+          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/09，2026/01/09，2026/01/23，2026/02/12，2026/02/25，2026/03/09，2026/03/28，2026/05/10，2026/06/06，2026/9/2</t>
         </is>
       </c>
       <c r="F565" t="inlineStr"/>
@@ -23186,7 +23186,7 @@
       </c>
       <c r="H565" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I565" t="inlineStr">
@@ -28219,7 +28219,7 @@
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>2025/10/13，2025/10/18，2026/03/15，2026/08/09</t>
+          <t>2025/10/13，2025/10/18，2026/03/15，2026/08/09，2026/9/2</t>
         </is>
       </c>
       <c r="F693" t="inlineStr"/>
@@ -28230,7 +28230,7 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I693" t="inlineStr">
@@ -29047,7 +29047,7 @@
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>2025/10/28，2025/11/01，2025/11/12，2025/12/19，2026/02/08，2026/02/10，2026/05/10，2026/08/16</t>
+          <t>2025/10/28，2025/11/01，2025/11/12，2025/12/19，2026/02/08，2026/02/10，2026/05/10，2026/08/16，2026/9/2</t>
         </is>
       </c>
       <c r="F714" t="inlineStr"/>
@@ -29058,7 +29058,7 @@
       </c>
       <c r="H714" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I714" t="inlineStr">
@@ -29471,7 +29471,7 @@
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/06，2025/12/12，2025/12/26，2026/01/05，2026/01/30，2026/02/09，2026/03/25，2026/05/01，2026/06/17，2026/07/25</t>
+          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/06，2025/12/12，2025/12/26，2026/01/05，2026/01/30，2026/02/09，2026/03/25，2026/05/01，2026/06/17，2026/07/25，2026/9/2</t>
         </is>
       </c>
       <c r="F725" t="inlineStr"/>
@@ -29482,7 +29482,7 @@
       </c>
       <c r="H725" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I725" t="inlineStr">
@@ -30047,7 +30047,7 @@
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/06，2025/12/13，2026/01/10，2026/01/24，2026/02/14，2026/03/14，2026/04/01，2026/04/08，2026/05/01，2026/05/06，2026/05/23，2026/06/20，2026/07/18，2026/08/07</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/06，2025/12/13，2026/01/10，2026/01/24，2026/02/14，2026/03/14，2026/04/01，2026/04/08，2026/05/01，2026/05/06，2026/05/23，2026/06/20，2026/07/18，2026/08/07，2026/9/2</t>
         </is>
       </c>
       <c r="F740" t="inlineStr"/>
@@ -30058,7 +30058,7 @@
       </c>
       <c r="H740" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I740" t="inlineStr">
@@ -30087,7 +30087,7 @@
       </c>
       <c r="E741" t="inlineStr">
         <is>
-          <t>2025/11/28</t>
+          <t>2025/11/28，2026/9/2</t>
         </is>
       </c>
       <c r="F741" t="inlineStr"/>
@@ -30098,10 +30098,14 @@
       </c>
       <c r="H741" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I741" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>BV1Q6to6JEEx</t>
+        </is>
+      </c>
       <c r="J741" t="inlineStr"/>
     </row>
     <row r="742">
@@ -30903,7 +30907,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08，2026/08/19</t>
+          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08，2026/08/19，2026/9/2</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -30914,7 +30918,7 @@
       </c>
       <c r="H762" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I762" t="inlineStr">
@@ -31939,7 +31943,7 @@
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>2026/02/08，2026/02/09，2026/02/12，2026/02/14，2026/02/19，2026/02/23，2026/02/24，2026/02/25，2026/03/01，2026/03/05，2026/03/12，2026/03/17，2026/03/19，2026/03/31，2026/04/20，2026/05/02，2026/05/21，2026/06/20，2026/07/16，2026/08/02</t>
+          <t>2026/02/08，2026/02/09，2026/02/12，2026/02/14，2026/02/19，2026/02/23，2026/02/24，2026/02/25，2026/03/01，2026/03/05，2026/03/12，2026/03/17，2026/03/19，2026/03/31，2026/04/20，2026/05/02，2026/05/21，2026/06/20，2026/07/16，2026/08/02，2026/9/2</t>
         </is>
       </c>
       <c r="F788" t="inlineStr"/>
@@ -31950,7 +31954,7 @@
       </c>
       <c r="H788" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I788" t="inlineStr">
@@ -34235,7 +34239,7 @@
       </c>
       <c r="E844" t="inlineStr">
         <is>
-          <t>2026/04/16，2026/04/29，2026/05/15，2026/05/25</t>
+          <t>2026/04/16，2026/04/29，2026/05/15，2026/05/25，2026/9/2</t>
         </is>
       </c>
       <c r="F844" t="inlineStr"/>
@@ -34246,7 +34250,7 @@
       </c>
       <c r="H844" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I844" t="inlineStr">
@@ -35666,7 +35670,11 @@
           <t>BV1Xx3P6cEfK</t>
         </is>
       </c>
-      <c r="J878" t="inlineStr"/>
+      <c r="J878" t="inlineStr">
+        <is>
+          <t>游戏</t>
+        </is>
+      </c>
     </row>
     <row r="879">
       <c r="A879" t="inlineStr">
@@ -35767,7 +35775,7 @@
       </c>
       <c r="E881" t="inlineStr">
         <is>
-          <t>2026/07/27，2026/07/30，2026/08/01，2026/08/03</t>
+          <t>2026/07/27，2026/07/30，2026/08/01，2026/08/03，2026/9/2</t>
         </is>
       </c>
       <c r="F881" t="inlineStr"/>
@@ -35778,7 +35786,7 @@
       </c>
       <c r="H881" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I881" t="inlineStr">
@@ -35786,7 +35794,11 @@
           <t>BV19x3P6cENj</t>
         </is>
       </c>
-      <c r="J881" t="inlineStr"/>
+      <c r="J881" t="inlineStr">
+        <is>
+          <t>动漫</t>
+        </is>
+      </c>
     </row>
     <row r="882">
       <c r="A882" t="inlineStr">
@@ -36411,7 +36423,7 @@
       </c>
       <c r="E897" t="inlineStr">
         <is>
-          <t>2026/08/23</t>
+          <t>2026/08/23，2026/9/2</t>
         </is>
       </c>
       <c r="F897" t="inlineStr"/>
@@ -36422,7 +36434,7 @@
       </c>
       <c r="H897" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I897" t="inlineStr">
@@ -36531,7 +36543,7 @@
       </c>
       <c r="E900" t="inlineStr">
         <is>
-          <t>2026/8/30</t>
+          <t>2026/8/30，2026/9/2</t>
         </is>
       </c>
       <c r="F900" t="inlineStr"/>
@@ -36542,7 +36554,7 @@
       </c>
       <c r="H900" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I900" t="inlineStr">
@@ -36711,6 +36723,46 @@
         </is>
       </c>
       <c r="J904" t="inlineStr"/>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>904</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>California King Bed</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr"/>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>Rihanna</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>2026/9/2</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr"/>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I905" t="inlineStr">
+        <is>
+          <t>BV15eto6sEMB</t>
+        </is>
+      </c>
+      <c r="J905" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Sep.4, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J905"/>
+  <dimension ref="A1:J906"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -663,7 +663,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/09，2025/12/11，2026/01/15，2026/02/12，2026/04/19，2026/08/08，2026/8/28</t>
+          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/09，2025/12/11，2026/01/15，2026/02/12，2026/04/19，2026/08/08，2026/8/28，2026/9/4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -674,7 +674,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/07，2025/12/17，2026/01/19，2026/01/29，2026/02/10，2026/02/12，2026/03/22，2026/04/18，2026/05/10，2026/06/06，2026/06/25，2026/07/17，2026/8/28</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/07，2025/12/17，2026/01/19，2026/01/29，2026/02/10，2026/02/12，2026/03/22，2026/04/18，2026/05/10，2026/06/06，2026/06/25，2026/07/17，2026/8/28，2026/9/4</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/01/09，2026/02/12，2026/03/09，2026/03/15，2026/05/01，2026/05/16，2026/05/23，2026/07/05，2026/07/28</t>
+          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/01/09，2026/02/12，2026/03/09，2026/03/15，2026/05/01，2026/05/16，2026/05/23，2026/07/05，2026/07/28，2026/9/4</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/02，2025/09/12，2025/09/17，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/05，2025/11/14，2025/11/21，2025/11/28，2025/12/08，2025/12/17，2026/01/10，2026/01/22，2026/02/10，2026/02/14，2026/02/14，2026/02/27，2026/03/28，2026/04/09，2026/04/14，2026/05/06，2026/05/23，2026/06/06，2026/06/25，2026/07/09，2026/07/16，2026/07/27，2026/08/21</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/02，2025/09/12，2025/09/17，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/05，2025/11/14，2025/11/21，2025/11/28，2025/12/08，2025/12/17，2026/01/10，2026/01/22，2026/02/10，2026/02/14，2026/02/14，2026/02/27，2026/03/28，2026/04/09，2026/04/14，2026/05/06，2026/05/23，2026/06/06，2026/06/25，2026/07/09，2026/07/16，2026/07/27，2026/08/21，2026/9/4</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/13，2025/05/01，2025/05/06，2025/05/24，2025/06/09，2025/06/24，2025/07/08，2025/08/16，2025/08/19，2025/09/08，2025/10/07，2025/10/28，2025/11/18，2025/12/11，2026/01/14，2026/02/04，2026/05/20，2026/07/09</t>
+          <t>2025/03/12，2025/04/13，2025/05/01，2025/05/06，2025/05/24，2025/06/09，2025/06/24，2025/07/08，2025/08/16，2025/08/19，2025/09/08，2025/10/07，2025/10/28，2025/11/18，2025/12/11，2026/01/14，2026/02/04，2026/05/20，2026/07/09，2026/9/4</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/02/10，2026/02/24，2026/03/18，2026/05/20，2026/06/19，2026/08/25，2026/8/30</t>
+          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/02/10，2026/02/24，2026/03/18，2026/05/20，2026/06/19，2026/08/25，2026/8/30，2026/9/4</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/20，2025/04/07，2025/05/06，2025/05/18，2025/05/30，2025/06/16，2025/06/27，2025/08/13，2025/08/24，2025/09/18，2025/09/19，2025/11/01，2026/02/14，2026/06/28，2026/07/22</t>
+          <t>2025/03/14，2025/03/20，2025/04/07，2025/05/06，2025/05/18，2025/05/30，2025/06/16，2025/06/27，2025/08/13，2025/08/24，2025/09/18，2025/09/19，2025/11/01，2026/02/14，2026/06/28，2026/07/22，2026/9/4</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -5167,7 +5167,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/05，2025/07/22，2026/02/27，2026/04/09，2026/04/14，2026/04/22，2026/06/10，2026/06/19</t>
+          <t>2025/03/14，2025/04/05，2025/07/22，2026/02/27，2026/04/09，2026/04/14，2026/04/22，2026/06/10，2026/06/19，2026/9/4</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/07，2026/03/06，2026/04/02，2026/06/20，2026/07/22</t>
+          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/07，2026/03/06，2026/04/02，2026/06/20，2026/07/22，2026/9/4</t>
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08，2026/08/23，2026/8/30</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08，2026/08/23，2026/8/30，2026/9/4</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/05/13，2025/06/10，2025/08/21，2025/11/19，2026/01/10，2026/04/09</t>
+          <t>2025/03/19，2025/04/07，2025/05/13，2025/06/10，2025/08/21，2025/11/19，2026/01/10，2026/04/09，2026/9/4</t>
         </is>
       </c>
       <c r="F144" t="inlineStr"/>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/08，2026/02/18，2026/03/06，2026/03/13，2026/03/14，2026/03/31，2026/05/01，2026/06/28，2026/07/17，2026/08/02，2026/08/21</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/08，2026/02/18，2026/03/06，2026/03/13，2026/03/14，2026/03/31，2026/05/01，2026/06/28，2026/07/17，2026/08/02，2026/08/21，2026/9/4</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -7975,7 +7975,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/03，2025/04/19，2025/05/26，2025/09/18，2025/10/17，2026/01/01，2026/05/10</t>
+          <t>2025/03/22，2025/04/03，2025/04/19，2025/05/26，2025/09/18，2025/10/17，2026/01/01，2026/05/10，2026/9/4</t>
         </is>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -7986,7 +7986,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -8055,7 +8055,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/01/29，2026/02/09，2026/03/25，2026/04/19，2026/05/23，2026/06/12，2026/07/22，2026/07/27</t>
+          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/01/29，2026/02/09，2026/03/25，2026/04/19，2026/05/23，2026/06/12，2026/07/22，2026/07/27，2026/9/4</t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -8066,7 +8066,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -8135,7 +8135,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/04/10，2025/05/01，2025/05/19，2025/06/08，2025/07/14，2025/09/11，2025/09/12，2025/10/31，2026/01/09，2026/07/05</t>
+          <t>2025/03/23，2025/04/10，2025/05/01，2025/05/19，2025/06/08，2025/07/14，2025/09/11，2025/09/12，2025/10/31，2026/01/09，2026/07/05，2026/9/4</t>
         </is>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/07，2026/01/17，2026/02/14，2026/04/09，2026/05/20，2026/06/19，2026/06/28，2026/07/31</t>
+          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/07，2026/01/17，2026/02/14，2026/04/09，2026/05/20，2026/06/19，2026/06/28，2026/07/31，2026/9/4</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -8306,7 +8306,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/09/19，2025/10/10，2025/11/09</t>
+          <t>2025/03/25，2025/09/19，2025/10/10，2025/11/09，2026/9/4</t>
         </is>
       </c>
       <c r="F206" t="inlineStr"/>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -9983,7 +9983,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/07，2025/11/13，2025/12/02，2026/01/14，2026/01/24，2026/03/07，2026/03/15，2026/04/24，2026/06/06，2026/06/23，2026/08/05，2026/08/05，2026/08/19</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/07，2025/11/13，2025/12/02，2026/01/14，2026/01/24，2026/03/07，2026/03/15，2026/04/24，2026/06/06，2026/06/23，2026/08/05，2026/08/05，2026/08/19，2026/9/4</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
@@ -9994,7 +9994,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -10431,7 +10431,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/04，2025/04/26，2025/05/06，2025/05/18，2025/06/10，2025/07/03，2025/07/10，2025/07/24，2025/08/16，2025/09/18，2025/10/03，2025/11/01，2026/02/14，2026/04/09，2026/07/09</t>
+          <t>2025/03/30，2025/04/04，2025/04/26，2025/05/06，2025/05/18，2025/06/10，2025/07/03，2025/07/10，2025/07/24，2025/08/16，2025/09/18，2025/10/03，2025/11/01，2026/02/14，2026/04/09，2026/07/09，2026/9/4</t>
         </is>
       </c>
       <c r="F247" t="inlineStr"/>
@@ -10442,7 +10442,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -10525,7 +10525,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I249" t="inlineStr"/>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>BV12Wth6NEcs</t>
+        </is>
+      </c>
       <c r="J249" t="inlineStr"/>
     </row>
     <row r="250">
@@ -10547,7 +10551,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/19，2025/06/23，2025/07/08，2025/09/21，2025/10/23，2025/11/14，2025/12/17，2026/02/07，2026/08/18</t>
+          <t>2025/03/30，2025/04/19，2025/06/23，2025/07/08，2025/09/21，2025/10/23，2025/11/14，2025/12/17，2026/02/07，2026/08/18，2026/9/4</t>
         </is>
       </c>
       <c r="F250" t="inlineStr"/>
@@ -10558,7 +10562,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -11427,7 +11431,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/03，2025/04/08，2025/05/26，2025/07/18，2025/08/16，2025/09/30，2025/11/26，2026/01/23，2026/02/18，2026/03/12，2026/06/10</t>
+          <t>2025/04/02，2025/04/03，2025/04/08，2025/05/26，2025/07/18，2025/08/16，2025/09/30，2025/11/26，2026/01/23，2026/02/18，2026/03/12，2026/06/10，2026/9/4</t>
         </is>
       </c>
       <c r="F272" t="inlineStr"/>
@@ -11438,7 +11442,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -11791,7 +11795,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/24，2025/09/12，2026/01/10，2026/06/03</t>
+          <t>2025/04/03，2025/04/24，2025/09/12，2026/01/10，2026/06/03，2026/9/4</t>
         </is>
       </c>
       <c r="F281" t="inlineStr"/>
@@ -11802,7 +11806,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -12667,7 +12671,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/05/09，2025/06/19，2025/07/22，2026/03/09，2026/8/30</t>
+          <t>2025/04/07，2025/05/09，2025/06/19，2025/07/22，2026/03/09，2026/8/30，2026/9/4</t>
         </is>
       </c>
       <c r="F303" t="inlineStr"/>
@@ -12678,7 +12682,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -13859,7 +13863,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>2025/04/12，2025/07/14，2025/09/24，2025/09/28，2025/11/09，2026/04/24</t>
+          <t>2025/04/12，2025/07/14，2025/09/24，2025/09/28，2025/11/09，2026/04/24，2026/9/4</t>
         </is>
       </c>
       <c r="F333" t="inlineStr"/>
@@ -13870,7 +13874,7 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I333" t="inlineStr">
@@ -13939,7 +13943,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>2025/04/12，2026/8/30</t>
+          <t>2025/04/12，2026/8/30，2026/9/4</t>
         </is>
       </c>
       <c r="F335" t="inlineStr"/>
@@ -13950,10 +13954,14 @@
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I335" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>BV1xbtW6UEw8</t>
+        </is>
+      </c>
       <c r="J335" t="inlineStr"/>
     </row>
     <row r="336">
@@ -13975,7 +13983,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/01/09，2026/02/08，2026/03/01，2026/03/09，2026/03/24，2026/04/17，2026/05/01，2026/05/21，2026/06/10，2026/06/25，2026/07/27，2026/08/23，2026/8/28</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/01/09，2026/02/08，2026/03/01，2026/03/09，2026/03/24，2026/04/17，2026/05/01，2026/05/21，2026/06/10，2026/06/25，2026/07/27，2026/08/23，2026/8/28，2026/9/4</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13986,7 +13994,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -14151,7 +14159,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/07/13，2025/07/18，2025/08/02，2025/09/04，2025/09/12，2025/10/17，2025/11/28，2026/01/22，2026/02/23</t>
+          <t>2025/04/13，2025/07/13，2025/07/18，2025/08/02，2025/09/04，2025/09/12，2025/10/17，2025/11/28，2026/01/22，2026/02/23，2026/9/4</t>
         </is>
       </c>
       <c r="F340" t="inlineStr"/>
@@ -14162,7 +14170,7 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
@@ -15611,7 +15619,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>2025/04/21，2025/05/23，2025/06/29，2025/07/26，2025/09/28，2025/12/02，2025/12/17，2026/05/06，2026/9/2</t>
+          <t>2025/04/21，2025/05/23，2025/06/29，2025/07/26，2025/09/28，2025/12/02，2025/12/17，2026/05/06，2026/9/2，2026/9/4</t>
         </is>
       </c>
       <c r="F376" t="inlineStr"/>
@@ -15622,7 +15630,7 @@
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">
@@ -16827,7 +16835,7 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/11/18，2026/02/14，2026/04/09，2026/05/16，2026/06/14，2026/08/02</t>
+          <t>2025/04/28，2025/11/18，2026/02/14，2026/04/09，2026/05/16，2026/06/14，2026/08/02，2026/9/4</t>
         </is>
       </c>
       <c r="F407" t="inlineStr"/>
@@ -16838,7 +16846,7 @@
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I407" t="inlineStr">
@@ -17543,7 +17551,7 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/04/20，2026/05/23，2026/8/28</t>
+          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/04/20，2026/05/23，2026/8/28，2026/9/4</t>
         </is>
       </c>
       <c r="F425" t="inlineStr"/>
@@ -17554,7 +17562,7 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
@@ -18419,7 +18427,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/01/02，2026/03/17，2026/04/29，2026/05/10，2026/07/09，2026/07/31，2026/08/11，2026/08/25</t>
+          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/01/02，2026/03/17，2026/04/29，2026/05/10，2026/07/09，2026/07/31，2026/08/11，2026/08/25，2026/9/4</t>
         </is>
       </c>
       <c r="F447" t="inlineStr"/>
@@ -18430,7 +18438,7 @@
       </c>
       <c r="H447" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I447" t="inlineStr">
@@ -22699,7 +22707,7 @@
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/08/16，2026/8/30</t>
+          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/08/16，2026/8/30，2026/9/4</t>
         </is>
       </c>
       <c r="F553" t="inlineStr"/>
@@ -22710,7 +22718,7 @@
       </c>
       <c r="H553" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I553" t="inlineStr">
@@ -25115,7 +25123,7 @@
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/01，2025/11/26，2025/12/30，2026/01/10，2026/02/18，2026/04/10，2026/04/23，2026/05/23，2026/06/18，2026/07/13，2026/08/07</t>
+          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/01，2025/11/26，2025/12/30，2026/01/10，2026/02/18，2026/04/10，2026/04/23，2026/05/23，2026/06/18，2026/07/13，2026/08/07，2026/9/4</t>
         </is>
       </c>
       <c r="F614" t="inlineStr"/>
@@ -25126,7 +25134,7 @@
       </c>
       <c r="H614" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I614" t="inlineStr">
@@ -26883,7 +26891,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31，2026/08/23</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31，2026/08/23，2026/9/4</t>
         </is>
       </c>
       <c r="F659" t="inlineStr"/>
@@ -26894,7 +26902,7 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
@@ -27499,7 +27507,7 @@
       </c>
       <c r="E675" t="inlineStr">
         <is>
-          <t>2025/09/28</t>
+          <t>2025/09/28，2026/9/4</t>
         </is>
       </c>
       <c r="F675" t="inlineStr"/>
@@ -27510,10 +27518,14 @@
       </c>
       <c r="H675" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I675" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>BV1Datr6zEvQ</t>
+        </is>
+      </c>
       <c r="J675" t="inlineStr"/>
     </row>
     <row r="676">
@@ -28579,7 +28591,7 @@
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>2025/10/23，2026/08/16，2026/08/21</t>
+          <t>2025/10/23，2026/08/16，2026/08/21，2026/9/4</t>
         </is>
       </c>
       <c r="F702" t="inlineStr"/>
@@ -28590,7 +28602,7 @@
       </c>
       <c r="H702" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I702" t="inlineStr">
@@ -30831,7 +30843,7 @@
       </c>
       <c r="E760" t="inlineStr">
         <is>
-          <t>2025/12/19</t>
+          <t>2025/12/19，2026/9/4</t>
         </is>
       </c>
       <c r="F760" t="inlineStr"/>
@@ -30842,10 +30854,14 @@
       </c>
       <c r="H760" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I760" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>BV1getr6uEAQ</t>
+        </is>
+      </c>
       <c r="J760" t="inlineStr"/>
     </row>
     <row r="761">
@@ -31623,7 +31639,7 @@
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>2026/01/25，2026/01/30，2026/02/02，2026/02/08，2026/02/19，2026/02/23，2026/02/25，2026/03/12，2026/03/28，2026/04/12，2026/04/20，2026/06/26，2026/07/22</t>
+          <t>2026/01/25，2026/01/30，2026/02/02，2026/02/08，2026/02/19，2026/02/23，2026/02/25，2026/03/12，2026/03/28，2026/04/12，2026/04/20，2026/06/26，2026/07/22，2026/9/4</t>
         </is>
       </c>
       <c r="F780" t="inlineStr"/>
@@ -31634,7 +31650,7 @@
       </c>
       <c r="H780" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I780" t="inlineStr">
@@ -34919,7 +34935,7 @@
       </c>
       <c r="E860" t="inlineStr">
         <is>
-          <t>2026/05/25，2026/05/26，2026/06/15，2026/08/02</t>
+          <t>2026/05/25，2026/05/26，2026/06/15，2026/08/02，2026/9/4</t>
         </is>
       </c>
       <c r="F860" t="inlineStr"/>
@@ -34930,7 +34946,7 @@
       </c>
       <c r="H860" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I860" t="inlineStr">
@@ -35119,7 +35135,7 @@
       </c>
       <c r="E865" t="inlineStr">
         <is>
-          <t>2026/06/14，2026/07/10，2026/07/15，2026/07/27</t>
+          <t>2026/06/14，2026/07/10，2026/07/15，2026/07/27，2026/9/4</t>
         </is>
       </c>
       <c r="F865" t="inlineStr"/>
@@ -35130,7 +35146,7 @@
       </c>
       <c r="H865" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I865" t="inlineStr">
@@ -36763,6 +36779,46 @@
         </is>
       </c>
       <c r="J905" t="inlineStr"/>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>905</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>willow</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr"/>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>2026/9/4</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr"/>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>BV1Setr6MEBW</t>
+        </is>
+      </c>
+      <c r="J906" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Sep.13, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J906"/>
+  <dimension ref="A1:J909"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,7 +527,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/02，2025/09/07，2025/09/17，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/09，2025/11/14，2025/12/24，2025/12/26，2026/01/16，2026/01/24，2026/01/28，2026/01/30，2026/02/10，2026/02/14，2026/03/09，2026/03/27，2026/04/01，2026/04/14，2026/04/24，2026/06/12，2026/07/22，2026/08/11</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/02，2025/09/07，2025/09/17，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/09，2025/11/14，2025/12/24，2025/12/26，2026/01/16，2026/01/24，2026/01/28，2026/01/30，2026/02/10，2026/02/14，2026/03/09，2026/03/27，2026/04/01，2026/04/14，2026/04/24，2026/06/12，2026/07/22，2026/08/11，2026/09/12</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -538,7 +538,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/09，2025/12/11，2026/01/15，2026/02/12，2026/04/19，2026/08/08，2026/8/28，2026/9/4</t>
+          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/09，2025/12/11，2026/01/15，2026/02/12，2026/04/19，2026/08/08，2026/08/28，2026/09/04，2026/09/13</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -674,7 +674,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/01，2025/11/17，2025/12/02，2025/12/31，2026/02/02，2026/02/14，2026/03/06，2026/04/01，2026/04/20，2026/05/15，2026/06/10，2026/07/22，2026/08/09，2026/9/2</t>
+          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/01，2025/11/17，2025/12/02，2025/12/31，2026/02/02，2026/02/14，2026/03/06，2026/04/01，2026/04/20，2026/05/15，2026/06/10，2026/07/22，2026/08/09，2026/09/02</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -747,7 +747,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/09，2025/11/19，2025/12/16，2026/01/16，2026/01/28，2026/02/07，2026/02/10，2026/03/17，2026/04/19，2026/05/23，2026/06/19，2026/07/22，2026/08/08，2026/9/2</t>
+          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/09，2025/11/19，2025/12/16，2026/01/16，2026/01/28，2026/02/07，2026/02/10，2026/03/17，2026/04/19，2026/05/23，2026/06/19，2026/07/22，2026/08/08，2026/09/02</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -787,7 +787,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/04/20，2025/06/16，2025/06/27，2025/07/31，2025/10/05，2025/11/07，2025/12/04，2026/01/28，2026/04/29，2026/06/25</t>
+          <t>2025/03/03，2025/04/20，2025/06/16，2025/06/27，2025/07/31，2025/10/05，2025/11/07，2025/12/04，2026/01/28，2026/04/29，2026/06/25，2026/09/12</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -798,7 +798,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/07，2025/12/31，2026/01/14，2026/01/19，2026/03/29，2026/04/12，2026/04/27，2026/05/01，2026/06/03，2026/06/18，2026/06/25，2026/07/31</t>
+          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/07，2025/12/31，2026/01/14，2026/01/19，2026/03/29，2026/04/12，2026/04/27，2026/05/01，2026/06/03，2026/06/18，2026/06/25，2026/07/31，2026/09/11，2026/09/13</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -918,7 +918,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>39</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/04，2026/01/24，2026/01/24，2026/02/19，2026/02/25，2026/03/13，2026/04/08，2026/06/10，2026/07/27，2026/08/18</t>
+          <t>2025/03/04，2025/03/12，2025/03/17，2025/03/28，2025/04/07，2025/04/19，2025/04/26，2025/05/06，2025/05/16，2025/05/22，2025/05/30，2025/06/21，2025/07/06，2025/08/22，2025/09/06，2025/09/21，2025/10/23，2025/11/10，2025/11/13，2025/12/04，2026/01/24，2026/01/24，2026/02/19，2026/02/25，2026/03/13，2026/04/08，2026/06/10，2026/07/27，2026/08/18，2026/09/06</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/07，2025/12/17，2026/01/19，2026/01/29，2026/02/10，2026/02/12，2026/03/22，2026/04/18，2026/05/10，2026/06/06，2026/06/25，2026/07/17，2026/8/28，2026/9/4</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/07，2025/12/17，2026/01/19，2026/01/29，2026/02/10，2026/02/12，2026/03/22，2026/04/18，2026/05/10，2026/06/06，2026/06/25，2026/07/17，2026/08/28，2026/09/04，2026/09/06</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/01/10，2026/01/24，2026/04/09，2026/05/21，2026/07/17</t>
+          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/01/10，2026/01/24，2026/04/09，2026/05/21，2026/07/17，2026/09/06</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/03，2025/04/17，2025/05/22，2025/06/03，2025/07/24，2025/08/12，2025/09/03，2025/10/10，2025/11/09，2025/11/10，2026/03/13，2026/06/03</t>
+          <t>2025/03/04，2025/04/03，2025/04/17，2025/05/22，2025/06/03，2025/07/24，2025/08/12，2025/09/03，2025/10/10，2025/11/09，2025/11/10，2026/03/13，2026/06/03，2026/09/08</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/01/09，2026/02/12，2026/03/09，2026/03/15，2026/05/01，2026/05/16，2026/05/23，2026/07/05，2026/07/28，2026/9/4</t>
+          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/01/09，2026/02/12，2026/03/09，2026/03/15，2026/05/01，2026/05/16，2026/05/23，2026/07/05，2026/07/28，2026/08/30，2026/09/04</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/29，2025/05/20，2025/07/13，2025/07/25，2025/07/31，2025/10/09，2025/12/02，2026/01/09，2026/03/21，2026/07/19</t>
+          <t>2025/03/04，2025/04/29，2025/05/20，2025/07/13，2025/07/25，2025/07/31，2025/10/09，2025/12/02，2026/01/09，2026/03/21，2026/07/19，2026/09/13</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/09，2025/12/16，2026/02/14，2026/03/07，2026/03/17，2026/03/21，2026/05/01，2026/07/04，2026/07/26，2026/8/28</t>
+          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/09，2025/12/16，2026/02/14，2026/03/07，2026/03/17，2026/03/21，2026/05/01，2026/07/04，2026/07/26，2026/08/28</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/09，2025/11/12，2025/11/27，2025/12/04，2025/12/28，2026/01/22，2026/02/02，2026/02/23，2026/03/25，2026/04/16，2026/05/06，2026/05/21，2026/07/10，2026/07/15，2026/08/21，2026/8/28，2026/8/28</t>
+          <t>2025/03/04，2025/05/01，2025/05/08，2025/05/26，2025/06/05，2025/06/23，2025/06/26，2025/07/03，2025/07/20，2025/07/26，2025/08/03，2025/08/12，2025/08/30，2025/09/21，2025/09/29，2025/11/09，2025/11/12，2025/11/27，2025/12/04，2025/12/28，2026/01/22，2026/02/02，2026/02/23，2026/03/25，2026/04/16，2026/05/06，2026/05/21，2026/07/10，2026/07/15，2026/08/21，2026/08/28，2026/08/28</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/01，2025/11/09，2025/11/21，2025/12/08，2026/01/15，2026/01/24，2026/03/04，2026/03/14，2026/05/06，2026/05/16，2026/05/20，2026/06/12，2026/07/16，2026/07/26，2026/07/31，2026/8/28</t>
+          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/01，2025/11/09，2025/11/21，2025/12/08，2026/01/15，2026/01/24，2026/03/04，2026/03/14，2026/05/06，2026/05/16，2026/05/20，2026/06/12，2026/07/16，2026/07/26，2026/07/31，2026/08/28，2026/09/06</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/02，2025/09/12，2025/09/17，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/05，2025/11/14，2025/11/21，2025/11/28，2025/12/08，2025/12/17，2026/01/10，2026/01/22，2026/02/10，2026/02/14，2026/02/14，2026/02/27，2026/03/28，2026/04/09，2026/04/14，2026/05/06，2026/05/23，2026/06/06，2026/06/25，2026/07/09，2026/07/16，2026/07/27，2026/08/21，2026/9/4</t>
+          <t>2025/03/04，2025/03/25，2025/04/29，2025/05/09，2025/05/13，2025/05/22，2025/05/26，2025/05/30，2025/06/08，2025/06/13，2025/06/20，2025/07/05，2025/07/14，2025/07/20，2025/08/01，2025/08/30，2025/09/02，2025/09/12，2025/09/17，2025/09/22，2025/09/24，2025/10/03，2025/10/12，2025/11/05，2025/11/14，2025/11/21，2025/11/28，2025/12/08，2025/12/17，2026/01/10，2026/01/22，2026/02/10，2026/02/14，2026/02/14，2026/02/27，2026/03/28，2026/04/09，2026/04/14，2026/05/06，2026/05/23，2026/06/06，2026/06/25，2026/07/09，2026/07/16，2026/07/27，2026/08/21，2026/09/04，2026/09/06</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/07，2025/12/24，2026/01/01，2026/01/16，2026/03/14，2026/05/01，2026/05/20，2026/08/01，2026/9/2</t>
+          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/07，2025/12/24，2026/01/01，2026/01/16，2026/03/14，2026/05/01，2026/05/20，2026/08/01，2026/09/02</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/03/15，2026/06/23，2026/8/30</t>
+          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/03/15，2026/06/23，2026/08/30，2026/08/30</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/18，2025/05/03，2025/05/08，2025/06/05，2025/06/19，2025/07/15，2025/09/08，2025/10/07，2025/10/17，2025/10/23，2025/12/24，2026/9/2</t>
+          <t>2025/03/04，2025/04/18，2025/05/03，2025/05/08，2025/06/05，2025/06/19，2025/07/15，2025/09/08，2025/10/07，2025/10/17，2025/10/23，2025/12/24，2026/09/02，2026/09/12</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2002,7 +2002,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/18，2025/07/26，2025/08/12，2025/11/28，2026/02/19，2026/03/04，2026/07/17，2026/9/2</t>
+          <t>2025/03/04，2025/05/18，2025/07/26，2025/08/12，2025/11/28，2026/02/19，2026/03/04，2026/07/17，2026/09/02</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/01/09，2026/01/28，2026/02/25，2026/03/12，2026/03/21，2026/04/26，2026/05/10，2026/06/26，2026/9/2</t>
+          <t>2025/03/04，2025/03/17，2025/03/21，2025/04/04，2025/04/14，2025/04/19，2025/04/25，2025/05/08，2025/05/09，2025/05/19，2025/05/27，2025/05/29，2025/06/08，2025/06/09，2025/07/11，2025/07/14，2025/08/04，2025/08/08，2025/08/12，2025/09/18，2025/10/03，2025/10/10，2025/10/23，2025/11/13，2025/11/28，2025/12/13，2025/12/28，2026/01/09，2026/01/28，2026/02/25，2026/03/12，2026/03/21，2026/04/26，2026/05/10，2026/06/26，2026/09/02</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/21，2025/04/19，2025/05/11，2025/06/03，2026/01/19，2026/01/25，2026/02/25，2026/04/01，2026/07/27</t>
+          <t>2025/03/06，2025/03/21，2025/04/19，2025/05/11，2025/06/03，2026/01/19，2026/01/25，2026/02/25，2026/04/01，2026/07/27，2026/09/08</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/03，2025/04/14，2025/05/05，2025/05/15，2025/05/29，2025/06/20，2025/06/27，2025/08/07，2025/08/24，2025/09/17，2025/10/16，2025/11/10，2025/12/09，2025/12/17，2026/01/21，2026/02/12，2026/02/25，2026/07/27</t>
+          <t>2025/03/06，2025/04/03，2025/04/14，2025/05/05，2025/05/15，2025/05/29，2025/06/20，2025/06/27，2025/08/07，2025/08/24，2025/09/17，2025/10/16，2025/11/10，2025/12/09，2025/12/17，2026/01/21，2026/02/12，2026/02/25，2026/07/27，2026/09/08</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/07，2025/11/09，2025/12/02，2026/01/21，2026/03/05，2026/04/16，2026/06/23，2026/07/05，2026/08/05，2026/08/05，2026/08/19</t>
+          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/07，2025/11/09，2025/12/02，2026/01/21，2026/03/05，2026/04/16，2026/06/23，2026/07/05，2026/08/05，2026/08/05，2026/08/19，2026/09/05</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2254,7 +2254,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/17，2025/05/18，2025/05/30，2025/06/06，2025/06/21，2025/06/27，2025/07/24，2025/08/24，2025/09/10，2025/09/30，2025/10/23，2025/11/10，2026/01/15，2026/02/14，2026/03/22，2026/05/20</t>
+          <t>2025/03/06，2025/04/17，2025/05/18，2025/05/30，2025/06/06，2025/06/21，2025/06/27，2025/07/24，2025/08/24，2025/09/10，2025/09/30，2025/10/23，2025/11/10，2026/01/15，2026/02/14，2026/03/22，2026/05/20，2026/09/13</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/27，2025/04/07，2025/04/12，2025/04/22，2025/04/26，2025/05/05，2025/05/19，2025/06/03，2025/06/09，2025/07/18，2025/07/22，2025/09/10，2025/09/19，2025/10/16，2025/12/24，2026/06/20</t>
+          <t>2025/03/07，2025/03/27，2025/04/07，2025/04/12，2025/04/22，2025/04/26，2025/05/05，2025/05/19，2025/06/03，2025/06/09，2025/07/18，2025/07/22，2025/09/10，2025/09/19，2025/10/16，2025/12/24，2026/06/20，2026/08/27</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/05/04，2025/05/18，2025/06/09，2025/08/04，2025/08/16，2025/09/18，2025/10/17，2025/11/21，2025/11/28，2026/05/10，2026/8/27</t>
+          <t>2025/03/07，2025/03/28，2025/05/04，2025/05/18，2025/06/09，2025/08/04，2025/08/16，2025/09/18，2025/10/17，2025/11/21，2025/11/28，2026/05/10，2026/08/27</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/07，2025/12/16，2025/12/28，2026/01/10，2026/01/15，2026/02/19，2026/03/07，2026/03/17，2026/03/21，2026/05/06，2026/07/05，2026/07/20，2026/8/30</t>
+          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/07，2025/12/16，2025/12/28，2026/01/10，2026/01/15，2026/02/19，2026/03/07，2026/03/17，2026/03/21，2026/05/06，2026/07/05，2026/07/20，2026/08/30</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/07，2025/11/19，2025/11/26，2025/12/30，2026/01/28，2026/02/14，2026/03/13，2026/04/10，2026/05/23，2026/06/18，2026/06/29，2026/07/25，2026/08/25</t>
+          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/07，2025/11/19，2025/11/26，2025/12/30，2026/01/28，2026/02/14，2026/03/13，2026/04/10，2026/05/23，2026/06/18，2026/06/29，2026/07/25，2026/08/25，2026/09/06</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/01，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/01/09，2026/01/22，2026/02/14，2026/03/22，2026/04/19，2026/05/01，2026/05/23，2026/06/25，2026/08/07</t>
+          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/01，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/01/09，2026/01/22，2026/02/14，2026/03/22，2026/04/19，2026/05/01，2026/05/23，2026/06/25，2026/08/07，2026/09/11</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/01，2025/11/09，2025/12/04，2025/12/16，2025/12/31，2026/01/09，2026/01/15，2026/01/21，2026/01/23，2026/01/29，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/02/24，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/05，2026/03/07，2026/03/08，2026/03/09，2026/03/12，2026/03/13，2026/03/14，2026/03/15，2026/03/17，2026/03/18，2026/03/19，2026/03/22，2026/03/24，2026/03/27，2026/03/28，2026/03/31，2026/04/08，2026/04/14，2026/04/18，2026/04/25，2026/05/01，2026/05/15，2026/05/25，2026/06/12，2026/06/23，2026/06/26，2026/07/04，2026/07/20，2026/07/30，2026/08/09，2026/8/28，2026/9/2</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/01，2025/11/09，2025/12/04，2025/12/16，2025/12/31，2026/01/09，2026/01/15，2026/01/21，2026/01/23，2026/01/29，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/02/24，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/05，2026/03/07，2026/03/08，2026/03/09，2026/03/12，2026/03/13，2026/03/14，2026/03/15，2026/03/17，2026/03/18，2026/03/19，2026/03/22，2026/03/24，2026/03/27，2026/03/28，2026/03/31，2026/04/08，2026/04/14，2026/04/18，2026/04/25，2026/05/01，2026/05/15，2026/05/25，2026/06/12，2026/06/23，2026/06/26，2026/07/04，2026/07/20，2026/07/30，2026/08/09，2026/08/28，2026/09/02，2026/09/11</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>75</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/14，2025/05/05，2025/05/19，2025/05/23，2025/06/13，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/12/02，2025/12/26，2026/05/04，2026/06/28</t>
+          <t>2025/03/07，2025/04/14，2025/05/05，2025/05/19，2025/05/23，2025/06/13，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/12/02，2025/12/26，2026/05/04，2026/06/28，2026/09/06</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
@@ -3006,7 +3006,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/05/01，2025/05/09，2025/05/26，2025/06/17，2025/06/20，2025/07/13，2025/09/12，2025/09/26，2025/10/11，2025/12/08，2026/01/12，2026/01/30，2026/02/07，2026/04/18，2026/05/23，2026/07/18，2026/08/21，2026/8/28</t>
+          <t>2025/03/07，2025/05/01，2025/05/09，2025/05/26，2025/06/17，2025/06/20，2025/07/13，2025/09/12，2025/09/26，2025/10/11，2025/12/08，2026/01/12，2026/01/30，2026/02/07，2026/04/18，2026/05/23，2026/07/18，2026/08/21，2026/08/28</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2025/03/08，2025/04/06，2025/05/15，2025/05/26，2025/07/22，2025/09/17，2025/12/30，2026/02/14，2026/05/04，2026/8/30</t>
+          <t>2025/03/08，2025/04/06，2025/05/15，2025/05/26，2025/07/22，2025/09/17，2025/12/30，2026/02/14，2026/05/04，2026/08/30</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/04/09，2026/05/10，2026/06/12，2026/07/27，2026/8/28</t>
+          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/04/09，2026/05/10，2026/06/12，2026/07/27，2026/08/28</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3199,7 +3199,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/02/02，2026/02/12，2026/04/14，2026/04/22，2026/06/10，2026/8/28</t>
+          <t>2025/03/09，2025/03/24，2025/04/06，2025/04/21，2025/04/28，2025/05/08，2025/05/20，2025/06/08，2025/07/08，2025/07/28，2025/09/24，2025/09/30，2025/11/18，2025/12/24，2026/02/02，2026/02/12，2026/04/14，2026/04/22，2026/06/10，2026/08/28，2026/09/08</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/04，2025/04/11，2025/05/20，2025/06/16，2025/06/24，2025/08/29，2025/09/12，2025/10/12，2026/01/09，2026/05/20</t>
+          <t>2025/03/09，2025/04/04，2025/04/11，2025/05/20，2025/06/16，2025/06/24，2025/08/29，2025/09/12，2025/10/12，2026/01/09，2026/05/20，2026/09/13</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/01，2026/01/16，2026/02/02，2026/02/23，2026/03/08，2026/03/19，2026/03/21，2026/04/16，2026/05/10，2026/06/14，2026/07/25，2026/08/07，2026/08/25</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/01，2026/01/16，2026/02/02，2026/02/23，2026/03/08，2026/03/19，2026/03/21，2026/04/16，2026/05/10，2026/06/14，2026/07/25，2026/08/07，2026/08/25，2026/09/08</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/30，2025/04/10，2025/04/20，2025/05/04，2025/05/13，2025/05/22，2025/06/05，2025/06/07，2025/08/29，2025/09/07，2025/09/11，2025/10/10，2025/11/09，2026/01/01，2026/06/20，2026/07/30，2026/9/2</t>
+          <t>2025/03/09，2025/03/30，2025/04/10，2025/04/20，2025/05/04，2025/05/13，2025/05/22，2025/06/05，2025/06/07，2025/08/29，2025/09/07，2025/09/11，2025/10/10，2025/11/09，2026/01/01，2026/06/20，2026/07/30，2026/09/02，2026/09/13</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/05/12，2025/06/12，2025/07/21，2025/12/11，2026/01/15，2026/03/01，2026/05/05，2026/07/16，2026/9/2</t>
+          <t>2025/03/09，2025/05/12，2025/06/12，2025/07/21，2025/12/11，2026/01/15，2026/03/01，2026/05/05，2026/07/16，2026/09/02</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/03/27，2026/04/01，2026/06/23，2026/07/31，2026/9/2</t>
+          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/03/27，2026/04/01，2026/06/23，2026/07/31，2026/09/02</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/06/05，2025/07/05，2025/08/22，2026/04/26</t>
+          <t>2025/03/10，2025/06/05，2025/07/05，2025/08/22，2026/04/26，2026/09/04</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/05/05，2025/05/13，2025/05/24，2025/08/12，2025/08/30，2025/11/26，2026/08/21，2026/8/30</t>
+          <t>2025/03/10，2025/05/05，2025/05/13，2025/05/24，2025/08/12，2025/08/30，2025/11/26，2026/08/21，2026/08/30</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/01/01，2026/02/14，2026/05/06，2026/05/23，2026/07/07，2026/08/02，2026/9/2</t>
+          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/01/01，2026/02/14，2026/05/06，2026/05/23，2026/07/07，2026/08/02，2026/09/02</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/03，2025/12/02，2025/12/04，2025/12/12，2026/01/05，2026/01/14，2026/02/19，2026/03/04，2026/03/31，2026/04/12，2026/04/29，2026/05/15，2026/06/12，2026/06/23，2026/07/09，2026/08/11，2026/9/2</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/03，2025/12/02，2025/12/04，2025/12/12，2026/01/05，2026/01/14，2026/02/19，2026/03/04，2026/03/31，2026/04/12，2026/04/29，2026/05/15，2026/06/12，2026/06/23，2026/07/09，2026/08/11，2026/09/02</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3955,7 +3955,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/13，2025/05/01，2025/05/06，2025/05/24，2025/06/09，2025/06/24，2025/07/08，2025/08/16，2025/08/19，2025/09/08，2025/10/07，2025/10/28，2025/11/18，2025/12/11，2026/01/14，2026/02/04，2026/05/20，2026/07/09，2026/9/4</t>
+          <t>2025/03/12，2025/04/13，2025/05/01，2025/05/06，2025/05/24，2025/06/09，2025/06/24，2025/07/08，2025/08/16，2025/08/19，2025/09/08，2025/10/07，2025/10/28，2025/11/18，2025/12/11，2026/01/14，2026/02/04，2026/05/20，2026/07/09，2026/09/04，2026/09/06</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/03，2025/05/26，2025/06/01，2025/06/06，2025/09/08，2025/09/12，2026/04/09，2026/06/20，2026/07/22</t>
+          <t>2025/03/13，2025/04/03，2025/05/26，2025/06/01，2025/06/06，2025/09/08，2025/09/12，2026/04/09，2026/06/20，2026/07/22，2026/09/13</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/30，2025/04/17，2025/04/21，2025/05/05，2025/05/13，2025/05/20，2025/06/06，2025/06/20，2025/06/27，2025/07/05，2025/07/31，2025/08/24，2025/08/29，2025/09/20，2025/09/30，2025/10/22，2025/11/26，2026/01/15，2026/02/14，2026/04/08，2026/05/20</t>
+          <t>2025/03/13，2025/03/30，2025/04/17，2025/04/21，2025/05/05，2025/05/13，2025/05/20，2025/06/06，2025/06/20，2025/06/27，2025/07/05，2025/07/31，2025/08/24，2025/08/29，2025/09/20，2025/09/30，2025/10/22，2025/11/26，2026/01/15，2026/02/14，2026/04/08，2026/05/20，2026/09/13</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/21，2025/05/15，2025/07/28，2025/09/10，2026/01/14，2026/06/28</t>
+          <t>2025/03/13，2025/04/21，2025/05/15，2025/07/28，2025/09/10，2026/01/14，2026/06/28，2026/09/13</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/17，2025/05/04，2025/05/13，2025/07/22，2025/09/05，2025/09/28，2026/06/03，2026/8/30</t>
+          <t>2025/03/13，2025/04/17，2025/05/04，2025/05/13，2025/07/22，2025/09/05，2025/09/28，2026/06/03，2026/08/30</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4275,7 +4275,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/09，2026/01/23，2026/02/18，2026/04/09，2026/06/15，2026/07/22，2026/8/28</t>
+          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/09，2026/01/23，2026/02/18，2026/04/09，2026/06/15，2026/07/22，2026/08/28</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/02/10，2026/02/24，2026/03/18，2026/05/20，2026/06/19，2026/08/25，2026/8/30，2026/9/4</t>
+          <t>2025/03/13，2025/03/14，2025/03/29，2025/04/19，2025/04/26，2025/05/09，2025/05/19，2025/05/22，2025/05/25，2025/07/03，2025/07/05，2025/07/28，2025/08/04，2025/08/21，2025/09/30，2025/11/14，2025/11/17，2026/02/10，2026/02/24，2026/03/18，2026/05/20，2026/06/19，2026/08/25，2026/08/30，2026/09/04</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4435,7 +4435,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/05/12，2025/05/22，2025/06/16，2025/06/30，2025/08/01，2025/08/16，2025/09/19，2025/10/05，2025/11/18，2025/12/23，2026/01/09，2026/02/27，2026/04/29，2026/07/05，2026/07/22</t>
+          <t>2025/03/13，2025/05/12，2025/05/22，2025/06/16，2025/06/30，2025/08/01，2025/08/16，2025/09/19，2025/10/05，2025/11/18，2025/12/23，2026/01/09，2026/02/27，2026/04/29，2026/07/05，2026/07/22，2026/09/06</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4446,7 +4446,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -4475,7 +4475,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/19，2025/05/20，2025/07/26，2025/08/16，2025/12/11，2026/04/09，2026/04/18，2026/07/22</t>
+          <t>2025/03/14，2025/05/19，2025/05/20，2025/07/26，2025/08/16，2025/12/11，2026/04/09，2026/04/18，2026/07/22，2026/09/08</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -4555,7 +4555,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/28，2025/05/15，2025/06/07，2025/07/18，2025/09/12，2025/11/09，2025/11/22，2026/03/09，2026/04/14，2026/05/20</t>
+          <t>2025/03/14，2025/03/28，2025/05/15，2025/06/07，2025/07/18，2025/09/12，2025/11/09，2025/11/22，2026/03/09，2026/04/14，2026/05/20，2026/09/13</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/20，2025/04/07，2025/05/06，2025/05/18，2025/05/30，2025/06/16，2025/06/27，2025/08/13，2025/08/24，2025/09/18，2025/09/19，2025/11/01，2026/02/14，2026/06/28，2026/07/22，2026/9/4</t>
+          <t>2025/03/14，2025/03/20，2025/04/07，2025/05/06，2025/05/18，2025/05/30，2025/06/16，2025/06/27，2025/08/13，2025/08/24，2025/09/18，2025/09/19，2025/11/01，2026/02/14，2026/06/28，2026/07/22，2026/09/04</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/01/12，2026/02/07，2026/03/15，2026/04/19，2026/06/26，2026/08/25，2026/8/30</t>
+          <t>2025/03/14，2025/04/14，2025/05/06，2025/05/30，2025/07/22，2025/08/26，2025/09/03，2025/10/10，2025/11/13，2025/12/19，2026/01/12，2026/02/07，2026/03/15，2026/04/19，2026/06/26，2026/08/25，2026/08/30</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/10/11，2025/11/14，2026/8/30</t>
+          <t>2025/03/14，2025/10/11，2025/11/14，2026/08/30</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/09，2026/01/15，2026/02/19，2026/03/13，2026/03/15，2026/03/21，2026/06/14，2026/06/17，2026/07/20，2026/07/31，2026/08/21，2026/8/28</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/09，2026/01/15，2026/02/19，2026/03/13，2026/03/15，2026/03/21，2026/06/14，2026/06/17，2026/07/20，2026/07/31，2026/08/21，2026/08/28，2026/08/30，2026/09/11</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5098,7 +5098,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/01/19，2026/04/18，2026/05/01，2026/05/23，2026/07/17，2026/08/25，2026/8/30</t>
+          <t>2025/03/14，2025/04/24，2025/05/03，2025/06/23，2025/08/21，2025/10/07，2025/10/31，2026/01/19，2026/04/18，2026/05/01，2026/05/23，2026/07/17，2026/08/25，2026/08/30，2026/09/11</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5167,7 +5167,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/05，2025/07/22，2026/02/27，2026/04/09，2026/04/14，2026/04/22，2026/06/10，2026/06/19，2026/9/4</t>
+          <t>2025/03/14，2025/04/05，2025/07/22，2026/02/27，2026/04/09，2026/04/14，2026/04/22，2026/06/10，2026/06/19，2026/09/04</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/28，2025/04/18，2025/09/20，2025/10/12，2025/10/22，2026/01/02，2026/01/30，2026/04/09，2026/07/31，2026/8/27</t>
+          <t>2025/03/14，2025/03/28，2025/04/18，2025/09/20，2025/10/12，2025/10/22，2026/01/02，2026/01/30，2026/04/09，2026/07/31，2026/08/27</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/03，2025/11/24，2026/04/09，2026/04/14，2026/04/24，2026/05/23，2026/08/02，2026/8/27</t>
+          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/03，2025/11/24，2026/04/09，2026/04/14，2026/04/24，2026/05/23，2026/08/02，2026/08/27，2026/09/06</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5258,7 +5258,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/05，2025/05/15，2025/08/12，2026/03/28</t>
+          <t>2025/03/15，2025/04/05，2025/05/15，2025/08/12，2026/03/28，2026/09/06</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/06/26，2025/08/04，2025/09/18，2025/10/25，2026/03/05，2026/07/28，2026/8/30</t>
+          <t>2025/03/15，2025/06/26，2025/08/04，2025/09/18，2025/10/25，2026/03/05，2026/07/28，2026/08/30</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -5607,7 +5607,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/08，2025/12/12，2026/02/14，2026/03/12，2026/04/09，2026/05/10，2026/05/23，2026/06/06，2026/06/25，2026/07/18，2026/08/25，2026/8/28</t>
+          <t>2025/03/15，2025/04/03，2025/04/11，2025/04/29，2025/05/18，2025/05/26，2025/06/02，2025/07/03，2025/08/21，2025/09/12，2025/11/19，2025/12/08，2025/12/12，2026/02/14，2026/03/12，2026/04/09，2026/05/10，2026/05/23，2026/06/06，2026/06/25，2026/07/18，2026/08/25，2026/08/28，2026/09/06</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -5618,7 +5618,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/07，2025/12/23，2026/01/05，2026/01/21，2026/01/29，2026/02/09，2026/02/20，2026/02/23，2026/03/04，2026/03/06，2026/03/07，2026/04/11，2026/04/14，2026/04/29，2026/05/23，2026/07/03，2026/07/21，2026/08/11，2026/08/25</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/07，2025/12/23，2026/01/05，2026/01/21，2026/01/29，2026/02/09，2026/02/20，2026/02/23，2026/03/04，2026/03/06，2026/03/07，2026/04/11，2026/04/14，2026/04/29，2026/05/23，2026/07/03，2026/07/21，2026/08/11，2026/08/25，2026/09/06</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5738,7 +5738,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/07，2026/03/06，2026/04/02，2026/06/20，2026/07/22，2026/9/4</t>
+          <t>2025/03/17，2025/04/14，2025/04/29，2025/07/15，2025/07/25，2025/08/04，2025/08/22，2025/09/11，2025/09/30，2025/10/25，2025/11/07，2026/03/06，2026/04/02，2026/06/20，2026/07/22，2026/09/04，2026/09/08</t>
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/29，2025/06/03，2025/07/24，2025/08/01，2025/08/03，2025/10/10，2025/11/09，2026/04/26，2026/08/02，2026/8/30</t>
+          <t>2025/03/17，2025/04/29，2025/06/03，2025/07/24，2025/08/01，2025/08/03，2025/10/10，2025/11/09，2026/04/26，2026/08/02，2026/08/30</t>
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/02，2025/09/12，2025/11/09，2025/12/04，2026/01/01，2026/01/29，2026/04/09，2026/06/15，2026/08/05，2026/8/30</t>
+          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/02，2025/09/12，2025/11/09，2025/12/04，2026/01/01，2026/01/29，2026/04/09，2026/06/15，2026/08/05，2026/08/30</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -6087,7 +6087,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08，2026/08/23，2026/8/30，2026/9/4</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08，2026/08/23，2026/08/30，2026/09/04</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/01/02，2026/01/15，2026/01/28，2026/02/19，2026/03/05，2026/04/09，2026/06/06，2026/06/20，2026/07/31，2026/07/31</t>
+          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/01/02，2026/01/15，2026/01/28，2026/02/19，2026/03/05，2026/04/09，2026/06/06，2026/06/20，2026/07/31，2026/07/31，2026/09/11</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -6247,7 +6247,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/05，2025/04/24，2025/05/12，2025/06/19，2025/07/11，2025/07/31，2025/09/03，2025/09/20，2025/10/17，2025/11/09，2025/11/21，2026/01/15，2026/8/27</t>
+          <t>2025/03/19，2025/04/05，2025/04/24，2025/05/12，2025/06/19，2025/07/11，2025/07/31，2025/09/03，2025/09/20，2025/10/17，2025/11/09，2025/11/21，2026/01/15，2026/08/27</t>
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -6287,7 +6287,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/05/13，2025/06/10，2025/08/21，2025/11/19，2026/01/10，2026/04/09，2026/9/4</t>
+          <t>2025/03/19，2025/04/07，2025/05/13，2025/06/10，2025/08/21，2025/11/19，2026/01/10，2026/04/09，2026/09/04</t>
         </is>
       </c>
       <c r="F144" t="inlineStr"/>
@@ -6327,7 +6327,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/08，2025/04/18，2025/05/12，2025/05/23，2025/06/27，2025/07/24，2025/08/28，2025/10/11，2025/10/31，2025/11/24，2025/12/19，2026/02/02，2026/04/19，2026/07/25，2026/9/2</t>
+          <t>2025/03/19，2025/04/08，2025/04/18，2025/05/12，2025/05/23，2025/06/27，2025/07/24，2025/08/28，2025/10/11，2025/10/31，2025/11/24，2025/12/19，2026/02/02，2026/04/19，2026/07/25，2026/09/02</t>
         </is>
       </c>
       <c r="F145" t="inlineStr"/>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/04，2026/01/03，2026/02/10，2026/03/13，2026/03/22，2026/04/14，2026/06/17，2026/08/25</t>
+          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/04，2026/01/03，2026/02/10，2026/03/13，2026/03/22，2026/04/14，2026/06/17，2026/08/25，2026/09/06</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/05/18，2025/06/13，2025/09/12，2025/10/01，2026/04/20，2026/06/10</t>
+          <t>2025/03/19，2025/04/07，2025/05/18，2025/06/13，2025/09/12，2025/10/01，2026/04/20，2026/06/10，2026/09/11</t>
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/01/01，2026/01/09，2026/03/22，2026/04/09，2026/04/20，2026/05/25，2026/06/10，2026/06/19，2026/08/11，2026/8/28，2026/8/28</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/01/01，2026/01/09，2026/03/22，2026/04/09，2026/04/20，2026/05/25，2026/06/10，2026/06/19，2026/08/11，2026/08/28，2026/08/28</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6527,7 +6527,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/17，2025/05/20，2025/05/31，2025/09/15，2025/10/13，2025/10/22，2025/12/24，2026/04/26，2026/06/19，2026/06/20，2026/8/28</t>
+          <t>2025/03/19，2025/04/17，2025/05/20，2025/05/31，2025/09/15，2025/10/13，2025/10/22，2025/12/24，2026/04/26，2026/06/19，2026/06/20，2026/08/28</t>
         </is>
       </c>
       <c r="F150" t="inlineStr"/>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/02，2026/01/16，2026/02/02，2026/02/23，2026/02/25，2026/03/17，2026/04/08，2026/05/06，2026/05/21，2026/06/25，2026/07/18，2026/08/25，2026/8/30</t>
+          <t>2025/03/20，2025/05/19，2025/06/12，2025/06/19，2025/06/23，2025/07/11，2025/08/03，2025/08/12，2025/08/21，2025/09/15，2025/10/07，2025/12/02，2026/01/16，2026/02/02，2026/02/23，2026/02/25，2026/03/17，2026/04/08，2026/05/06，2026/05/21，2026/06/25，2026/07/18，2026/08/25，2026/08/30</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/16，2025/08/26，2025/09/21，2025/10/03，2025/11/12，2025/12/08，2026/01/23，2026/01/26，2026/02/07，2026/02/10，2026/02/23，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/13，2026/03/24，2026/03/28，2026/03/29，2026/04/27，2026/05/02，2026/06/18，2026/07/04，2026/07/31，2026/08/25，2026/8/28</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/16，2025/08/26，2025/09/21，2025/10/03，2025/11/12，2025/12/08，2026/01/23，2026/01/26，2026/02/07，2026/02/10，2026/02/23，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/13，2026/03/24，2026/03/28，2026/03/29，2026/04/27，2026/05/02，2026/06/18，2026/07/04，2026/07/31，2026/08/25，2026/08/28，2026/09/06</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -6895,7 +6895,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/17，2025/05/13，2025/05/30，2025/06/06，2025/07/08，2025/08/07，2025/08/22，2025/09/30，2025/11/09，2025/11/13，2025/12/31，2026/04/16，2026/06/20</t>
+          <t>2025/03/20，2025/04/17，2025/05/13，2025/05/30，2025/06/06，2025/07/08，2025/08/07，2025/08/22，2025/09/30，2025/11/09，2025/11/13，2025/12/31，2026/04/16，2026/06/20，2026/09/08</t>
         </is>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -6906,7 +6906,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/08，2025/12/26，2026/01/05，2026/01/24，2026/02/05，2026/02/14，2026/03/09，2026/03/28，2026/04/26，2026/05/05，2026/05/23，2026/06/12，2026/8/27</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/08，2025/12/26，2026/01/05，2026/01/24，2026/02/05，2026/02/14，2026/03/09，2026/03/28，2026/04/26，2026/05/05，2026/05/23，2026/06/12，2026/08/27，2026/09/11</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/06/28，2025/08/04，2026/01/19，2026/04/08，2026/8/30</t>
+          <t>2025/03/21，2025/06/28，2025/08/04，2026/01/19，2026/04/08，2026/08/30，2026/09/06</t>
         </is>
       </c>
       <c r="F163" t="inlineStr"/>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/12，2025/12/07，2026/04/24，2026/8/30</t>
+          <t>2025/03/21，2025/05/12，2025/12/07，2026/04/24，2026/08/30</t>
         </is>
       </c>
       <c r="F164" t="inlineStr"/>
@@ -7331,7 +7331,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/06，2026/02/07，2026/03/24，2026/04/26，2026/05/04，2026/05/23，2026/07/09，2026/07/27，2026/9/2</t>
+          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/06，2026/02/07，2026/03/24，2026/04/26，2026/05/04，2026/05/23，2026/07/09，2026/07/27，2026/09/02，2026/09/08</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -7342,7 +7342,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -7482,18 +7482,18 @@
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
-          <t>TWICE</t>
+          <t>Lenka</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/09/28，2026/8/27</t>
+          <t>2025/03/21，2025/09/28，2026/08/27</t>
         </is>
       </c>
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>韩语</t>
+          <t>英语</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -7527,7 +7527,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11，2026/8/28</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11，2026/08/28</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7611,7 +7611,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/08，2026/02/18，2026/03/06，2026/03/13，2026/03/14，2026/03/31，2026/05/01，2026/06/28，2026/07/17，2026/08/02，2026/08/21，2026/9/4</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/08，2026/02/18，2026/03/06，2026/03/13，2026/03/14，2026/03/31，2026/05/01，2026/06/28，2026/07/17，2026/08/02，2026/08/21，2026/09/04</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7735,7 +7735,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/01/19，2026/03/09，2026/04/18，2026/04/20，2026/05/10，2026/06/19，2026/06/26，2026/07/27，2026/8/28</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/01/19，2026/03/09，2026/04/18，2026/04/20，2026/05/10，2026/06/19，2026/06/26，2026/07/27，2026/08/28</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7775,7 +7775,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/07，2025/04/18，2025/05/08，2025/10/24，2025/12/12，2026/04/26</t>
+          <t>2025/03/21，2025/04/07，2025/04/18，2025/05/08，2025/10/24，2025/12/12，2026/04/26，2026/09/06</t>
         </is>
       </c>
       <c r="F181" t="inlineStr"/>
@@ -7786,7 +7786,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -7895,7 +7895,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/02，2025/12/05，2025/12/30，2026/01/23，2026/01/29，2026/02/23，2026/03/17，2026/03/22，2026/04/19，2026/05/10，2026/06/12，2026/07/22，2026/08/08，2026/8/28，2026/8/28</t>
+          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/02，2025/12/05，2025/12/30，2026/01/23，2026/01/29，2026/02/23，2026/03/17，2026/03/22，2026/04/19，2026/05/10，2026/06/12，2026/07/22，2026/08/08，2026/08/28，2026/08/28</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -7975,7 +7975,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/03，2025/04/19，2025/05/26，2025/09/18，2025/10/17，2026/01/01，2026/05/10，2026/9/4</t>
+          <t>2025/03/22，2025/04/03，2025/04/19，2025/05/26，2025/09/18，2025/10/17，2026/01/01，2026/05/10，2026/09/04</t>
         </is>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -8015,7 +8015,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/04/01，2025/05/12，2025/05/31，2025/07/11，2025/08/16，2025/09/19，2025/09/24，2025/11/18，2026/01/09，2026/02/14</t>
+          <t>2025/03/23，2025/04/01，2025/05/12，2025/05/31，2025/07/11，2025/08/16，2025/09/19，2025/09/24，2025/11/18，2026/01/09，2026/02/14，2026/09/08</t>
         </is>
       </c>
       <c r="F187" t="inlineStr"/>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -8055,7 +8055,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/01/29，2026/02/09，2026/03/25，2026/04/19，2026/05/23，2026/06/12，2026/07/22，2026/07/27，2026/9/4</t>
+          <t>2025/03/23，2025/03/28，2025/04/06，2025/05/15，2025/05/22，2025/05/29，2025/06/07，2025/06/09，2025/07/06，2025/07/15，2025/09/06，2025/09/14，2025/09/30，2025/11/13，2026/01/29，2026/02/09，2026/03/25，2026/04/19，2026/05/23，2026/06/12，2026/07/22，2026/07/27，2026/09/04，2026/09/13</t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -8066,7 +8066,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/04/17，2025/05/25，2025/12/02，2026/01/14，2026/06/06</t>
+          <t>2025/03/23，2025/04/17，2025/05/25，2025/12/02，2026/01/14，2026/06/06，2026/09/08</t>
         </is>
       </c>
       <c r="F189" t="inlineStr"/>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -8135,7 +8135,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/04/10，2025/05/01，2025/05/19，2025/06/08，2025/07/14，2025/09/11，2025/09/12，2025/10/31，2026/01/09，2026/07/05，2026/9/4</t>
+          <t>2025/03/23，2025/04/10，2025/05/01，2025/05/19，2025/06/08，2025/07/14，2025/09/11，2025/09/12，2025/10/31，2026/01/09，2026/07/05，2026/09/04，2026/09/11</t>
         </is>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/07，2026/01/17，2026/02/14，2026/04/09，2026/05/20，2026/06/19，2026/06/28，2026/07/31，2026/9/4</t>
+          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/07，2026/01/17，2026/02/14，2026/04/09，2026/05/20，2026/06/19，2026/06/28，2026/07/31，2026/09/04</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -8535,7 +8535,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/07/24，2025/07/29，2025/07/31，2025/09/04，2025/09/24，2025/10/03，2025/10/16，2025/11/18，2025/11/21，2026/03/05，2026/06/06</t>
+          <t>2025/03/25，2025/07/24，2025/07/29，2025/07/31，2025/09/04，2025/09/24，2025/10/03，2025/10/16，2025/11/18，2025/11/21，2026/03/05，2026/06/06，2026/09/11</t>
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -8615,7 +8615,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/09/24，2025/11/27，2026/04/14，2026/06/10，2026/8/30</t>
+          <t>2025/03/25，2025/09/24，2025/11/27，2026/04/14，2026/06/10，2026/08/30</t>
         </is>
       </c>
       <c r="F202" t="inlineStr"/>
@@ -8775,7 +8775,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/09/19，2025/10/10，2025/11/09，2026/9/4</t>
+          <t>2025/03/25，2025/09/19，2025/10/10，2025/11/09，2026/09/04</t>
         </is>
       </c>
       <c r="F206" t="inlineStr"/>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/24，2025/05/13，2025/06/02，2025/06/27，2025/07/14，2025/08/26，2025/09/02，2025/10/03，2025/10/17，2025/11/21，2026/02/14，2026/02/23，2026/02/25，2026/03/09，2026/03/15，2026/8/28</t>
+          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/24，2025/05/13，2025/06/02，2025/06/27，2025/07/14，2025/08/26，2025/09/02，2025/10/03，2025/10/17，2025/11/21，2026/02/14，2026/02/23，2026/02/25，2026/03/09，2026/03/15，2026/08/28</t>
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
@@ -8895,7 +8895,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/17，2025/05/15，2025/05/27，2025/11/27，2025/12/24，2026/01/14，2026/06/28，2026/08/18</t>
+          <t>2025/03/27，2025/04/17，2025/05/15，2025/05/27，2025/11/27，2025/12/24，2026/01/14，2026/06/28，2026/08/18，2026/09/08</t>
         </is>
       </c>
       <c r="F209" t="inlineStr"/>
@@ -8906,7 +8906,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/15，2025/05/08，2025/06/10，2025/07/07，2025/08/04，2025/09/04，2025/10/01，2025/11/26，2026/01/10，2026/03/22，2026/06/20，2026/07/20</t>
+          <t>2025/03/27，2025/04/15，2025/05/08，2025/06/10，2025/07/07，2025/08/04，2025/09/04，2025/10/01，2025/11/26，2026/01/10，2026/03/22，2026/06/20，2026/07/20，2026/09/11</t>
         </is>
       </c>
       <c r="F213" t="inlineStr"/>
@@ -9078,7 +9078,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/03/25，2026/04/09，2026/05/10，2026/06/10，2026/8/30</t>
+          <t>2025/03/27，2025/05/09，2025/05/29，2025/07/24，2025/09/04，2025/10/24，2025/11/19，2026/03/25，2026/04/09，2026/05/10，2026/06/10，2026/08/30</t>
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
@@ -9183,7 +9183,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/01/16，2026/02/02，2026/02/07，2026/03/31，2026/04/17，2026/04/29，2026/05/15，2026/05/19，2026/06/12，2026/08/07</t>
+          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/01/16，2026/02/02，2026/02/07，2026/03/31，2026/04/17，2026/04/29，2026/05/15，2026/05/19，2026/06/12，2026/08/07，2026/09/11</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -9194,7 +9194,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -9263,7 +9263,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/01/16，2026/06/06，2026/07/09，2026/08/08，2026/9/2</t>
+          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/01/16，2026/06/06，2026/07/09，2026/08/08，2026/09/02</t>
         </is>
       </c>
       <c r="F218" t="inlineStr"/>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/23，2025/06/13，2025/06/26，2025/07/11，2025/09/18，2025/11/03，2025/12/23，2025/12/26，2026/01/24，2026/06/03，2026/07/18，2026/8/30，2026/8/30</t>
+          <t>2025/03/28，2025/05/23，2025/06/13，2025/06/26，2025/07/11，2025/09/18，2025/11/03，2025/12/23，2025/12/26，2026/01/24，2026/06/03，2026/07/18，2026/08/30，2026/08/30</t>
         </is>
       </c>
       <c r="F220" t="inlineStr"/>
@@ -9463,7 +9463,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/09，2026/01/09，2026/02/19，2026/05/10，2026/07/10，2026/07/15，2026/07/31，2026/8/28</t>
+          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/09，2026/01/09，2026/02/19，2026/05/10，2026/07/10，2026/07/15，2026/07/31，2026/08/28</t>
         </is>
       </c>
       <c r="F223" t="inlineStr"/>
@@ -9659,7 +9659,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/08/16，2026/9/2</t>
+          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/08/16，2026/09/02</t>
         </is>
       </c>
       <c r="F228" t="inlineStr"/>
@@ -9739,7 +9739,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/24，2025/06/02，2025/06/27，2025/09/21，2025/10/07，2025/11/13，2025/12/02，2026/08/01，2026/8/28</t>
+          <t>2025/03/28，2025/04/24，2025/06/02，2025/06/27，2025/09/21，2025/10/07，2025/11/13，2025/12/02，2026/08/01，2026/08/28</t>
         </is>
       </c>
       <c r="F230" t="inlineStr"/>
@@ -9943,7 +9943,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/03，2025/11/09，2025/12/23，2026/04/08，2026/04/24，2026/05/21，2026/06/10，2026/08/02，2026/8/28，2026/8/30</t>
+          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/03，2025/11/09，2025/12/23，2026/04/08，2026/04/24，2026/05/21，2026/06/10，2026/08/02，2026/08/28，2026/08/30</t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
@@ -9983,7 +9983,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/07，2025/11/13，2025/12/02，2026/01/14，2026/01/24，2026/03/07，2026/03/15，2026/04/24，2026/06/06，2026/06/23，2026/08/05，2026/08/05，2026/08/19，2026/9/4</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/07，2025/11/13，2025/12/02，2026/01/14，2026/01/24，2026/03/07，2026/03/15，2026/04/24，2026/06/06，2026/06/23，2026/08/05，2026/08/05，2026/08/19，2026/09/04</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
@@ -10023,7 +10023,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/25，2025/05/03，2025/06/23，2025/09/28，2025/11/28，2025/12/26，2026/06/28，2026/8/27</t>
+          <t>2025/03/29，2025/04/25，2025/05/03，2025/06/23，2025/09/28，2025/11/28，2025/12/26，2026/06/28，2026/08/27</t>
         </is>
       </c>
       <c r="F237" t="inlineStr"/>
@@ -10271,7 +10271,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/22，2025/06/29，2025/09/30，2025/10/23，2026/01/19，2026/08/18，2026/8/30</t>
+          <t>2025/03/30，2025/05/22，2025/06/29，2025/09/30，2025/10/23，2026/01/19，2026/08/18，2026/08/30</t>
         </is>
       </c>
       <c r="F243" t="inlineStr"/>
@@ -10351,7 +10351,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/01/09，2026/03/07，2026/04/19，2026/05/23，2026/07/16，2026/8/27</t>
+          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/01/09，2026/03/07，2026/04/19，2026/05/23，2026/07/16，2026/08/27</t>
         </is>
       </c>
       <c r="F245" t="inlineStr"/>
@@ -10391,7 +10391,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/27，2025/05/19，2025/05/31，2025/08/30，2025/09/02，2025/11/18，2026/04/22，2026/07/31，2026/8/28</t>
+          <t>2025/03/30，2025/04/27，2025/05/19，2025/05/31，2025/08/30，2025/09/02，2025/11/18，2026/04/22，2026/07/31，2026/08/28</t>
         </is>
       </c>
       <c r="F246" t="inlineStr"/>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/04，2025/04/26，2025/05/06，2025/05/18，2025/06/10，2025/07/03，2025/07/10，2025/07/24，2025/08/16，2025/09/18，2025/10/03，2025/11/01，2026/02/14，2026/04/09，2026/07/09，2026/9/4</t>
+          <t>2025/03/30，2025/04/04，2025/04/26，2025/05/06，2025/05/18，2025/06/10，2025/07/03，2025/07/10，2025/07/24，2025/08/16，2025/09/18，2025/10/03，2025/11/01，2026/02/14，2026/04/09，2026/07/09，2026/09/04</t>
         </is>
       </c>
       <c r="F247" t="inlineStr"/>
@@ -10471,7 +10471,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/01/01，2026/01/25，2026/03/08，2026/04/27，2026/06/13，2026/07/28，2026/8/28</t>
+          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/01/01，2026/01/25，2026/03/08，2026/04/27，2026/06/13，2026/07/28，2026/08/28</t>
         </is>
       </c>
       <c r="F248" t="inlineStr"/>
@@ -10511,7 +10511,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>2025/03/30，2026/8/30</t>
+          <t>2025/03/30，2026/08/30</t>
         </is>
       </c>
       <c r="F249" t="inlineStr"/>
@@ -10551,7 +10551,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/19，2025/06/23，2025/07/08，2025/09/21，2025/10/23，2025/11/14，2025/12/17，2026/02/07，2026/08/18，2026/9/4</t>
+          <t>2025/03/30，2025/04/19，2025/06/23，2025/07/08，2025/09/21，2025/10/23，2025/11/14，2025/12/17，2026/02/07，2026/08/18，2026/09/04</t>
         </is>
       </c>
       <c r="F250" t="inlineStr"/>
@@ -10631,7 +10631,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/02/12，2026/04/16，2026/05/20，2026/06/20，2026/8/27</t>
+          <t>2025/04/01，2025/04/11，2025/04/18，2025/04/29，2025/05/08，2025/07/22，2025/07/29，2025/08/04，2025/08/21，2025/09/06，2025/10/09，2025/12/12，2026/02/12，2026/04/16，2026/05/20，2026/06/20，2026/08/27</t>
         </is>
       </c>
       <c r="F252" t="inlineStr"/>
@@ -10751,7 +10751,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/06/23，2025/07/08，2025/09/30，2025/10/23，2026/02/07，2026/06/28，2026/08/18</t>
+          <t>2025/04/01，2025/06/23，2025/07/08，2025/09/30，2025/10/23，2026/02/07，2026/06/28，2026/08/18，2026/09/08</t>
         </is>
       </c>
       <c r="F255" t="inlineStr"/>
@@ -10762,7 +10762,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -10791,7 +10791,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/01/21，2026/02/25，2026/02/27，2026/03/01，2026/03/08，2026/03/13，2026/03/25，2026/04/01，2026/05/01，2026/05/07，2026/05/08，2026/05/23，2026/06/13，2026/08/21</t>
+          <t>2025/04/01，2025/04/28，2025/05/22，2025/06/08，2025/06/27，2025/07/08，2025/08/01，2025/09/03，2025/09/28，2025/10/16，2025/10/23，2025/10/31，2025/12/19，2025/12/31，2026/01/21，2026/02/25，2026/02/27，2026/03/01，2026/03/08，2026/03/13，2026/03/25，2026/04/01，2026/05/01，2026/05/07，2026/05/08，2026/05/23，2026/06/13，2026/08/21，2026/09/12</t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
@@ -10802,7 +10802,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -10871,7 +10871,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/05/10，2025/09/04，2025/09/10，2025/09/28，2025/11/26，2026/01/19，2026/05/10，2026/08/18</t>
+          <t>2025/04/01，2025/05/10，2025/09/04，2025/09/10，2025/09/28，2025/11/26，2026/01/19，2026/05/10，2026/08/18，2026/09/06</t>
         </is>
       </c>
       <c r="F258" t="inlineStr"/>
@@ -10882,7 +10882,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/02/08，2026/03/17，2026/05/05，2026/05/21，2026/06/25，2026/07/16，2026/08/23，2026/8/28</t>
+          <t>2025/04/01，2025/04/24，2025/05/12，2025/05/26，2025/06/23，2025/06/27，2025/07/20，2025/08/30，2025/09/15，2025/09/22，2025/10/07，2025/10/28，2025/11/26，2025/12/28，2026/02/08，2026/03/17，2026/05/05，2026/05/21，2026/06/25，2026/07/16，2026/08/23，2026/08/28，2026/09/11</t>
         </is>
       </c>
       <c r="F259" t="inlineStr"/>
@@ -10922,7 +10922,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -10951,7 +10951,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/01/02，2026/01/05，2026/02/02，2026/02/09，2026/02/19，2026/03/25，2026/05/10，2026/05/21，2026/07/16，2026/8/27，2026/8/27</t>
+          <t>2025/04/01，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/11，2026/01/02，2026/01/05，2026/02/02，2026/02/09，2026/02/19，2026/03/25，2026/05/10，2026/05/21，2026/07/16，2026/08/27，2026/09/11</t>
         </is>
       </c>
       <c r="F260" t="inlineStr"/>
@@ -11071,7 +11071,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/21，2025/05/19，2025/06/02，2025/07/03，2025/09/19，2025/10/16</t>
+          <t>2025/04/02，2025/04/21，2025/05/19，2025/06/02，2025/07/03，2025/09/19，2025/10/16，2026/09/13</t>
         </is>
       </c>
       <c r="F263" t="inlineStr"/>
@@ -11082,7 +11082,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/27，2025/07/24，2026/01/01，2026/06/14，2026/8/30</t>
+          <t>2025/04/02，2025/05/27，2025/07/24，2026/01/01，2026/06/14，2026/08/30，2026/09/08</t>
         </is>
       </c>
       <c r="F265" t="inlineStr"/>
@@ -11162,7 +11162,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/12，2025/05/23，2025/06/08，2025/07/29，2025/08/13，2025/08/28，2025/09/28，2025/09/29，2025/11/09，2025/12/06，2025/12/24，2026/04/13，2026/05/04，2026/07/27，2026/9/2</t>
+          <t>2025/04/02，2025/04/12，2025/05/23，2025/06/08，2025/07/29，2025/08/13，2025/08/28，2025/09/28，2025/09/29，2025/11/09，2025/12/06，2025/12/24，2026/04/13，2026/05/04，2026/07/27，2026/09/02</t>
         </is>
       </c>
       <c r="F268" t="inlineStr"/>
@@ -11311,7 +11311,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/13，2025/05/10，2025/05/26，2025/06/02，2025/06/05，2025/06/17，2025/08/04，2025/09/10，2025/09/30，2025/10/16，2025/11/17，2025/12/06，2025/12/31，2026/04/26，2026/07/22，2026/8/30</t>
+          <t>2025/04/02，2025/04/13，2025/05/10，2025/05/26，2025/06/02，2025/06/05，2025/06/17，2025/08/04，2025/09/10，2025/09/30，2025/10/16，2025/11/17，2025/12/06，2025/12/31，2026/04/26，2026/07/22，2026/08/30</t>
         </is>
       </c>
       <c r="F269" t="inlineStr"/>
@@ -11431,7 +11431,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/04/03，2025/04/08，2025/05/26，2025/07/18，2025/08/16，2025/09/30，2025/11/26，2026/01/23，2026/02/18，2026/03/12，2026/06/10，2026/9/4</t>
+          <t>2025/04/02，2025/04/03，2025/04/08，2025/05/26，2025/07/18，2025/08/16，2025/09/30，2025/11/26，2026/01/23，2026/02/18，2026/03/12，2026/06/10，2026/09/04</t>
         </is>
       </c>
       <c r="F272" t="inlineStr"/>
@@ -11471,7 +11471,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08，2026/8/28</t>
+          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08，2026/08/28</t>
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
@@ -11515,7 +11515,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/03/09，2026/03/13，2026/03/17，2026/05/01，2026/06/18，2026/8/30</t>
+          <t>2025/04/03，2025/06/20，2025/09/19，2025/10/12，2026/03/09，2026/03/13，2026/03/17，2026/05/01，2026/06/18，2026/08/30</t>
         </is>
       </c>
       <c r="F274" t="inlineStr"/>
@@ -11595,7 +11595,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/05/17，2025/05/29，2025/06/16，2025/07/10，2025/08/24，2025/10/16，2025/11/26，2026/04/26</t>
+          <t>2025/04/03，2025/05/17，2025/05/29，2025/06/16，2025/07/10，2025/08/24，2025/10/16，2025/11/26，2026/04/26，2026/09/11</t>
         </is>
       </c>
       <c r="F276" t="inlineStr"/>
@@ -11606,7 +11606,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -11635,7 +11635,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/14，2025/04/24，2025/06/01，2025/07/06，2025/09/21，2025/11/03，2025/12/12，2025/12/26，2026/04/08，2026/07/20，2026/8/30</t>
+          <t>2025/04/03，2025/04/14，2025/04/24，2025/06/01，2025/07/06，2025/09/21，2025/11/03，2025/12/12，2025/12/26，2026/04/08，2026/07/20，2026/08/30</t>
         </is>
       </c>
       <c r="F277" t="inlineStr"/>
@@ -11675,7 +11675,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/06，2026/01/09，2026/01/29，2026/03/25，2026/04/24，2026/05/23，2026/06/15，2026/07/09，2026/07/22，2026/08/25，2026/8/28</t>
+          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/06，2026/01/09，2026/01/29，2026/03/25，2026/04/24，2026/05/23，2026/06/15，2026/07/09，2026/07/22，2026/08/25，2026/08/28</t>
         </is>
       </c>
       <c r="F278" t="inlineStr"/>
@@ -11795,7 +11795,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/24，2025/09/12，2026/01/10，2026/06/03，2026/9/4</t>
+          <t>2025/04/03，2025/04/24，2025/09/12，2026/01/10，2026/06/03，2026/09/04</t>
         </is>
       </c>
       <c r="F281" t="inlineStr"/>
@@ -11835,7 +11835,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/05/12，2025/05/18，2025/06/20，2025/07/05，2025/07/14，2025/12/23，2026/01/30，2026/04/09，2026/8/30</t>
+          <t>2025/04/04，2025/05/12，2025/05/18，2025/06/20，2025/07/05，2025/07/14，2025/12/23，2026/01/30，2026/04/09，2026/08/30</t>
         </is>
       </c>
       <c r="F282" t="inlineStr"/>
@@ -11875,7 +11875,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/06/02，2025/06/29，2025/07/24，2025/07/26，2025/08/21，2025/11/09，2025/12/16，2026/9/2</t>
+          <t>2025/04/04，2025/06/02，2025/06/29，2025/07/24，2025/07/26，2025/08/21，2025/11/09，2025/12/16，2026/09/02</t>
         </is>
       </c>
       <c r="F283" t="inlineStr"/>
@@ -11915,7 +11915,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>2025/04/04，2026/01/29</t>
+          <t>2025/04/04，2026/01/29，2026/09/08</t>
         </is>
       </c>
       <c r="F284" t="inlineStr"/>
@@ -11926,7 +11926,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I284" t="inlineStr"/>
@@ -12187,7 +12187,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/07/13，2025/07/18，2025/11/03，2025/11/28，2026/08/16，2026/8/30</t>
+          <t>2025/04/04，2025/07/13，2025/07/18，2025/11/03，2025/11/28，2026/08/16，2026/08/30</t>
         </is>
       </c>
       <c r="F291" t="inlineStr"/>
@@ -12307,7 +12307,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/02/14，2026/03/05，2026/04/02，2026/05/20，2026/8/28</t>
+          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/02/14，2026/03/05，2026/04/02，2026/05/20，2026/08/28</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -12387,7 +12387,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>2025/04/06，2025/04/10，2025/06/20，2025/12/23，2026/04/09</t>
+          <t>2025/04/06，2025/04/10，2025/06/20，2025/12/23，2026/04/09，2026/09/08</t>
         </is>
       </c>
       <c r="F296" t="inlineStr"/>
@@ -12398,7 +12398,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -12631,7 +12631,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>2025/04/06，2025/05/23，2025/06/10，2025/10/03，2025/11/01</t>
+          <t>2025/04/06，2025/05/23，2025/06/10，2025/10/03，2025/11/01，2026/09/08</t>
         </is>
       </c>
       <c r="F302" t="inlineStr"/>
@@ -12642,7 +12642,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -12671,7 +12671,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/05/09，2025/06/19，2025/07/22，2026/03/09，2026/8/30，2026/9/4</t>
+          <t>2025/04/07，2025/05/09，2025/06/19，2025/07/22，2026/03/09，2026/08/30，2026/09/04</t>
         </is>
       </c>
       <c r="F303" t="inlineStr"/>
@@ -12751,7 +12751,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23，2026/8/30</t>
+          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23，2026/08/30，2026/09/11</t>
         </is>
       </c>
       <c r="F305" t="inlineStr"/>
@@ -12762,7 +12762,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/01/03，2026/01/22，2026/02/14，2026/05/20，2026/08/08，2026/08/19，2026/08/25</t>
+          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/01/03，2026/01/22，2026/02/14，2026/05/20，2026/08/08，2026/08/19，2026/08/25，2026/09/06</t>
         </is>
       </c>
       <c r="F307" t="inlineStr"/>
@@ -12842,7 +12842,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -12871,7 +12871,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/05/08，2025/05/20，2025/05/30，2025/06/16，2025/08/29，2025/09/12，2025/10/09，2025/10/16，2025/11/18，2026/02/04，2026/02/14，2026/04/15，2026/06/13，2026/07/07，2026/07/28，2026/8/28</t>
+          <t>2025/04/07，2025/04/17，2025/05/08，2025/05/20，2025/05/30，2025/06/16，2025/08/29，2025/09/12，2025/10/09，2025/10/16，2025/11/18，2026/02/04，2026/02/14，2026/04/15，2026/06/13，2026/07/07，2026/07/28，2026/08/28，2026/08/28，2026/09/13</t>
         </is>
       </c>
       <c r="F308" t="inlineStr"/>
@@ -12882,7 +12882,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
@@ -12911,7 +12911,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/03，2025/11/09，2025/11/26，2025/12/09，2026/01/23，2026/03/13，2026/03/25，2026/04/08，2026/05/23，2026/06/20，2026/08/02，2026/8/28</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/03，2025/11/09，2025/11/26，2025/12/09，2026/01/23，2026/03/13，2026/03/25，2026/04/08，2026/05/23，2026/06/20，2026/08/02，2026/08/28，2026/09/11</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12922,7 +12922,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -12951,7 +12951,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/09，2026/01/24，2026/03/31，2026/04/02，2026/06/15，2026/07/27，2026/9/2</t>
+          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/09，2026/01/24，2026/03/31，2026/04/02，2026/06/15，2026/07/27，2026/09/02</t>
         </is>
       </c>
       <c r="F310" t="inlineStr"/>
@@ -13231,7 +13231,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/06/29，2025/08/01，2025/09/04，2025/09/21，2025/10/17，2025/11/09，2025/11/13，2025/12/04，2025/12/13，2026/03/04，2026/05/07，2026/06/20，2026/8/28</t>
+          <t>2025/04/11，2025/06/29，2025/08/01，2025/09/04，2025/09/21，2025/10/17，2025/11/09，2025/11/13，2025/12/04，2025/12/13，2026/03/04，2026/05/07，2026/06/20，2026/08/28</t>
         </is>
       </c>
       <c r="F317" t="inlineStr"/>
@@ -13307,7 +13307,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/18，2025/06/09，2025/07/07，2025/08/26，2025/09/03，2025/09/13，2025/10/17，2025/10/30，2025/11/21，2025/12/17，2026/04/19，2026/8/27</t>
+          <t>2025/04/11，2025/05/18，2025/06/09，2025/07/07，2025/08/26，2025/09/03，2025/09/13，2025/10/17，2025/10/30，2025/11/21，2025/12/17，2026/04/19，2026/08/27</t>
         </is>
       </c>
       <c r="F319" t="inlineStr"/>
@@ -13391,7 +13391,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/09，2025/12/08，2026/01/05，2026/02/14，2026/05/23，2026/06/20，2026/07/18，2026/08/25</t>
+          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/09，2025/12/08，2026/01/05，2026/02/14，2026/05/23，2026/06/20，2026/07/18，2026/08/25，2026/08/30</t>
         </is>
       </c>
       <c r="F321" t="inlineStr"/>
@@ -13402,7 +13402,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -13863,7 +13863,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>2025/04/12，2025/07/14，2025/09/24，2025/09/28，2025/11/09，2026/04/24，2026/9/4</t>
+          <t>2025/04/12，2025/07/14，2025/09/24，2025/09/28，2025/11/09，2026/04/24，2026/09/04</t>
         </is>
       </c>
       <c r="F333" t="inlineStr"/>
@@ -13943,7 +13943,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>2025/04/12，2026/8/30，2026/9/4</t>
+          <t>2025/04/12，2026/08/30，2026/09/04</t>
         </is>
       </c>
       <c r="F335" t="inlineStr"/>
@@ -13983,7 +13983,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/01/09，2026/02/08，2026/03/01，2026/03/09，2026/03/24，2026/04/17，2026/05/01，2026/05/21，2026/06/10，2026/06/25，2026/07/27，2026/08/23，2026/8/28，2026/9/4</t>
+          <t>2025/04/13，2025/05/26，2025/06/07，2025/06/21，2025/07/05，2025/08/21，2025/09/15，2025/10/23，2025/11/24，2025/12/23，2026/01/09，2026/02/08，2026/03/01，2026/03/09，2026/03/24，2026/04/17，2026/05/01，2026/05/21，2026/06/10，2026/06/25，2026/07/27，2026/08/23，2026/08/28，2026/09/04</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -14027,7 +14027,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/21，2025/04/22，2025/04/25，2025/04/26，2025/04/29，2025/05/08，2025/05/12，2025/05/22，2025/05/30，2025/06/06，2025/06/08，2025/06/28，2025/07/13，2025/08/12，2025/08/24，2025/09/07，2025/09/30，2025/10/05，2025/11/21，2025/12/17，2026/01/14，2026/01/23，2026/02/12，2026/03/31，2026/06/18，2026/07/17，2026/9/2</t>
+          <t>2025/04/13，2025/04/21，2025/04/22，2025/04/25，2025/04/26，2025/04/29，2025/05/08，2025/05/12，2025/05/22，2025/05/30，2025/06/06，2025/06/08，2025/06/28，2025/07/13，2025/08/12，2025/08/24，2025/09/07，2025/09/30，2025/10/05，2025/11/21，2025/12/17，2026/01/14，2026/01/23，2026/02/12，2026/03/31，2026/06/18，2026/07/17，2026/09/02，2026/09/08</t>
         </is>
       </c>
       <c r="F337" t="inlineStr"/>
@@ -14038,7 +14038,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
@@ -14119,7 +14119,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/04/18，2025/08/28，2026/01/16，2026/05/01，2026/8/30</t>
+          <t>2025/04/13，2025/04/18，2025/08/28，2026/01/16，2026/05/01，2026/08/30</t>
         </is>
       </c>
       <c r="F339" t="inlineStr"/>
@@ -14159,7 +14159,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/07/13，2025/07/18，2025/08/02，2025/09/04，2025/09/12，2025/10/17，2025/11/28，2026/01/22，2026/02/23，2026/9/4</t>
+          <t>2025/04/13，2025/07/13，2025/07/18，2025/08/02，2025/09/04，2025/09/12，2025/10/17，2025/11/28，2026/01/22，2026/02/23，2026/09/04</t>
         </is>
       </c>
       <c r="F340" t="inlineStr"/>
@@ -14323,7 +14323,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>2025/04/14，2025/05/24，2025/06/15，2025/06/19，2025/07/21，2025/08/22，2025/09/20，2025/10/09，2025/10/28，2025/12/22，2026/06/20，2026/8/27</t>
+          <t>2025/04/14，2025/05/24，2025/06/15，2025/06/19，2025/07/21，2025/08/22，2025/09/20，2025/10/09，2025/10/28，2025/12/22，2026/06/20，2026/08/27</t>
         </is>
       </c>
       <c r="F344" t="inlineStr"/>
@@ -14403,7 +14403,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/05/13，2025/07/14，2025/09/18，2026/01/01，2026/01/09，2026/02/20，2026/04/18，2026/05/10，2026/07/16，2026/9/2</t>
+          <t>2025/04/15，2025/05/13，2025/07/14，2025/09/18，2026/01/01，2026/01/09，2026/02/20，2026/04/18，2026/05/10，2026/07/16，2026/09/02</t>
         </is>
       </c>
       <c r="F346" t="inlineStr"/>
@@ -14443,7 +14443,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/01/16，2026/03/25，2026/04/24，2026/05/23，2026/07/17，2026/08/21</t>
+          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/01/16，2026/03/25，2026/04/24，2026/05/23，2026/07/17，2026/08/21，2026/09/11</t>
         </is>
       </c>
       <c r="F347" t="inlineStr"/>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -14727,7 +14727,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/06/01，2025/08/18，2026/03/06，2026/03/17</t>
+          <t>2025/04/17，2025/06/01，2025/08/18，2026/03/06，2026/03/17，2026/09/13</t>
         </is>
       </c>
       <c r="F354" t="inlineStr"/>
@@ -14738,7 +14738,7 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
@@ -14851,7 +14851,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/04/29，2025/05/22，2025/05/25，2025/05/31，2025/08/29，2025/09/20，2025/10/09，2025/10/30，2025/12/11，2026/02/18，2026/05/20，2026/07/05，2026/07/31</t>
+          <t>2025/04/17，2025/04/29，2025/05/22，2025/05/25，2025/05/31，2025/08/29，2025/09/20，2025/10/09，2025/10/30，2025/12/11，2026/02/18，2026/05/20，2026/07/05，2026/07/31，2026/09/06</t>
         </is>
       </c>
       <c r="F357" t="inlineStr"/>
@@ -14862,7 +14862,7 @@
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
@@ -14891,7 +14891,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/05/31，2025/06/03，2025/06/14，2025/09/10，2026/03/28，2026/8/28</t>
+          <t>2025/04/17，2025/05/31，2025/06/03，2025/06/14，2025/09/10，2026/03/28，2026/08/28</t>
         </is>
       </c>
       <c r="F358" t="inlineStr"/>
@@ -15291,7 +15291,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/06/17，2025/08/28，2026/8/30</t>
+          <t>2025/04/19，2025/06/17，2025/08/28，2026/08/30</t>
         </is>
       </c>
       <c r="F368" t="inlineStr"/>
@@ -15411,7 +15411,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/09，2025/11/26，2025/12/05，2025/12/06，2026/01/01，2026/01/29，2026/03/01，2026/04/09，2026/05/20，2026/07/27</t>
+          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/09，2025/11/26，2025/12/05，2025/12/06，2026/01/01，2026/01/29，2026/03/01，2026/04/09，2026/05/20，2026/07/27，2026/09/11</t>
         </is>
       </c>
       <c r="F371" t="inlineStr"/>
@@ -15422,7 +15422,7 @@
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I371" t="inlineStr">
@@ -15619,7 +15619,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>2025/04/21，2025/05/23，2025/06/29，2025/07/26，2025/09/28，2025/12/02，2025/12/17，2026/05/06，2026/9/2，2026/9/4</t>
+          <t>2025/04/21，2025/05/23，2025/06/29，2025/07/26，2025/09/28，2025/12/02，2025/12/17，2026/05/06，2026/09/02，2026/09/04</t>
         </is>
       </c>
       <c r="F376" t="inlineStr"/>
@@ -15699,7 +15699,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>2025/04/22，2025/04/29，2025/05/03，2025/05/03，2025/06/03，2025/09/02，2025/10/10，2025/10/20，2025/10/31，2026/02/07，2026/03/13，2026/08/11</t>
+          <t>2025/04/22，2025/04/29，2025/05/03，2025/05/03，2025/06/03，2025/09/02，2025/10/10，2025/10/20，2025/10/31，2026/02/07，2026/03/13，2026/08/11，2026/09/06</t>
         </is>
       </c>
       <c r="F378" t="inlineStr"/>
@@ -15710,7 +15710,7 @@
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I378" t="inlineStr">
@@ -15851,7 +15851,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>2025/04/24，2025/09/22，2026/03/29，2026/06/10，2026/8/28</t>
+          <t>2025/04/24，2025/09/22，2026/03/29，2026/06/10，2026/08/28</t>
         </is>
       </c>
       <c r="F382" t="inlineStr"/>
@@ -16039,7 +16039,7 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/05/15，2025/09/12，2025/09/30，2025/10/16，2025/11/13</t>
+          <t>2025/04/25，2025/05/15，2025/09/12，2025/09/30，2025/10/16，2025/11/13，2026/09/13</t>
         </is>
       </c>
       <c r="F387" t="inlineStr"/>
@@ -16050,7 +16050,7 @@
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I387" t="inlineStr">
@@ -16431,7 +16431,7 @@
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/07/23，2025/09/19，2026/07/22</t>
+          <t>2025/04/25，2025/07/23，2025/09/19，2026/07/22，2026/09/13</t>
         </is>
       </c>
       <c r="F397" t="inlineStr"/>
@@ -16442,7 +16442,7 @@
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
@@ -16591,7 +16591,7 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/05/04，2025/05/26，2025/06/08，2025/08/28，2025/10/18，2025/11/18，2025/12/24，2026/01/29，2026/02/27，2026/04/09，2026/04/20</t>
+          <t>2025/04/27，2025/05/04，2025/05/26，2025/06/08，2025/08/28，2025/10/18，2025/11/18，2025/12/24，2026/01/29，2026/02/27，2026/04/09，2026/04/20，2026/09/06</t>
         </is>
       </c>
       <c r="F401" t="inlineStr"/>
@@ -16602,7 +16602,7 @@
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
@@ -16835,7 +16835,7 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/11/18，2026/02/14，2026/04/09，2026/05/16，2026/06/14，2026/08/02，2026/9/4</t>
+          <t>2025/04/28，2025/11/18，2026/02/14，2026/04/09，2026/05/16，2026/06/14，2026/08/02，2026/09/04</t>
         </is>
       </c>
       <c r="F407" t="inlineStr"/>
@@ -16875,7 +16875,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/05/12，2025/05/23，2025/07/20，2025/10/18，2026/01/19，2026/07/27，2026/9/2</t>
+          <t>2025/04/28，2025/05/12，2025/05/23，2025/07/20，2025/10/18，2026/01/19，2026/07/27，2026/09/02</t>
         </is>
       </c>
       <c r="F408" t="inlineStr"/>
@@ -16991,7 +16991,7 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>2025/04/29，2025/05/03，2026/04/20</t>
+          <t>2025/04/29，2025/05/03，2026/04/20，2026/09/11</t>
         </is>
       </c>
       <c r="F411" t="inlineStr"/>
@@ -17002,7 +17002,7 @@
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I411" t="inlineStr">
@@ -17071,7 +17071,7 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>2025/05/01，2025/08/12，2025/08/26，2025/11/24，2026/06/20，2026/8/30</t>
+          <t>2025/05/01，2025/08/12，2025/08/26，2025/11/24，2026/06/20，2026/08/30</t>
         </is>
       </c>
       <c r="F413" t="inlineStr"/>
@@ -17231,7 +17231,7 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/07/18，2025/08/02，2025/10/16，2026/05/01，2026/8/27</t>
+          <t>2025/05/03，2025/07/18，2025/08/02，2025/10/16，2026/05/01，2026/08/27</t>
         </is>
       </c>
       <c r="F417" t="inlineStr"/>
@@ -17271,7 +17271,7 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/06/13，2025/09/08，2026/04/25，2026/8/30</t>
+          <t>2025/05/03，2025/06/13，2025/09/08，2026/04/25，2026/08/30</t>
         </is>
       </c>
       <c r="F418" t="inlineStr"/>
@@ -17351,7 +17351,7 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>2025/05/03，2026/8/27</t>
+          <t>2025/05/03，2026/08/27</t>
         </is>
       </c>
       <c r="F420" t="inlineStr"/>
@@ -17551,7 +17551,7 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/04/20，2026/05/23，2026/8/28，2026/9/4</t>
+          <t>2025/05/08，2025/06/16，2025/06/21，2025/07/05，2025/07/14，2025/09/12，2025/11/26，2026/04/20，2026/05/23，2026/08/28，2026/09/04，2026/09/11</t>
         </is>
       </c>
       <c r="F425" t="inlineStr"/>
@@ -17562,7 +17562,7 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
@@ -17822,12 +17822,12 @@
       <c r="C432" t="inlineStr"/>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Adele</t>
+          <t>张靓颖</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/04/29，2026/08/07，2026/9/2</t>
+          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/04/29，2026/08/07，2026/09/02</t>
         </is>
       </c>
       <c r="F432" t="inlineStr"/>
@@ -18227,7 +18227,7 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/27，2025/07/10，2026/03/09，2026/04/09，2026/06/10，2026/8/28，2026/8/28</t>
+          <t>2025/05/18，2025/06/27，2025/07/10，2026/03/09，2026/04/09，2026/06/10，2026/08/28，2026/08/28</t>
         </is>
       </c>
       <c r="F442" t="inlineStr"/>
@@ -18427,7 +18427,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/01/02，2026/03/17，2026/04/29，2026/05/10，2026/07/09，2026/07/31，2026/08/11，2026/08/25，2026/9/4</t>
+          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/01/02，2026/03/17，2026/04/29，2026/05/10，2026/07/09，2026/07/31，2026/08/11，2026/08/25，2026/09/04</t>
         </is>
       </c>
       <c r="F447" t="inlineStr"/>
@@ -18507,7 +18507,7 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/12/16，2025/12/24，2026/08/16，2026/8/30</t>
+          <t>2025/05/19，2025/12/16，2025/12/24，2026/08/16，2026/08/30</t>
         </is>
       </c>
       <c r="F449" t="inlineStr"/>
@@ -18547,7 +18547,7 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/07/13，2025/08/21，2025/12/17，2026/05/23，2026/08/11</t>
+          <t>2025/05/19，2025/07/13，2025/08/21，2025/12/17，2026/05/23，2026/08/11，2026/09/06</t>
         </is>
       </c>
       <c r="F450" t="inlineStr"/>
@@ -18558,7 +18558,7 @@
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I450" t="inlineStr">
@@ -18711,7 +18711,7 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/06/17，2025/06/23，2025/07/06，2025/07/15，2025/09/10，2025/10/18，2025/11/13，2026/05/04，2026/07/09</t>
+          <t>2025/05/22，2025/06/17，2025/06/23，2025/07/06，2025/07/15，2025/09/10，2025/10/18，2025/11/13，2026/05/04，2026/07/09，2026/08/30</t>
         </is>
       </c>
       <c r="F454" t="inlineStr"/>
@@ -18722,7 +18722,7 @@
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I454" t="inlineStr">
@@ -18751,7 +18751,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/09/02，2025/09/12，2025/12/05，2026/04/09，2026/05/10，2026/8/30</t>
+          <t>2025/05/22，2025/09/02，2025/09/12，2025/12/05，2026/04/09，2026/05/10，2026/08/30</t>
         </is>
       </c>
       <c r="F455" t="inlineStr"/>
@@ -18919,7 +18919,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/01/05，2026/02/02，2026/03/17，2026/05/10，2026/06/14，2026/06/15，2026/07/31，2026/9/2</t>
+          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/01/05，2026/02/02，2026/03/17，2026/05/10，2026/06/14，2026/06/15，2026/07/31，2026/09/02</t>
         </is>
       </c>
       <c r="F459" t="inlineStr"/>
@@ -19083,7 +19083,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>2025/05/23，2026/8/30</t>
+          <t>2025/05/23，2026/08/30</t>
         </is>
       </c>
       <c r="F463" t="inlineStr"/>
@@ -19163,7 +19163,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>2025/05/23，2025/06/26，2025/07/21，2025/08/12，2025/09/10，2025/09/19，2025/11/01，2025/12/09，2025/12/13，2026/02/14，2026/04/24，2026/06/16</t>
+          <t>2025/05/23，2025/06/26，2025/07/21，2025/08/12，2025/09/10，2025/09/19，2025/11/01，2025/12/09，2025/12/13，2026/02/14，2026/04/24，2026/06/16，2026/09/13</t>
         </is>
       </c>
       <c r="F465" t="inlineStr"/>
@@ -19174,7 +19174,7 @@
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I465" t="inlineStr">
@@ -19243,7 +19243,7 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>2025/05/24，2025/07/13，2025/08/23，2025/09/29，2025/12/24，2025/12/30，2026/01/28，2026/04/08，2026/08/16</t>
+          <t>2025/05/24，2025/07/13，2025/08/23，2025/09/29，2025/12/24，2025/12/30，2026/01/28，2026/04/08，2026/08/16，2026/09/12</t>
         </is>
       </c>
       <c r="F467" t="inlineStr"/>
@@ -19254,7 +19254,7 @@
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I467" t="inlineStr">
@@ -19403,7 +19403,7 @@
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>2025/05/26，2025/07/03，2025/09/15，2026/9/2</t>
+          <t>2025/05/26，2025/07/03，2025/09/15，2026/09/02</t>
         </is>
       </c>
       <c r="F471" t="inlineStr"/>
@@ -19683,7 +19683,7 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/09/03，2025/09/11，2025/09/29，2025/11/09，2026/01/01，2026/04/20，2026/8/30</t>
+          <t>2025/05/30，2025/09/03，2025/09/11，2025/09/29，2025/11/09，2026/01/01，2026/04/20，2026/08/30</t>
         </is>
       </c>
       <c r="F478" t="inlineStr"/>
@@ -20407,7 +20407,7 @@
       </c>
       <c r="E496" t="inlineStr">
         <is>
-          <t>2025/06/01，2026/01/23，2026/02/02，2026/02/23，2026/03/05，2026/03/17，2026/04/24，2026/05/16</t>
+          <t>2025/06/01，2026/01/23，2026/02/02，2026/02/23，2026/03/05，2026/03/17，2026/04/24，2026/05/16，2026/09/13</t>
         </is>
       </c>
       <c r="F496" t="inlineStr"/>
@@ -20418,7 +20418,7 @@
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I496" t="inlineStr">
@@ -20607,7 +20607,7 @@
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>2025/06/02，2025/06/07，2025/06/12，2025/06/28，2025/08/13，2025/09/11，2025/09/30，2025/11/27，2026/8/27</t>
+          <t>2025/06/02，2025/06/07，2025/06/12，2025/06/28，2025/08/13，2025/09/11，2025/09/30，2025/11/27，2026/08/27</t>
         </is>
       </c>
       <c r="F501" t="inlineStr"/>
@@ -20800,7 +20800,11 @@
         </is>
       </c>
       <c r="C506" t="inlineStr"/>
-      <c r="D506" t="inlineStr"/>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>中央人民广播电台少年广播合唱团</t>
+        </is>
+      </c>
       <c r="E506" t="inlineStr">
         <is>
           <t>2025/06/06</t>
@@ -21287,7 +21291,7 @@
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/02，2025/12/09，2025/12/16，2025/12/26，2026/01/05，2026/01/15，2026/01/28，2026/03/06，2026/04/22，2026/05/10，2026/05/15，2026/06/19，2026/07/09，2026/07/31，2026/08/21</t>
+          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/02，2025/12/09，2025/12/16，2025/12/26，2026/01/05，2026/01/15，2026/01/28，2026/03/06，2026/04/22，2026/05/10，2026/05/15，2026/06/19，2026/07/09，2026/07/31，2026/08/21，2026/09/11</t>
         </is>
       </c>
       <c r="F518" t="inlineStr"/>
@@ -21298,7 +21302,7 @@
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I518" t="inlineStr">
@@ -21487,7 +21491,7 @@
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>2025/06/17，2025/09/24，2026/9/2</t>
+          <t>2025/06/17，2025/09/24，2026/09/02</t>
         </is>
       </c>
       <c r="F523" t="inlineStr"/>
@@ -21767,7 +21771,7 @@
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/07，2025/11/21，2025/12/02，2025/12/17，2026/01/01，2026/01/05，2026/01/14，2026/01/22，2026/01/24，2026/02/02，2026/03/05，2026/03/15，2026/04/01，2026/05/04，2026/05/25，2026/06/20，2026/07/05，2026/07/18，2026/07/28，2026/08/11，2026/8/30</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/07，2025/11/21，2025/12/02，2025/12/17，2026/01/01，2026/01/05，2026/01/14，2026/01/22，2026/01/24，2026/02/02，2026/03/05，2026/03/15，2026/04/01，2026/05/04，2026/05/25，2026/06/20，2026/07/05，2026/07/18，2026/07/28，2026/08/11，2026/08/30</t>
         </is>
       </c>
       <c r="F530" t="inlineStr"/>
@@ -21971,7 +21975,7 @@
       </c>
       <c r="E535" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/02/18，2026/03/09，2026/04/16，2026/04/24，2026/05/15，2026/05/23，2026/06/12，2026/07/22，2026/08/11</t>
+          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/02/18，2026/03/09，2026/04/16，2026/04/24，2026/05/15，2026/05/23，2026/06/12，2026/07/22，2026/08/11，2026/09/06</t>
         </is>
       </c>
       <c r="F535" t="inlineStr"/>
@@ -21982,7 +21986,7 @@
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I535" t="inlineStr">
@@ -22051,7 +22055,7 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>2025/06/23，2025/10/23，2026/07/09，2026/9/2</t>
+          <t>2025/06/23，2025/10/23，2026/07/09，2026/09/02</t>
         </is>
       </c>
       <c r="F537" t="inlineStr"/>
@@ -22091,7 +22095,7 @@
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>2025/06/23，2026/8/30</t>
+          <t>2025/06/23，2026/08/30</t>
         </is>
       </c>
       <c r="F538" t="inlineStr"/>
@@ -22371,7 +22375,7 @@
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/01/14，2026/01/22，2026/02/19，2026/03/13，2026/04/12，2026/05/10，2026/06/17，2026/08/08，2026/08/18</t>
+          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/01/14，2026/01/22，2026/02/19，2026/03/13，2026/04/12，2026/05/10，2026/06/17，2026/08/08，2026/08/18，2026/09/11</t>
         </is>
       </c>
       <c r="F545" t="inlineStr"/>
@@ -22382,7 +22386,7 @@
       </c>
       <c r="H545" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I545" t="inlineStr">
@@ -22415,7 +22419,7 @@
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/03/08，2026/05/01，2026/05/23，2026/07/17，2026/08/25</t>
+          <t>2025/06/26，2025/09/21，2025/10/31，2025/11/28，2026/03/08，2026/05/01，2026/05/23，2026/07/17，2026/08/25，2026/09/06</t>
         </is>
       </c>
       <c r="F546" t="inlineStr"/>
@@ -22426,7 +22430,7 @@
       </c>
       <c r="H546" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I546" t="inlineStr">
@@ -22667,7 +22671,7 @@
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>2025/06/29，2025/09/19，2025/11/22，2026/07/22，2026/9/2</t>
+          <t>2025/06/29，2025/09/19，2025/11/22，2026/07/22，2026/09/02</t>
         </is>
       </c>
       <c r="F552" t="inlineStr"/>
@@ -22707,7 +22711,7 @@
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/08/16，2026/8/30，2026/9/4</t>
+          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/08/16，2026/08/30，2026/09/04，2026/09/12</t>
         </is>
       </c>
       <c r="F553" t="inlineStr"/>
@@ -22718,7 +22722,7 @@
       </c>
       <c r="H553" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I553" t="inlineStr">
@@ -22747,7 +22751,7 @@
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>2025/06/29，2026/08/11，2026/08/21，2026/8/30</t>
+          <t>2025/06/29，2026/08/11，2026/08/21，2026/08/30，2026/09/06</t>
         </is>
       </c>
       <c r="F554" t="inlineStr"/>
@@ -22758,7 +22762,7 @@
       </c>
       <c r="H554" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I554" t="inlineStr">
@@ -22827,7 +22831,7 @@
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>2025/06/29，2026/8/30</t>
+          <t>2025/06/29，2026/08/30</t>
         </is>
       </c>
       <c r="F556" t="inlineStr"/>
@@ -22867,7 +22871,7 @@
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>2025/06/29，2026/8/30</t>
+          <t>2025/06/29，2026/08/30</t>
         </is>
       </c>
       <c r="F557" t="inlineStr"/>
@@ -23183,7 +23187,7 @@
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/09，2026/01/09，2026/01/23，2026/02/12，2026/02/25，2026/03/09，2026/03/28，2026/05/10，2026/06/06，2026/9/2</t>
+          <t>2025/07/03，2025/07/07，2025/07/26，2025/08/28，2025/09/14，2025/10/11，2025/11/26，2025/12/09，2026/01/09，2026/01/23，2026/02/12，2026/02/25，2026/03/09，2026/03/28，2026/05/10，2026/06/06，2026/09/02</t>
         </is>
       </c>
       <c r="F565" t="inlineStr"/>
@@ -23419,7 +23423,7 @@
       </c>
       <c r="E571" t="inlineStr">
         <is>
-          <t>2025/07/07，2025/07/31，2025/09/11，2025/10/11，2025/11/07，2025/11/12，2025/12/09，2026/01/14，2026/01/30，2026/04/09，2026/8/28</t>
+          <t>2025/07/07，2025/07/31，2025/09/11，2025/10/11，2025/11/07，2025/11/12，2025/12/09，2026/01/14，2026/01/30，2026/04/09，2026/08/28，2026/09/06</t>
         </is>
       </c>
       <c r="F571" t="inlineStr"/>
@@ -23430,7 +23434,7 @@
       </c>
       <c r="H571" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I571" t="inlineStr">
@@ -23699,7 +23703,7 @@
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/01/09，2026/03/07，2026/03/08，2026/06/14，2026/8/27</t>
+          <t>2025/07/11，2025/07/15，2025/07/15，2025/08/04，2025/09/28，2025/10/05，2026/01/09，2026/03/07，2026/03/08，2026/06/14，2026/08/27</t>
         </is>
       </c>
       <c r="F578" t="inlineStr"/>
@@ -23899,7 +23903,7 @@
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>2025/07/14，2025/07/18，2025/07/28，2025/08/07，2025/08/10，2025/09/04，2025/09/18，2025/10/16，2025/10/22，2026/06/03，2026/07/26，2026/8/27</t>
+          <t>2025/07/14，2025/07/18，2025/07/28，2025/08/07，2025/08/10，2025/09/04，2025/09/18，2025/10/16，2025/10/22，2026/06/03，2026/07/26，2026/08/27</t>
         </is>
       </c>
       <c r="F583" t="inlineStr"/>
@@ -23979,7 +23983,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/03，2025/11/22，2026/01/05，2026/02/18，2026/02/23，2026/04/19，2026/06/06，2026/06/19，2026/07/28，2026/8/28</t>
+          <t>2025/07/14，2025/07/17，2025/07/18，2025/07/24，2025/07/28，2025/08/02，2025/08/03，2025/08/21，2025/09/05，2025/09/18，2025/09/30，2025/10/19，2025/11/03，2025/11/22，2026/01/05，2026/02/18，2026/02/23，2026/04/19，2026/06/06，2026/06/19，2026/07/28，2026/08/28</t>
         </is>
       </c>
       <c r="F585" t="inlineStr"/>
@@ -24059,7 +24063,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>2025/07/15，2026/01/05，2026/01/10，2026/01/25，2026/02/10，2026/02/27，2026/03/07，2026/03/15，2026/03/29，2026/06/23，2026/8/28</t>
+          <t>2025/07/15，2026/01/05，2026/01/10，2026/01/25，2026/02/10，2026/02/27，2026/03/07，2026/03/15，2026/03/29，2026/06/23，2026/08/28</t>
         </is>
       </c>
       <c r="F587" t="inlineStr"/>
@@ -24367,7 +24371,7 @@
       </c>
       <c r="E595" t="inlineStr">
         <is>
-          <t>2025/07/21</t>
+          <t>2025/07/21，2026/09/08</t>
         </is>
       </c>
       <c r="F595" t="inlineStr"/>
@@ -24378,7 +24382,7 @@
       </c>
       <c r="H595" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I595" t="inlineStr">
@@ -24531,7 +24535,7 @@
       </c>
       <c r="E599" t="inlineStr">
         <is>
-          <t>2025/07/26</t>
+          <t>2025/07/26，2026/09/06</t>
         </is>
       </c>
       <c r="F599" t="inlineStr"/>
@@ -24542,7 +24546,7 @@
       </c>
       <c r="H599" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I599" t="inlineStr">
@@ -24731,7 +24735,7 @@
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/01/19，2026/02/12，2026/02/14，2026/04/08，2026/04/19，2026/05/20，2026/06/06，2026/07/22，2026/8/27</t>
+          <t>2025/07/31，2025/08/01，2025/08/04，2025/08/09，2025/08/13，2025/08/21，2025/08/29，2025/09/10，2025/09/30，2025/10/30，2025/11/14，2025/12/24，2026/01/19，2026/02/12，2026/02/14，2026/04/08，2026/04/19，2026/05/20，2026/06/06，2026/07/22，2026/08/27，2026/09/08</t>
         </is>
       </c>
       <c r="F604" t="inlineStr"/>
@@ -24742,7 +24746,7 @@
       </c>
       <c r="H604" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I604" t="inlineStr">
@@ -25003,7 +25007,7 @@
       </c>
       <c r="E611" t="inlineStr">
         <is>
-          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/02，2025/12/17，2026/01/14，2026/02/02，2026/03/22，2026/04/01，2026/04/08，2026/05/15，2026/06/10，2026/07/31，2026/08/25</t>
+          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/02，2025/12/17，2026/01/14，2026/02/02，2026/03/22，2026/04/01，2026/04/08，2026/05/15，2026/06/10，2026/07/31，2026/08/25，2026/09/06</t>
         </is>
       </c>
       <c r="F611" t="inlineStr"/>
@@ -25014,7 +25018,7 @@
       </c>
       <c r="H611" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I611" t="inlineStr">
@@ -25123,7 +25127,7 @@
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/01，2025/11/26，2025/12/30，2026/01/10，2026/02/18，2026/04/10，2026/04/23，2026/05/23，2026/06/18，2026/07/13，2026/08/07，2026/9/4</t>
+          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/01，2025/11/26，2025/12/30，2026/01/10，2026/02/18，2026/04/10，2026/04/23，2026/05/23，2026/06/18，2026/07/13，2026/08/07，2026/09/04</t>
         </is>
       </c>
       <c r="F614" t="inlineStr"/>
@@ -26307,7 +26311,7 @@
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/03，2025/11/13，2025/11/24，2025/12/05，2025/12/12，2025/12/17，2026/01/06，2026/01/15，2026/01/24，2026/02/27，2026/04/19，2026/06/06，2026/07/17，2026/07/28，2026/8/28，2026/8/30</t>
+          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/03，2025/11/13，2025/11/24，2025/12/05，2025/12/12，2025/12/17，2026/01/06，2026/01/15，2026/01/24，2026/02/27，2026/04/19，2026/06/06，2026/07/17，2026/07/28，2026/08/28，2026/08/30</t>
         </is>
       </c>
       <c r="F644" t="inlineStr"/>
@@ -26423,7 +26427,7 @@
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/02/23，2026/03/17，2026/03/25，2026/05/23，2026/8/27</t>
+          <t>2025/09/17，2025/10/11，2025/10/13，2025/10/20，2025/10/25，2025/11/21，2025/12/17，2026/02/23，2026/03/17，2026/03/25，2026/05/23，2026/08/27</t>
         </is>
       </c>
       <c r="F647" t="inlineStr"/>
@@ -26851,7 +26855,7 @@
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>2025/09/20，2025/09/21，2025/09/22，2025/09/24，2025/09/27，2025/10/05，2025/10/12，2025/10/22，2025/11/01，2025/12/06，2025/12/12，2026/01/19，2026/04/08，2026/05/20，2026/06/06，2026/06/28，2026/07/22</t>
+          <t>2025/09/20，2025/09/21，2025/09/22，2025/09/24，2025/09/27，2025/10/05，2025/10/12，2025/10/22，2025/11/01，2025/12/06，2025/12/12，2026/01/19，2026/04/08，2026/05/20，2026/06/06，2026/06/28，2026/07/22，2026/09/13</t>
         </is>
       </c>
       <c r="F658" t="inlineStr"/>
@@ -26862,7 +26866,7 @@
       </c>
       <c r="H658" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I658" t="inlineStr">
@@ -26891,7 +26895,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31，2026/08/23，2026/9/4</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31，2026/08/23，2026/09/04</t>
         </is>
       </c>
       <c r="F659" t="inlineStr"/>
@@ -27159,7 +27163,7 @@
       </c>
       <c r="E666" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/29，2025/10/13，2025/10/17，2025/10/19，2025/10/20，2025/10/25，2025/10/28，2025/11/07，2025/11/26，2025/12/06，2025/12/12，2025/12/24，2026/01/05，2026/01/19，2026/02/18，2026/03/14，2026/03/24，2026/06/10，2026/07/22</t>
+          <t>2025/09/24，2025/09/29，2025/10/13，2025/10/17，2025/10/19，2025/10/20，2025/10/25，2025/10/28，2025/11/07，2025/11/26，2025/12/06，2025/12/12，2025/12/24，2026/01/05，2026/01/19，2026/02/18，2026/03/14，2026/03/24，2026/06/10，2026/07/22，2026/09/11</t>
         </is>
       </c>
       <c r="F666" t="inlineStr"/>
@@ -27170,7 +27174,7 @@
       </c>
       <c r="H666" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I666" t="inlineStr">
@@ -27271,7 +27275,7 @@
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/26，2025/09/28，2025/09/29，2025/10/01，2025/10/07，2025/10/10，2025/10/11，2025/10/17，2025/10/23，2025/10/28，2025/12/26，2026/02/05，2026/07/16，2026/07/31，2026/08/19，2026/8/30</t>
+          <t>2025/09/24，2025/09/26，2025/09/28，2025/09/29，2025/10/01，2025/10/07，2025/10/10，2025/10/11，2025/10/17，2025/10/23，2025/10/28，2025/12/26，2026/02/05，2026/07/16，2026/07/31，2026/08/19，2026/08/30</t>
         </is>
       </c>
       <c r="F669" t="inlineStr"/>
@@ -27507,7 +27511,7 @@
       </c>
       <c r="E675" t="inlineStr">
         <is>
-          <t>2025/09/28，2026/9/4</t>
+          <t>2025/09/28，2026/09/04</t>
         </is>
       </c>
       <c r="F675" t="inlineStr"/>
@@ -27587,7 +27591,7 @@
       </c>
       <c r="E677" t="inlineStr">
         <is>
-          <t>2025/09/29，2025/10/07，2025/10/10，2025/10/13，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/06，2026/01/15，2026/01/19，2026/03/07，2026/05/05</t>
+          <t>2025/09/29，2025/10/07，2025/10/10，2025/10/13，2025/10/17，2025/10/22，2025/10/25，2025/11/21，2025/12/06，2026/01/15，2026/01/19，2026/03/07，2026/05/05，2026/09/11</t>
         </is>
       </c>
       <c r="F677" t="inlineStr"/>
@@ -27598,7 +27602,7 @@
       </c>
       <c r="H677" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I677" t="inlineStr">
@@ -28231,7 +28235,7 @@
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>2025/10/13，2025/10/18，2026/03/15，2026/08/09，2026/9/2</t>
+          <t>2025/10/13，2025/10/18，2026/03/15，2026/08/09，2026/09/02</t>
         </is>
       </c>
       <c r="F693" t="inlineStr"/>
@@ -28591,7 +28595,7 @@
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>2025/10/23，2026/08/16，2026/08/21，2026/9/4</t>
+          <t>2025/10/23，2026/08/16，2026/08/21，2026/09/04</t>
         </is>
       </c>
       <c r="F702" t="inlineStr"/>
@@ -29059,7 +29063,7 @@
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>2025/10/28，2025/11/01，2025/11/12，2025/12/19，2026/02/08，2026/02/10，2026/05/10，2026/08/16，2026/9/2</t>
+          <t>2025/10/28，2025/11/01，2025/11/12，2025/12/19，2026/02/08，2026/02/10，2026/05/10，2026/08/16，2026/09/02</t>
         </is>
       </c>
       <c r="F714" t="inlineStr"/>
@@ -29175,7 +29179,7 @@
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>2025/10/31，2025/11/12</t>
+          <t>2025/10/31，2025/11/12，2026/09/06</t>
         </is>
       </c>
       <c r="F717" t="inlineStr"/>
@@ -29186,7 +29190,7 @@
       </c>
       <c r="H717" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I717" t="inlineStr">
@@ -29483,7 +29487,7 @@
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/06，2025/12/12，2025/12/26，2026/01/05，2026/01/30，2026/02/09，2026/03/25，2026/05/01，2026/06/17，2026/07/25，2026/9/2</t>
+          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/06，2025/12/12，2025/12/26，2026/01/05，2026/01/30，2026/02/09，2026/03/25，2026/05/01，2026/06/17，2026/07/25，2026/09/02</t>
         </is>
       </c>
       <c r="F725" t="inlineStr"/>
@@ -29679,7 +29683,11 @@
         </is>
       </c>
       <c r="F730" t="inlineStr"/>
-      <c r="G730" t="inlineStr"/>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>西语</t>
+        </is>
+      </c>
       <c r="H730" t="inlineStr">
         <is>
           <t>2</t>
@@ -30059,7 +30067,7 @@
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/06，2025/12/13，2026/01/10，2026/01/24，2026/02/14，2026/03/14，2026/04/01，2026/04/08，2026/05/01，2026/05/06，2026/05/23，2026/06/20，2026/07/18，2026/08/07，2026/9/2</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/06，2025/12/13，2026/01/10，2026/01/24，2026/02/14，2026/03/14，2026/04/01，2026/04/08，2026/05/01，2026/05/06，2026/05/23，2026/06/20，2026/07/18，2026/08/07，2026/09/02</t>
         </is>
       </c>
       <c r="F740" t="inlineStr"/>
@@ -30099,7 +30107,7 @@
       </c>
       <c r="E741" t="inlineStr">
         <is>
-          <t>2025/11/28，2026/9/2</t>
+          <t>2025/11/28，2026/09/02</t>
         </is>
       </c>
       <c r="F741" t="inlineStr"/>
@@ -30115,7 +30123,7 @@
       </c>
       <c r="I741" t="inlineStr">
         <is>
-          <t>BV1Q6to6JEEx</t>
+          <t>BV1UatD6hEMa，BV1Q6to6JEEx</t>
         </is>
       </c>
       <c r="J741" t="inlineStr"/>
@@ -30371,7 +30379,7 @@
       </c>
       <c r="E748" t="inlineStr">
         <is>
-          <t>2025/12/09，2026/02/02，2026/04/14</t>
+          <t>2025/12/09，2026/02/02，2026/04/14，2026/09/06</t>
         </is>
       </c>
       <c r="F748" t="inlineStr"/>
@@ -30382,7 +30390,7 @@
       </c>
       <c r="H748" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I748" t="inlineStr">
@@ -30415,7 +30423,7 @@
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>2025/12/09，2025/12/17，2026/01/14，2026/01/23，2026/02/05，2026/02/10，2026/02/25，2026/04/08，2026/05/01，2026/06/16，2026/08/16</t>
+          <t>2025/12/09，2025/12/17，2026/01/14，2026/01/23，2026/02/05，2026/02/10，2026/02/25，2026/04/08，2026/05/01，2026/06/16，2026/08/16，2026/09/06</t>
         </is>
       </c>
       <c r="F749" t="inlineStr"/>
@@ -30426,7 +30434,7 @@
       </c>
       <c r="H749" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I749" t="inlineStr">
@@ -30763,7 +30771,7 @@
       </c>
       <c r="E758" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/24，2025/12/26，2026/01/02，2026/01/09，2026/01/23，2026/01/29，2026/03/22，2026/04/29，2026/06/20，2026/08/11</t>
+          <t>2025/12/19，2025/12/24，2025/12/26，2026/01/02，2026/01/09，2026/01/23，2026/01/29，2026/03/22，2026/04/29，2026/06/20，2026/08/11，2026/09/13</t>
         </is>
       </c>
       <c r="F758" t="inlineStr"/>
@@ -30774,7 +30782,7 @@
       </c>
       <c r="H758" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I758" t="inlineStr">
@@ -30843,7 +30851,7 @@
       </c>
       <c r="E760" t="inlineStr">
         <is>
-          <t>2025/12/19，2026/9/4</t>
+          <t>2025/12/19，2026/09/04</t>
         </is>
       </c>
       <c r="F760" t="inlineStr"/>
@@ -30883,7 +30891,7 @@
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/01/02，2026/01/05，2026/01/11，2026/01/25，2026/02/09，2026/02/23，2026/03/20，2026/04/02，2026/04/16，2026/04/29，2026/05/10，2026/06/06，2026/06/14，2026/06/20，2026/07/16，2026/08/02，2026/08/07，2026/08/23，2026/8/28</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/01/02，2026/01/05，2026/01/11，2026/01/25，2026/02/09，2026/02/23，2026/03/20，2026/04/02，2026/04/16，2026/04/29，2026/05/10，2026/06/06，2026/06/14，2026/06/20，2026/07/16，2026/08/02，2026/08/07，2026/08/23，2026/08/28，2026/09/11</t>
         </is>
       </c>
       <c r="F761" t="inlineStr"/>
@@ -30894,7 +30902,7 @@
       </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I761" t="inlineStr">
@@ -30923,7 +30931,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08，2026/08/19，2026/9/2</t>
+          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08，2026/08/19，2026/09/02</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -30963,7 +30971,7 @@
       </c>
       <c r="E763" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/01/05，2026/01/19，2026/01/21，2026/01/22，2026/01/24，2026/02/07，2026/02/19，2026/02/24，2026/02/24，2026/02/25，2026/03/06，2026/03/25，2026/04/11，2026/04/20，2026/05/15，2026/06/19，2026/07/18，2026/08/21，2026/8/28</t>
+          <t>2025/12/26，2026/01/05，2026/01/19，2026/01/21，2026/01/22，2026/01/24，2026/02/07，2026/02/19，2026/02/24，2026/02/24，2026/02/25，2026/03/06，2026/03/25，2026/04/11，2026/04/20，2026/05/15，2026/06/19，2026/07/18，2026/08/21，2026/08/28</t>
         </is>
       </c>
       <c r="F763" t="inlineStr"/>
@@ -31047,7 +31055,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/01/10，2026/01/22，2026/01/23，2026/01/31，2026/02/10，2026/02/23，2026/03/09，2026/03/12，2026/03/14，2026/03/17，2026/03/27，2026/04/24，2026/05/01，2026/06/14，2026/08/01，2026/8/28</t>
+          <t>2025/12/26，2026/01/10，2026/01/22，2026/01/23，2026/01/31，2026/02/10，2026/02/23，2026/03/09，2026/03/12，2026/03/14，2026/03/17，2026/03/27，2026/04/24，2026/05/01，2026/06/14，2026/08/01，2026/08/28</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -31283,7 +31291,7 @@
       </c>
       <c r="E771" t="inlineStr">
         <is>
-          <t>2026/01/19</t>
+          <t>2026/01/19，2026/09/06</t>
         </is>
       </c>
       <c r="F771" t="inlineStr"/>
@@ -31294,10 +31302,14 @@
       </c>
       <c r="H771" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I771" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>BV11cb46tE4x</t>
+        </is>
+      </c>
       <c r="J771" t="inlineStr"/>
     </row>
     <row r="772">
@@ -31431,7 +31443,7 @@
       </c>
       <c r="E775" t="inlineStr">
         <is>
-          <t>2026/01/23，2026/03/29，2026/07/26，2026/07/27</t>
+          <t>2026/01/23，2026/03/29，2026/07/26，2026/07/27，2026/09/11</t>
         </is>
       </c>
       <c r="F775" t="inlineStr"/>
@@ -31442,7 +31454,7 @@
       </c>
       <c r="H775" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I775" t="inlineStr">
@@ -31555,7 +31567,7 @@
       </c>
       <c r="E778" t="inlineStr">
         <is>
-          <t>2026/01/25，2026/08/19</t>
+          <t>2026/01/25，2026/08/19，2026/09/05</t>
         </is>
       </c>
       <c r="F778" t="inlineStr"/>
@@ -31566,7 +31578,7 @@
       </c>
       <c r="H778" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I778" t="inlineStr">
@@ -31639,7 +31651,7 @@
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>2026/01/25，2026/01/30，2026/02/02，2026/02/08，2026/02/19，2026/02/23，2026/02/25，2026/03/12，2026/03/28，2026/04/12，2026/04/20，2026/06/26，2026/07/22，2026/9/4</t>
+          <t>2026/01/25，2026/01/30，2026/02/02，2026/02/08，2026/02/19，2026/02/23，2026/02/25，2026/03/12，2026/03/28，2026/04/12，2026/04/20，2026/06/26，2026/07/22，2026/09/04</t>
         </is>
       </c>
       <c r="F780" t="inlineStr"/>
@@ -31959,7 +31971,7 @@
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>2026/02/08，2026/02/09，2026/02/12，2026/02/14，2026/02/19，2026/02/23，2026/02/24，2026/02/25，2026/03/01，2026/03/05，2026/03/12，2026/03/17，2026/03/19，2026/03/31，2026/04/20，2026/05/02，2026/05/21，2026/06/20，2026/07/16，2026/08/02，2026/9/2</t>
+          <t>2026/02/08，2026/02/09，2026/02/12，2026/02/14，2026/02/19，2026/02/23，2026/02/24，2026/02/25，2026/03/01，2026/03/05，2026/03/12，2026/03/17，2026/03/19，2026/03/31，2026/04/20，2026/05/02，2026/05/21，2026/06/20，2026/07/16，2026/08/02，2026/09/02</t>
         </is>
       </c>
       <c r="F788" t="inlineStr"/>
@@ -32247,7 +32259,7 @@
       </c>
       <c r="E795" t="inlineStr">
         <is>
-          <t>2026/02/19</t>
+          <t>2026/02/19，2026/08/30</t>
         </is>
       </c>
       <c r="F795" t="inlineStr"/>
@@ -32258,7 +32270,7 @@
       </c>
       <c r="H795" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I795" t="inlineStr">
@@ -32367,7 +32379,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>2026/02/22，2026/02/23，2026/02/24，2026/02/25，2026/03/14，2026/04/20，2026/06/16，2026/08/01，2026/8/27</t>
+          <t>2026/02/22，2026/02/23，2026/02/24，2026/02/25，2026/03/14，2026/04/20，2026/06/16，2026/08/01，2026/08/27</t>
         </is>
       </c>
       <c r="F798" t="inlineStr"/>
@@ -32491,7 +32503,7 @@
       </c>
       <c r="E801" t="inlineStr">
         <is>
-          <t>2026/02/25，2026/02/28，2026/03/01，2026/04/20</t>
+          <t>2026/02/25，2026/02/28，2026/03/01，2026/04/20，2026/09/06</t>
         </is>
       </c>
       <c r="F801" t="inlineStr"/>
@@ -32502,7 +32514,7 @@
       </c>
       <c r="H801" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I801" t="inlineStr">
@@ -33039,7 +33051,7 @@
       </c>
       <c r="E814" t="inlineStr">
         <is>
-          <t>2026/03/13，2026/03/14，2026/03/28，2026/04/29，2026/05/25，2026/06/03，2026/06/13，2026/07/02，2026/07/10，2026/07/15，2026/07/22，2026/07/27，2026/07/31，2026/08/11</t>
+          <t>2026/03/13，2026/03/14，2026/03/28，2026/04/29，2026/05/25，2026/06/03，2026/06/13，2026/07/02，2026/07/10，2026/07/15，2026/07/22，2026/07/27，2026/07/31，2026/08/11，2026/08/27，2026/09/11</t>
         </is>
       </c>
       <c r="F814" t="inlineStr"/>
@@ -33050,7 +33062,7 @@
       </c>
       <c r="H814" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I814" t="inlineStr">
@@ -33391,7 +33403,7 @@
       </c>
       <c r="E823" t="inlineStr">
         <is>
-          <t>2026/03/17，2026/03/17，2026/03/25，2026/03/27，2026/03/29，2026/04/02，2026/04/08，2026/04/16，2026/04/20，2026/05/02，2026/05/06，2026/05/26，2026/06/14，2026/07/18，2026/08/08，2026/08/21</t>
+          <t>2026/03/17，2026/03/17，2026/03/25，2026/03/27，2026/03/29，2026/04/02，2026/04/08，2026/04/16，2026/04/20，2026/05/02，2026/05/06，2026/05/26，2026/06/14，2026/07/18，2026/08/08，2026/08/21，2026/09/11</t>
         </is>
       </c>
       <c r="F823" t="inlineStr"/>
@@ -33402,7 +33414,7 @@
       </c>
       <c r="H823" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I823" t="inlineStr">
@@ -33607,7 +33619,7 @@
       </c>
       <c r="E828" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/25，2026/04/01</t>
+          <t>2025/12/24，2025/12/25，2026/04/01，2026/09/13</t>
         </is>
       </c>
       <c r="F828" t="inlineStr"/>
@@ -33618,7 +33630,7 @@
       </c>
       <c r="H828" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I828" t="inlineStr">
@@ -34247,7 +34259,11 @@
           <t>착하다는 말이 제일 싫어</t>
         </is>
       </c>
-      <c r="C844" t="inlineStr"/>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>最讨厌善良这句话</t>
+        </is>
+      </c>
       <c r="D844" t="inlineStr">
         <is>
           <t>YENA</t>
@@ -34255,7 +34271,7 @@
       </c>
       <c r="E844" t="inlineStr">
         <is>
-          <t>2026/04/16，2026/04/29，2026/05/15，2026/05/25，2026/9/2</t>
+          <t>2026/04/16，2026/04/29，2026/05/15，2026/05/25，2026/09/02</t>
         </is>
       </c>
       <c r="F844" t="inlineStr"/>
@@ -34295,7 +34311,7 @@
       </c>
       <c r="E845" t="inlineStr">
         <is>
-          <t>2026/04/17，2026/05/25，2026/05/25，2026/05/26，2026/08/02</t>
+          <t>2026/04/17，2026/05/25，2026/05/25，2026/05/26，2026/08/02，2026/09/06</t>
         </is>
       </c>
       <c r="F845" t="inlineStr"/>
@@ -34306,7 +34322,7 @@
       </c>
       <c r="H845" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I845" t="inlineStr">
@@ -34595,7 +34611,7 @@
       </c>
       <c r="E852" t="inlineStr">
         <is>
-          <t>2026/05/01，2026/07/31，2026/08/01，2026/08/08，2026/08/11，2026/08/25</t>
+          <t>2026/05/01，2026/07/31，2026/08/01，2026/08/08，2026/08/11，2026/08/25，2026/09/11</t>
         </is>
       </c>
       <c r="F852" t="inlineStr"/>
@@ -34606,7 +34622,7 @@
       </c>
       <c r="H852" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I852" t="inlineStr">
@@ -34675,7 +34691,7 @@
       </c>
       <c r="E854" t="inlineStr">
         <is>
-          <t>2026/05/01，2026/08/02，2026/8/30</t>
+          <t>2026/05/01，2026/08/02，2026/08/30</t>
         </is>
       </c>
       <c r="F854" t="inlineStr"/>
@@ -34759,7 +34775,7 @@
       </c>
       <c r="E856" t="inlineStr">
         <is>
-          <t>2026/05/01</t>
+          <t>2026/05/01，2026/09/13</t>
         </is>
       </c>
       <c r="F856" t="inlineStr"/>
@@ -34770,7 +34786,7 @@
       </c>
       <c r="H856" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I856" t="inlineStr">
@@ -34891,7 +34907,7 @@
       </c>
       <c r="E859" t="inlineStr">
         <is>
-          <t>2026/05/25，2026/05/25，2026/05/25，2026/05/26，2026/05/26，2026/06/25，2026/06/26，2026/07/09，2026/07/16，2026/08/23，2026/08/23</t>
+          <t>2026/05/25，2026/05/25，2026/05/25，2026/05/26，2026/05/26，2026/06/25，2026/06/26，2026/07/09，2026/07/16，2026/08/23，2026/08/23，2026/09/11</t>
         </is>
       </c>
       <c r="F859" t="inlineStr"/>
@@ -34902,7 +34918,7 @@
       </c>
       <c r="H859" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I859" t="inlineStr">
@@ -34935,7 +34951,7 @@
       </c>
       <c r="E860" t="inlineStr">
         <is>
-          <t>2026/05/25，2026/05/26，2026/06/15，2026/08/02，2026/9/4</t>
+          <t>2026/05/25，2026/05/26，2026/06/15，2026/08/02</t>
         </is>
       </c>
       <c r="F860" t="inlineStr"/>
@@ -34946,7 +34962,7 @@
       </c>
       <c r="H860" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I860" t="inlineStr">
@@ -35135,7 +35151,7 @@
       </c>
       <c r="E865" t="inlineStr">
         <is>
-          <t>2026/06/14，2026/07/10，2026/07/15，2026/07/27，2026/9/4</t>
+          <t>2026/06/14，2026/07/10，2026/07/15，2026/07/27，2026/09/04</t>
         </is>
       </c>
       <c r="F865" t="inlineStr"/>
@@ -35627,7 +35643,7 @@
       </c>
       <c r="E877" t="inlineStr">
         <is>
-          <t>2026/07/07，2026/07/09，2026/07/10，2026/07/15，2026/07/16，2026/07/18，2026/07/25，2026/07/27，2026/08/01，2026/08/08，2026/08/11，2026/08/18，2026/08/23，2026/08/25，2026/8/28</t>
+          <t>2026/07/07，2026/07/09，2026/07/10，2026/07/15，2026/07/16，2026/07/18，2026/07/25，2026/07/27，2026/08/01，2026/08/08，2026/08/11，2026/08/18，2026/08/23，2026/08/25，2026/08/28，2026/09/02，2026/09/11</t>
         </is>
       </c>
       <c r="F877" t="inlineStr"/>
@@ -35638,7 +35654,7 @@
       </c>
       <c r="H877" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I877" t="inlineStr">
@@ -35751,7 +35767,7 @@
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08，2026/8/28</t>
+          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08，2026/08/28</t>
         </is>
       </c>
       <c r="F880" t="inlineStr"/>
@@ -35791,7 +35807,7 @@
       </c>
       <c r="E881" t="inlineStr">
         <is>
-          <t>2026/07/27，2026/07/30，2026/08/01，2026/08/03，2026/9/2</t>
+          <t>2026/07/27，2026/07/30，2026/08/01，2026/08/03，2026/09/02</t>
         </is>
       </c>
       <c r="F881" t="inlineStr"/>
@@ -35875,7 +35891,7 @@
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>2026/07/27，2026/07/31</t>
+          <t>2026/07/27，2026/07/31，2026/09/13</t>
         </is>
       </c>
       <c r="F883" t="inlineStr"/>
@@ -35886,7 +35902,7 @@
       </c>
       <c r="H883" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I883" t="inlineStr">
@@ -35955,7 +35971,7 @@
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>2026/08/03，2026/08/08，2026/08/09，2026/08/11，2026/08/18，2026/08/25</t>
+          <t>2026/08/03，2026/08/08，2026/08/09，2026/08/11，2026/08/18，2026/08/25，2026/09/08</t>
         </is>
       </c>
       <c r="F885" t="inlineStr"/>
@@ -35966,7 +35982,7 @@
       </c>
       <c r="H885" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I885" t="inlineStr">
@@ -36075,7 +36091,7 @@
       </c>
       <c r="E888" t="inlineStr">
         <is>
-          <t>2026/08/11，2026/08/11，2026/08/18，2026/08/25</t>
+          <t>2026/08/11，2026/08/11，2026/08/18，2026/08/25，2026/09/06，2026/09/11</t>
         </is>
       </c>
       <c r="F888" t="inlineStr"/>
@@ -36086,7 +36102,7 @@
       </c>
       <c r="H888" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I888" t="inlineStr">
@@ -36115,7 +36131,7 @@
       </c>
       <c r="E889" t="inlineStr">
         <is>
-          <t>2026/08/11</t>
+          <t>2026/08/11，2026/09/06</t>
         </is>
       </c>
       <c r="F889" t="inlineStr"/>
@@ -36126,7 +36142,7 @@
       </c>
       <c r="H889" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I889" t="inlineStr">
@@ -36155,7 +36171,7 @@
       </c>
       <c r="E890" t="inlineStr">
         <is>
-          <t>2026/08/18，2026/08/19，2026/08/23，2026/8/30</t>
+          <t>2026/08/18，2026/08/19，2026/08/23，2026/08/30，2026/09/11</t>
         </is>
       </c>
       <c r="F890" t="inlineStr"/>
@@ -36166,7 +36182,7 @@
       </c>
       <c r="H890" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I890" t="inlineStr">
@@ -36399,7 +36415,7 @@
       </c>
       <c r="E896" t="inlineStr">
         <is>
-          <t>2026/08/23，2026/08/25</t>
+          <t>2026/08/23，2026/08/25，2026/09/02，2026/09/11</t>
         </is>
       </c>
       <c r="F896" t="inlineStr"/>
@@ -36410,7 +36426,7 @@
       </c>
       <c r="H896" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I896" t="inlineStr">
@@ -36439,7 +36455,7 @@
       </c>
       <c r="E897" t="inlineStr">
         <is>
-          <t>2026/08/23，2026/9/2</t>
+          <t>2026/08/23</t>
         </is>
       </c>
       <c r="F897" t="inlineStr"/>
@@ -36450,7 +36466,7 @@
       </c>
       <c r="H897" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I897" t="inlineStr">
@@ -36548,18 +36564,18 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>All About That Bass</t>
+          <t>Love Me Like You Do</t>
         </is>
       </c>
       <c r="C900" t="inlineStr"/>
       <c r="D900" t="inlineStr">
         <is>
-          <t>Meghan Trainor</t>
+          <t>Ellie Goulding</t>
         </is>
       </c>
       <c r="E900" t="inlineStr">
         <is>
-          <t>2026/8/30，2026/9/2</t>
+          <t>2026/08/30，2026/09/11</t>
         </is>
       </c>
       <c r="F900" t="inlineStr"/>
@@ -36575,7 +36591,7 @@
       </c>
       <c r="I900" t="inlineStr">
         <is>
-          <t>BV1y4th6AEz2</t>
+          <t>BV1W2tn6zEBJ，BV12wta6uEUK</t>
         </is>
       </c>
       <c r="J900" t="inlineStr"/>
@@ -36588,18 +36604,18 @@
       </c>
       <c r="B901" t="inlineStr">
         <is>
-          <t>Last Friday Night</t>
+          <t>Honeymoon Avenue</t>
         </is>
       </c>
       <c r="C901" t="inlineStr"/>
       <c r="D901" t="inlineStr">
         <is>
-          <t>Katy Perry</t>
+          <t>Ariana Grande</t>
         </is>
       </c>
       <c r="E901" t="inlineStr">
         <is>
-          <t>2026/8/30</t>
+          <t>2026/08/30</t>
         </is>
       </c>
       <c r="F901" t="inlineStr"/>
@@ -36615,7 +36631,7 @@
       </c>
       <c r="I901" t="inlineStr">
         <is>
-          <t>BV12Hth6iEup</t>
+          <t>BV1WhtW67ECn，BV1k8th6cEpk</t>
         </is>
       </c>
       <c r="J901" t="inlineStr"/>
@@ -36639,7 +36655,7 @@
       </c>
       <c r="E902" t="inlineStr">
         <is>
-          <t>2026/8/30，2026/8/30</t>
+          <t>2026/08/30，2026/08/30</t>
         </is>
       </c>
       <c r="F902" t="inlineStr"/>
@@ -36655,7 +36671,7 @@
       </c>
       <c r="I902" t="inlineStr">
         <is>
-          <t>BV1w8th6wERB</t>
+          <t>BV1wvtW6yE7K，BV1w8th6wERB</t>
         </is>
       </c>
       <c r="J902" t="inlineStr"/>
@@ -36668,18 +36684,18 @@
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>Honeymoon Avenue</t>
+          <t>Last Friday Night (T.G.I.F.)</t>
         </is>
       </c>
       <c r="C903" t="inlineStr"/>
       <c r="D903" t="inlineStr">
         <is>
-          <t>Ariana Grande</t>
+          <t>Katy Perry</t>
         </is>
       </c>
       <c r="E903" t="inlineStr">
         <is>
-          <t>2026/8/30</t>
+          <t>2026/08/30</t>
         </is>
       </c>
       <c r="F903" t="inlineStr"/>
@@ -36695,7 +36711,7 @@
       </c>
       <c r="I903" t="inlineStr">
         <is>
-          <t>BV1k8th6cEpk</t>
+          <t>BV12Hth6iEup</t>
         </is>
       </c>
       <c r="J903" t="inlineStr"/>
@@ -36708,18 +36724,18 @@
       </c>
       <c r="B904" t="inlineStr">
         <is>
-          <t>Love Me Like You Do</t>
+          <t>All About That Bass</t>
         </is>
       </c>
       <c r="C904" t="inlineStr"/>
       <c r="D904" t="inlineStr">
         <is>
-          <t>Ellie Goulding</t>
+          <t>Meghan Trainor</t>
         </is>
       </c>
       <c r="E904" t="inlineStr">
         <is>
-          <t>2026/8/30</t>
+          <t>2026/08/30，2026/09/02</t>
         </is>
       </c>
       <c r="F904" t="inlineStr"/>
@@ -36730,12 +36746,12 @@
       </c>
       <c r="H904" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I904" t="inlineStr">
         <is>
-          <t>BV12wta6uEUK</t>
+          <t>BV14Hth6qEwH，BV1y4th6AEz2</t>
         </is>
       </c>
       <c r="J904" t="inlineStr"/>
@@ -36751,7 +36767,11 @@
           <t>California King Bed</t>
         </is>
       </c>
-      <c r="C905" t="inlineStr"/>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>加州王床</t>
+        </is>
+      </c>
       <c r="D905" t="inlineStr">
         <is>
           <t>Rihanna</t>
@@ -36759,7 +36779,7 @@
       </c>
       <c r="E905" t="inlineStr">
         <is>
-          <t>2026/9/2</t>
+          <t>2026/09/02</t>
         </is>
       </c>
       <c r="F905" t="inlineStr"/>
@@ -36775,7 +36795,7 @@
       </c>
       <c r="I905" t="inlineStr">
         <is>
-          <t>BV15eto6sEMB</t>
+          <t>BV1oetS6gEcN，BV15eto6sEMB</t>
         </is>
       </c>
       <c r="J905" t="inlineStr"/>
@@ -36788,37 +36808,153 @@
       </c>
       <c r="B906" t="inlineStr">
         <is>
-          <t>willow</t>
+          <t>社畜少女</t>
         </is>
       </c>
       <c r="C906" t="inlineStr"/>
       <c r="D906" t="inlineStr">
         <is>
-          <t>Taylor Swift</t>
+          <t>ChiliChill</t>
         </is>
       </c>
       <c r="E906" t="inlineStr">
         <is>
-          <t>2026/9/4</t>
+          <t>2026/09/11</t>
         </is>
       </c>
       <c r="F906" t="inlineStr"/>
       <c r="G906" t="inlineStr">
         <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>BV1cJY26QEG7</t>
+        </is>
+      </c>
+      <c r="J906" t="inlineStr"/>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>906</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>还是会寂寞</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr"/>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>陈绮贞</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>2026/09/06，2026/09/11</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr"/>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I907" t="inlineStr"/>
+      <c r="J907" t="inlineStr"/>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>907</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>粛聖!! ロリ神レクイエム</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>肃静！萝莉神的镇魂曲</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>しぐれうい</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>2026/09/13</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr"/>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>日语</t>
+        </is>
+      </c>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I908" t="inlineStr"/>
+      <c r="J908" t="inlineStr"/>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>908</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>willow</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr"/>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>2026/09/04</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr"/>
+      <c r="G909" t="inlineStr">
+        <is>
           <t>英语</t>
         </is>
       </c>
-      <c r="H906" t="inlineStr">
+      <c r="H909" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I906" t="inlineStr">
+      <c r="I909" t="inlineStr">
         <is>
           <t>BV1Setr6MEBW</t>
         </is>
       </c>
-      <c r="J906" t="inlineStr"/>
+      <c r="J909" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Sep.14, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J909"/>
+  <dimension ref="A1:J910"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/09，2025/05/29，2025/06/28，2025/08/08，2025/08/21，2025/09/15，2025/10/24，2025/12/17，2026/01/15，2026/02/14，2026/03/04，2026/04/09，2026/08/25</t>
+          <t>2025/03/04，2025/05/09，2025/05/29，2025/06/28，2025/08/08，2025/08/21，2025/09/15，2025/10/24，2025/12/17，2026/01/15，2026/02/14，2026/03/04，2026/04/09，2026/08/25，2026/9/14</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/18，2025/04/28，2025/08/22，2025/09/17，2025/10/30，2025/11/09，2025/11/14，2025/11/26，2026/01/25，2026/07/17</t>
+          <t>2025/03/04，2025/04/18，2025/04/28，2025/08/22，2025/09/17，2025/10/30，2025/11/09，2025/11/14，2025/11/26，2026/01/25，2026/07/17，2026/9/14</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/07，2025/12/16，2025/12/28，2026/01/10，2026/01/15，2026/02/19，2026/03/07，2026/03/17，2026/03/21，2026/05/06，2026/07/05，2026/07/20，2026/08/30</t>
+          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/07，2025/12/16，2025/12/28，2026/01/10，2026/01/15，2026/02/19，2026/03/07，2026/03/17，2026/03/21，2026/05/06，2026/07/05，2026/07/20，2026/08/30，2026/9/14</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/04/09，2026/05/10，2026/06/12，2026/07/27，2026/08/28</t>
+          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/04/09，2026/05/10，2026/06/12，2026/07/27，2026/08/28，2026/9/14</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/06/05，2025/07/05，2025/08/22，2026/04/26，2026/09/04</t>
+          <t>2025/03/10，2025/06/05，2025/07/05，2025/08/22，2026/04/26，2026/09/04，2026/9/14</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/11，2025/05/04，2025/05/18，2025/06/06，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/09/18，2025/10/05，2025/12/02，2026/02/09</t>
+          <t>2025/03/12，2025/04/11，2025/05/04，2025/05/18，2025/06/06，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/09/18，2025/10/05，2025/12/02，2026/02/09，2026/9/14</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -3790,7 +3790,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/06/06，2025/06/27，2025/08/01，2025/11/09，2025/11/14，2026/06/12</t>
+          <t>2025/03/14，2025/06/06，2025/06/27，2025/08/01，2025/11/09，2025/11/14，2026/06/12，2026/9/14</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -4974,7 +4974,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -5687,7 +5687,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2025/03/16，2025/04/17，2025/05/08，2025/09/11，2025/10/03，2025/10/16，2025/11/19，2026/02/07，2026/06/23，2026/08/18</t>
+          <t>2025/03/16，2025/04/17，2025/05/08，2025/09/11，2025/10/03，2025/10/16，2025/11/19，2026/02/07，2026/06/23，2026/08/18，2026/9/14，2026/9/14</t>
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -5698,7 +5698,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/14，2025/05/12，2025/06/07，2025/07/06，2025/07/21，2025/09/14，2025/10/31，2025/11/09，2026/01/09，2026/05/04，2026/07/27</t>
+          <t>2025/03/21，2025/04/14，2025/05/12，2025/06/07，2025/07/06，2025/07/21，2025/09/14，2025/10/31，2025/11/09，2026/01/09，2026/05/04，2026/07/27，2026/9/14</t>
         </is>
       </c>
       <c r="F171" t="inlineStr"/>
@@ -7382,7 +7382,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -7527,7 +7527,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11，2026/08/28</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11，2026/08/28，2026/9/14</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7538,7 +7538,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -8575,7 +8575,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/03/25，2026/06/23，2026/08/21</t>
+          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/03/25，2026/06/23，2026/08/21，2026/9/14</t>
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -10023,7 +10023,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/25，2025/05/03，2025/06/23，2025/09/28，2025/11/28，2025/12/26，2026/06/28，2026/08/27</t>
+          <t>2025/03/29，2025/04/25，2025/05/03，2025/06/23，2025/09/28，2025/11/28，2025/12/26，2026/06/28，2026/08/27，2026/9/14</t>
         </is>
       </c>
       <c r="F237" t="inlineStr"/>
@@ -10034,7 +10034,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -11471,7 +11471,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08，2026/08/28</t>
+          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08，2026/08/28，2026/9/14，2026/9/14</t>
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
@@ -11482,7 +11482,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -12307,7 +12307,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/02/14，2026/03/05，2026/04/02，2026/05/20，2026/08/28</t>
+          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/02/14，2026/03/05，2026/04/02，2026/05/20，2026/08/28，2026/9/14</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -12318,7 +12318,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -12347,7 +12347,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/19，2025/05/20，2025/07/11，2025/09/12，2025/12/09，2025/12/16，2026/02/27，2026/06/13</t>
+          <t>2025/04/05，2025/04/19，2025/05/20，2025/07/11，2025/09/12，2025/12/09，2025/12/16，2026/02/27，2026/06/13，2026/9/14</t>
         </is>
       </c>
       <c r="F295" t="inlineStr"/>
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -12751,7 +12751,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23，2026/08/30，2026/09/11</t>
+          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23，2026/08/30，2026/09/11，2026/9/14，2026/9/14</t>
         </is>
       </c>
       <c r="F305" t="inlineStr"/>
@@ -12762,7 +12762,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -14483,7 +14483,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/25，2025/05/30，2025/06/17，2025/09/26，2025/10/03，2025/11/03，2025/12/23，2026/04/09</t>
+          <t>2025/04/15，2025/04/25，2025/05/30，2025/06/17，2025/09/26，2025/10/03，2025/11/03，2025/12/23，2026/04/09，2026/9/14</t>
         </is>
       </c>
       <c r="F348" t="inlineStr"/>
@@ -14494,7 +14494,7 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
@@ -16471,7 +16471,7 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/23，2025/10/09，2026/01/22，2026/03/09</t>
+          <t>2025/04/25，2025/06/23，2025/10/09，2026/01/22，2026/03/09，2026/9/14</t>
         </is>
       </c>
       <c r="F398" t="inlineStr"/>
@@ -16482,7 +16482,7 @@
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
@@ -16551,7 +16551,7 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/06/02，2025/06/09，2025/07/09，2025/07/14，2025/08/26，2025/11/21，2025/12/17，2026/01/09，2026/04/09</t>
+          <t>2025/04/27，2025/06/02，2025/06/09，2025/07/09，2025/07/14，2025/08/26，2025/11/21，2025/12/17，2026/01/09，2026/04/09，2026/9/14</t>
         </is>
       </c>
       <c r="F400" t="inlineStr"/>
@@ -16562,7 +16562,7 @@
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
@@ -17351,7 +17351,7 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>2025/05/03，2026/08/27</t>
+          <t>2025/05/03，2026/08/27，2026/9/14，2026/9/14</t>
         </is>
       </c>
       <c r="F420" t="inlineStr"/>
@@ -17362,7 +17362,7 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
@@ -18835,7 +18835,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/07/21，2026/04/14，2026/06/19</t>
+          <t>2025/05/22，2025/07/21，2026/04/14，2026/06/19，2026/9/14，2026/9/14</t>
         </is>
       </c>
       <c r="F457" t="inlineStr"/>
@@ -18846,7 +18846,7 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">
@@ -24655,7 +24655,7 @@
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>2025/07/26，2025/08/08，2026/07/22</t>
+          <t>2025/07/26，2025/08/08，2026/07/22，2026/9/14，2026/9/14</t>
         </is>
       </c>
       <c r="F602" t="inlineStr"/>
@@ -24666,7 +24666,7 @@
       </c>
       <c r="H602" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I602" t="inlineStr">
@@ -31931,7 +31931,7 @@
       </c>
       <c r="E787" t="inlineStr">
         <is>
-          <t>2026/02/08，2026/02/09，2026/02/14，2026/02/20，2026/02/28，2026/05/25，2026/06/13，2026/07/05，2026/07/18，2026/08/08，2026/08/23</t>
+          <t>2026/02/08，2026/02/09，2026/02/14，2026/02/20，2026/02/28，2026/05/25，2026/06/13，2026/07/05，2026/07/18，2026/08/08，2026/08/23，2026/9/14，2026/9/14</t>
         </is>
       </c>
       <c r="F787" t="inlineStr"/>
@@ -31942,7 +31942,7 @@
       </c>
       <c r="H787" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I787" t="inlineStr">
@@ -32587,7 +32587,7 @@
       </c>
       <c r="E803" t="inlineStr">
         <is>
-          <t>2026/03/01，2026/03/01，2026/03/01，2026/03/01，2026/03/01，2026/03/04，2026/03/05，2026/03/05，2026/03/06，2026/03/12，2026/03/21，2026/03/31，2026/04/20，2026/05/02，2026/05/06，2026/05/21，2026/05/26，2026/06/14，2026/07/16</t>
+          <t>2026/03/01，2026/03/01，2026/03/01，2026/03/01，2026/03/01，2026/03/04，2026/03/05，2026/03/05，2026/03/06，2026/03/12，2026/03/21，2026/03/31，2026/04/20，2026/05/02，2026/05/06，2026/05/21，2026/05/26，2026/06/14，2026/07/16，2026/9/14，2026/9/14</t>
         </is>
       </c>
       <c r="F803" t="inlineStr"/>
@@ -32598,7 +32598,7 @@
       </c>
       <c r="H803" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I803" t="inlineStr">
@@ -35767,7 +35767,7 @@
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08，2026/08/28</t>
+          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08，2026/08/28，2026/9/14</t>
         </is>
       </c>
       <c r="F880" t="inlineStr"/>
@@ -35778,7 +35778,7 @@
       </c>
       <c r="H880" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I880" t="inlineStr">
@@ -36091,7 +36091,7 @@
       </c>
       <c r="E888" t="inlineStr">
         <is>
-          <t>2026/08/11，2026/08/11，2026/08/18，2026/08/25，2026/09/06，2026/09/11</t>
+          <t>2026/08/11，2026/08/11，2026/08/18，2026/08/25，2026/09/06，2026/09/11，2026/9/14</t>
         </is>
       </c>
       <c r="F888" t="inlineStr"/>
@@ -36102,7 +36102,7 @@
       </c>
       <c r="H888" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I888" t="inlineStr">
@@ -36873,7 +36873,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I907" t="inlineStr"/>
+      <c r="I907" t="inlineStr">
+        <is>
+          <t>BV13fY16KELD</t>
+        </is>
+      </c>
       <c r="J907" t="inlineStr"/>
     </row>
     <row r="908">
@@ -36913,7 +36917,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I908" t="inlineStr"/>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>BV1FwY16LEko</t>
+        </is>
+      </c>
       <c r="J908" t="inlineStr"/>
     </row>
     <row r="909">
@@ -36955,6 +36963,46 @@
         </is>
       </c>
       <c r="J909" t="inlineStr"/>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>909</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Better Dig Two</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr"/>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>The Band Perry</t>
+        </is>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>2026/09/14</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr"/>
+      <c r="G910" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I910" t="inlineStr">
+        <is>
+          <t>BV1Pjen6QEeh</t>
+        </is>
+      </c>
+      <c r="J910" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Update song list to Sep 26, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J910"/>
+  <dimension ref="A1:J915"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,7 +487,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/04/01，2025/04/17，2025/04/29，2025/05/30，2025/08/02，2025/08/21，2025/09/18，2025/09/19，2025/09/28，2025/10/16，2025/11/14，2025/12/12，2026/01/23，2026/03/01，2026/03/22，2026/03/27，2026/06/28，2026/07/22</t>
+          <t>2025/03/01，2025/04/01，2025/04/17，2025/04/29，2025/05/30，2025/08/02，2025/08/21，2025/09/18，2025/09/19，2025/09/28，2025/10/16，2025/11/14，2025/12/12，2026/01/23，2026/03/01，2026/03/22，2026/03/27，2026/06/28，2026/07/22，2026/09/23</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -498,7 +498,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/07，2025/12/17，2026/01/19，2026/01/29，2026/02/10，2026/02/12，2026/03/22，2026/04/18，2026/05/10，2026/06/06，2026/06/25，2026/07/17，2026/08/28，2026/09/04，2026/09/06</t>
+          <t>2025/03/04，2025/03/19，2025/04/14，2025/04/22，2025/05/01，2025/05/13，2025/05/19，2025/05/27，2025/06/03，2025/06/12，2025/06/19，2025/06/27，2025/07/08，2025/07/14，2025/07/18，2025/07/20，2025/08/02，2025/08/08，2025/08/12，2025/09/02，2025/09/18，2025/10/01，2025/10/03，2025/10/11，2025/10/24，2025/11/13，2025/11/14，2025/11/28，2025/12/07，2025/12/17，2026/01/19，2026/01/29，2026/02/10，2026/02/12，2026/03/22，2026/04/18，2026/05/10，2026/06/06，2026/06/25，2026/07/17，2026/08/28，2026/09/04，2026/09/06，2026/09/23</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/01/10，2026/01/24，2026/04/09，2026/05/21，2026/07/17，2026/09/06</t>
+          <t>2025/03/04，2025/04/04，2025/04/18，2025/05/25，2025/05/26，2025/06/06，2025/06/13，2025/09/04，2025/09/17，2025/10/09，2025/10/28，2026/01/10，2026/01/24，2026/04/09，2026/05/21，2026/07/17，2026/09/06，2026/09/23</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/01/09，2026/02/12，2026/03/09，2026/03/15，2026/05/01，2026/05/16，2026/05/23，2026/07/05，2026/07/28，2026/08/30，2026/09/04</t>
+          <t>2025/03/04，2025/04/02，2025/04/17，2025/04/29，2025/05/12，2025/05/27，2025/06/10，2025/07/05，2025/08/10，2025/08/28，2025/09/05，2025/09/18，2025/11/12，2025/11/28，2026/01/09，2026/02/12，2026/03/09，2026/03/15，2026/05/01，2026/05/16，2026/05/23，2026/07/05，2026/07/28，2026/08/30，2026/09/04，2026/09/22</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/18，2025/05/23，2025/07/24，2025/08/28，2025/09/05，2026/03/09，2026/04/18，2026/05/23</t>
+          <t>2025/03/04，2025/04/18，2025/05/23，2025/07/24，2025/08/28，2025/09/05，2026/03/09，2026/04/18，2026/05/23，2026/09/17</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/09，2025/12/16，2026/02/14，2026/03/07，2026/03/17，2026/03/21，2026/05/01，2026/07/04，2026/07/26，2026/08/28</t>
+          <t>2025/03/04，2025/04/14，2025/04/24，2025/05/19，2025/08/21，2025/09/06，2025/09/17，2025/09/26，2025/10/01，2025/11/09，2025/12/16，2026/02/14，2026/03/07，2026/03/17，2026/03/21，2026/05/01，2026/07/04，2026/07/26，2026/08/28，2026/09/17</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/05/09，2025/05/29，2025/06/28，2025/08/08，2025/08/21，2025/09/15，2025/10/24，2025/12/17，2026/01/15，2026/02/14，2026/03/04，2026/04/09，2026/08/25，2026/9/14</t>
+          <t>2025/03/04，2025/05/09，2025/05/29，2025/06/28，2025/08/08，2025/08/21，2025/09/15，2025/10/24，2025/12/17，2026/01/15，2026/02/14，2026/03/04，2026/04/09，2026/08/25，2026/09/14，2026/09/22</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/01/03，2026/03/25，2026/05/10，2026/06/20，2026/08/16</t>
+          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/01/03，2026/03/25，2026/05/10，2026/06/20，2026/08/16，2026/09/23</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/09，2025/12/30，2026/02/20，2026/02/23，2026/03/04，2026/04/11，2026/04/16，2026/04/23，2026/06/14，2026/07/04，2026/07/31，2026/08/25</t>
+          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/09，2025/12/30，2026/02/20，2026/02/23，2026/03/04，2026/04/11，2026/04/16，2026/04/23，2026/06/14，2026/07/04，2026/07/31，2026/08/25，2026/09/26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/01，2025/11/28，2025/12/12，2026/01/05，2026/01/22，2026/03/04，2026/03/08，2026/03/22，2026/04/22，2026/04/24，2026/05/10，2026/05/23，2026/06/10，2026/06/15，2026/07/31，2026/08/11，2026/08/25</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/01，2025/11/28，2025/12/12，2026/01/05，2026/01/22，2026/03/04，2026/03/08，2026/03/22，2026/04/22，2026/04/24，2026/05/10，2026/05/23，2026/06/10，2026/06/15，2026/07/31，2026/08/11，2026/08/25，2026/09/21</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/03/15，2026/06/23，2026/08/30，2026/08/30</t>
+          <t>2025/03/04，2025/04/22，2025/05/18，2025/09/04，2025/09/10，2025/11/28，2026/03/15，2026/06/23，2026/08/30，2026/08/30，2026/09/23</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/18，2025/04/28，2025/08/22，2025/09/17，2025/10/30，2025/11/09，2025/11/14，2025/11/26，2026/01/25，2026/07/17，2026/9/14</t>
+          <t>2025/03/04，2025/04/18，2025/04/28，2025/08/22，2025/09/17，2025/10/30，2025/11/09，2025/11/14，2025/11/26，2026/01/25，2026/07/17，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/01/14，2026/02/19，2026/03/14，2026/04/16，2026/06/17，2026/07/16，2026/07/22，2026/08/11</t>
+          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/01/14，2026/02/19，2026/03/14，2026/04/16，2026/06/17，2026/07/16，2026/07/22，2026/08/11，2026/09/21</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/07，2025/11/09，2025/12/02，2026/01/21，2026/03/05，2026/04/16，2026/06/23，2026/07/05，2026/08/05，2026/08/05，2026/08/19，2026/09/05</t>
+          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/07，2025/11/09，2025/12/02，2026/01/21，2026/03/05，2026/04/16，2026/06/23，2026/07/05，2026/08/05，2026/08/05，2026/08/19，2026/09/05，2026/09/19</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2254,7 +2254,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/17，2025/05/18，2025/05/30，2025/06/06，2025/06/21，2025/06/27，2025/07/24，2025/08/24，2025/09/10，2025/09/30，2025/10/23，2025/11/10，2026/01/15，2026/02/14，2026/03/22，2026/05/20，2026/09/13</t>
+          <t>2025/03/06，2025/04/17，2025/05/18，2025/05/30，2025/06/06，2025/06/21，2025/06/27，2025/07/24，2025/08/24，2025/09/10，2025/09/30，2025/10/23，2025/11/10，2026/01/15，2026/02/14，2026/03/22，2026/05/20，2026/09/13，2026/09/23</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/06，2025/04/13，2025/04/22，2025/05/08，2025/05/09，2025/05/30，2025/06/08，2025/08/04，2025/09/18，2025/10/12，2025/11/21，2026/01/24，2026/02/14，2026/02/25，2026/04/10，2026/04/25</t>
+          <t>2025/03/06，2025/04/06，2025/04/13，2025/04/22，2025/05/08，2025/05/09，2025/05/30，2025/06/08，2025/08/04，2025/09/18，2025/10/12，2025/11/21，2026/01/24，2026/02/14，2026/02/25，2026/04/10，2026/04/25，2026/09/23</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/03，2025/12/12，2026/02/04，2026/04/18，2026/05/20，2026/06/20，2026/07/30，2026/08/09</t>
+          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/03，2025/12/12，2026/02/04，2026/04/18，2026/05/20，2026/06/20，2026/07/30，2026/08/09，2026/09/22</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/04，2025/04/19，2025/06/02，2025/06/17，2025/06/23，2025/07/20，2025/09/24，2025/10/09，2026/02/17，2026/03/07，2026/05/24</t>
+          <t>2025/03/07，2025/04/04，2025/04/19，2025/06/02，2025/06/17，2025/06/23，2025/07/20，2025/09/24，2025/10/09，2026/02/17，2026/03/07，2026/05/24，2026/09/16</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/27，2025/04/07，2025/04/12，2025/04/22，2025/04/26，2025/05/05，2025/05/19，2025/06/03，2025/06/09，2025/07/18，2025/07/22，2025/09/10，2025/09/19，2025/10/16，2025/12/24，2026/06/20，2026/08/27</t>
+          <t>2025/03/07，2025/03/27，2025/04/07，2025/04/12，2025/04/22，2025/04/26，2025/05/05，2025/05/19，2025/06/03，2025/06/09，2025/07/18，2025/07/22，2025/09/10，2025/09/19，2025/10/16，2025/12/24，2026/06/20，2026/08/27，2026/09/21</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/07，2025/12/16，2025/12/28，2026/01/10，2026/01/15，2026/02/19，2026/03/07，2026/03/17，2026/03/21，2026/05/06，2026/07/05，2026/07/20，2026/08/30，2026/9/14</t>
+          <t>2025/03/07，2025/04/20，2025/04/25，2025/05/18，2025/05/26，2025/06/02，2025/06/27，2025/07/07，2025/08/03，2025/09/14，2025/09/17，2025/10/03，2025/10/07，2025/12/07，2025/12/16，2025/12/28，2026/01/10，2026/01/15，2026/02/19，2026/03/07，2026/03/17，2026/03/21，2026/05/06，2026/07/05，2026/07/20，2026/08/30，2026/09/14</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/07，2025/11/19，2025/11/26，2025/12/30，2026/01/28，2026/02/14，2026/03/13，2026/04/10，2026/05/23，2026/06/18，2026/06/29，2026/07/25，2026/08/25，2026/09/06</t>
+          <t>2025/03/07，2025/04/06，2025/04/11，2025/04/18，2025/05/08，2025/05/25，2025/06/12，2025/07/03，2025/07/09，2025/07/29，2025/08/23，2025/09/13，2025/09/22，2025/09/26，2025/09/30，2025/10/23，2025/10/31，2025/11/07，2025/11/19，2025/11/26，2025/12/30，2026/01/28，2026/02/14，2026/03/13，2026/04/10，2026/05/23，2026/06/18，2026/06/29，2026/07/25，2026/08/25，2026/09/06，2026/09/19</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/14，2025/05/05，2025/05/19，2025/05/23，2025/06/13，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/12/02，2025/12/26，2026/05/04，2026/06/28，2026/09/06</t>
+          <t>2025/03/07，2025/04/14，2025/05/05，2025/05/19，2025/05/23，2025/06/13，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/12/02，2025/12/26，2026/05/04，2026/06/28，2026/09/06，2026/09/22</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
@@ -3006,7 +3006,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/04/09，2026/05/10，2026/06/12，2026/07/27，2026/08/28，2026/9/14</t>
+          <t>2025/03/09，2025/03/21，2025/04/11，2025/04/15，2025/04/29，2025/05/08，2025/05/16，2025/05/22，2025/05/30，2025/06/06，2025/06/13，2025/06/30，2025/07/21，2025/09/19，2025/11/14，2025/11/22，2026/04/09，2026/05/10，2026/06/12，2026/07/27，2026/08/28，2026/09/14</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/06，2025/05/08，2025/05/24，2025/06/06，2025/07/05，2025/07/24，2025/08/04，2025/09/08，2025/09/19，2025/10/16，2025/10/28，2025/11/13，2025/12/16，2025/12/30，2026/02/19，2026/04/14，2026/06/12，2026/06/14</t>
+          <t>2025/03/09，2025/04/06，2025/05/08，2025/05/24，2025/06/06，2025/07/05，2025/07/24，2025/08/04，2025/09/08，2025/09/19，2025/10/16，2025/10/28，2025/11/13，2025/12/16，2025/12/30，2026/02/19，2026/04/14，2026/06/12，2026/06/14，2026/09/21</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -3294,7 +3294,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/04/04，2025/04/28，2025/07/08，2025/07/21，2025/08/18，2026/02/09，2026/04/08，2026/08/21</t>
+          <t>2025/03/09，2025/04/04，2025/04/28，2025/07/08，2025/07/21，2025/08/18，2026/02/09，2026/04/08，2026/08/21，2026/09/16，2026/09/22</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/06/05，2025/07/05，2025/08/22，2026/04/26，2026/09/04，2026/9/14</t>
+          <t>2025/03/10，2025/06/05，2025/07/05，2025/08/22，2026/04/26，2026/09/04，2026/09/14，2026/09/23</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/11，2025/05/04，2025/05/18，2025/06/06，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/09/18，2025/10/05，2025/12/02，2026/02/09，2026/9/14</t>
+          <t>2025/03/12，2025/04/11，2025/05/04，2025/05/18，2025/06/06，2025/06/27，2025/07/15，2025/08/16，2025/09/11，2025/09/18，2025/10/05，2025/12/02，2026/02/09，2026/09/14</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/05/10，2025/05/24，2025/06/20，2025/07/13，2025/08/23，2025/09/05，2025/09/18，2025/09/30，2025/11/27，2026/02/07</t>
+          <t>2025/03/13，2025/05/10，2025/05/24，2025/06/20，2025/07/13，2025/08/23，2025/09/05，2025/09/18，2025/09/30，2025/11/27，2026/02/07，2026/09/23</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/09，2026/01/23，2026/02/18，2026/04/09，2026/06/15，2026/07/22，2026/08/28</t>
+          <t>2025/03/13，2025/03/28，2025/04/11，2025/04/25，2025/05/15，2025/05/29，2025/06/20，2025/07/13，2025/09/19，2025/10/05，2025/10/23，2025/11/09，2026/01/23，2026/02/18，2026/04/09，2026/06/15，2026/07/22，2026/08/28，2026/09/23</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/09，2026/03/25，2026/04/26，2026/06/15，2026/08/25</t>
+          <t>2025/03/14，2025/03/14，2025/04/14，2025/05/26，2025/06/02，2025/06/12，2025/06/23，2025/07/06，2025/07/10，2025/07/25，2025/08/23，2025/09/20，2025/11/09，2026/03/25，2026/04/26，2026/06/15，2026/08/25，2026/09/21，2026/09/22</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -4606,7 +4606,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/17，2025/04/25，2025/06/23，2025/08/30，2025/09/12，2025/09/15，2025/11/19，2026/02/08，2026/04/09，2026/07/16</t>
+          <t>2025/03/14，2025/04/17，2025/04/25，2025/06/23，2025/08/30，2025/09/12，2025/09/15，2025/11/19，2026/02/08，2026/04/09，2026/07/16，2026/09/21</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -4795,7 +4795,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/25，2025/06/26，2025/07/05，2025/09/05</t>
+          <t>2025/03/14，2025/03/25，2025/06/26，2025/07/05，2025/09/05，2026/09/21</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -4919,7 +4919,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/19，2025/07/21，2025/10/20，2025/11/09，2026/01/14，2026/02/19，2026/04/19，2026/06/03</t>
+          <t>2025/03/14，2025/05/19，2025/07/21，2025/10/20，2025/11/09，2026/01/14，2026/02/19，2026/04/19，2026/06/03，2026/09/26</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -4930,7 +4930,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/06/06，2025/06/27，2025/08/01，2025/11/09，2025/11/14，2026/06/12，2026/9/14</t>
+          <t>2025/03/14，2025/06/06，2025/06/27，2025/08/01，2025/11/09，2025/11/14，2026/06/12，2026/09/14，2026/09/22</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -4974,7 +4974,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/20，2025/07/23，2025/11/28，2025/12/09，2026/07/31</t>
+          <t>2025/03/14，2025/05/20，2025/07/23，2025/11/28，2025/12/09，2026/07/31，2026/09/16</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -5058,7 +5058,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/12，2025/05/20，2025/05/30，2025/06/27，2025/08/13，2025/09/11，2025/10/28，2025/12/20，2026/01/16，2026/04/17，2026/08/08</t>
+          <t>2025/03/14，2025/04/12，2025/05/20，2025/05/30，2025/06/27，2025/08/13，2025/09/11，2025/10/28，2025/12/20，2026/01/16，2026/04/17，2026/08/08，2026/09/22</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/04/05，2025/05/15，2025/08/12，2026/03/28，2026/09/06</t>
+          <t>2025/03/15，2025/04/05，2025/05/15，2025/08/12，2026/03/28，2026/09/06，2026/09/22</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -5687,7 +5687,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2025/03/16，2025/04/17，2025/05/08，2025/09/11，2025/10/03，2025/10/16，2025/11/19，2026/02/07，2026/06/23，2026/08/18，2026/9/14，2026/9/14</t>
+          <t>2025/03/16，2025/04/17，2025/05/08，2025/09/11，2025/10/03，2025/10/16，2025/11/19，2026/02/07，2026/06/23，2026/08/18，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -5727,7 +5727,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/07，2025/12/23，2026/01/05，2026/01/21，2026/01/29，2026/02/09，2026/02/20，2026/02/23，2026/03/04，2026/03/06，2026/03/07，2026/04/11，2026/04/14，2026/04/29，2026/05/23，2026/07/03，2026/07/21，2026/08/11，2026/08/25，2026/09/06</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/07，2025/12/23，2026/01/05，2026/01/21，2026/01/29，2026/02/09，2026/02/20，2026/02/23，2026/03/04，2026/03/06，2026/03/07，2026/04/11，2026/04/14，2026/04/29，2026/05/23，2026/07/03，2026/07/21，2026/08/11，2026/08/25，2026/09/06，2026/09/23</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5738,7 +5738,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -5887,7 +5887,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/17，2025/05/13，2025/05/23，2025/07/21，2025/07/29，2025/08/07，2025/09/30，2025/10/31，2025/12/09，2026/01/12，2026/04/26，2026/07/09，2026/08/02</t>
+          <t>2025/03/17，2025/04/17，2025/05/13，2025/05/23，2025/07/21，2025/07/29，2025/08/07，2025/09/30，2025/10/31，2025/12/09，2026/01/12，2026/04/26，2026/07/09，2026/08/02，2026/09/17</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
@@ -5898,7 +5898,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/01/03，2026/01/05，2026/01/30，2026/03/14，2026/03/31，2026/04/20，2026/05/01，2026/06/19，2026/06/30，2026/07/18，2026/08/03</t>
+          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/01/03，2026/01/05，2026/01/30，2026/03/14，2026/03/31，2026/04/20，2026/05/01，2026/06/19，2026/06/30，2026/07/18，2026/08/03，2026/09/26</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -6178,7 +6178,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/04，2026/01/03，2026/02/10，2026/03/13，2026/03/22，2026/04/14，2026/06/17，2026/08/25，2026/09/06</t>
+          <t>2025/03/19，2025/04/07，2025/04/17，2025/04/22，2025/05/22，2025/06/23，2025/07/09，2025/08/26，2025/09/28，2025/11/21，2025/12/04，2026/01/03，2026/02/10，2026/03/13，2026/03/22，2026/04/14，2026/06/17，2026/08/25，2026/09/06，2026/09/21</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/01/01，2026/01/09，2026/03/22，2026/04/09，2026/04/20，2026/05/25，2026/06/10，2026/06/19，2026/08/11，2026/08/28，2026/08/28</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/01/01，2026/01/09，2026/03/22，2026/04/09，2026/04/20，2026/05/25，2026/06/10，2026/06/19，2026/08/11，2026/08/28，2026/08/28，2026/09/26</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/08，2025/12/24，2026/01/28，2026/04/22，2026/05/05，2026/06/14，2026/07/22，2026/07/31</t>
+          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/08，2025/12/24，2026/01/28，2026/04/22，2026/05/05，2026/06/14，2026/07/22，2026/07/31，2026/09/22</t>
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/05/22，2025/05/29，2025/06/03，2025/08/28，2025/09/11，2025/10/18，2025/10/30，2025/11/28，2025/12/28，2026/03/15，2026/05/19，2026/07/13</t>
+          <t>2025/03/20，2025/05/22，2025/05/29，2025/06/03，2025/08/28，2025/09/11，2025/10/18，2025/10/30，2025/11/28，2025/12/28，2026/03/15，2026/05/19，2026/07/13，2026/09/16</t>
         </is>
       </c>
       <c r="F156" t="inlineStr"/>
@@ -6782,7 +6782,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -6811,7 +6811,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/16，2025/08/26，2025/09/21，2025/10/03，2025/11/12，2025/12/08，2026/01/23，2026/01/26，2026/02/07，2026/02/10，2026/02/23，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/13，2026/03/24，2026/03/28，2026/03/29，2026/04/27，2026/05/02，2026/06/18，2026/07/04，2026/07/31，2026/08/25，2026/08/28，2026/09/06</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/16，2025/08/26，2025/09/21，2025/10/03，2025/11/12，2025/12/08，2026/01/23，2026/01/26，2026/02/07，2026/02/10，2026/02/23，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/13，2026/03/24，2026/03/28，2026/03/29，2026/04/27，2026/05/02，2026/06/18，2026/07/04，2026/07/31，2026/08/25，2026/08/28，2026/09/06，2026/09/21</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/17，2025/05/01，2025/05/03，2025/05/18，2025/05/22，2025/05/29，2025/06/06，2025/06/13，2025/06/30，2025/07/09，2025/07/27，2025/08/23，2025/09/03，2025/09/11，2025/10/11，2025/10/17，2025/12/24，2026/01/16，2026/02/07，2026/03/28，2026/08/16</t>
+          <t>2025/03/20，2025/04/17，2025/05/01，2025/05/03，2025/05/18，2025/05/22，2025/05/29，2025/06/06，2025/06/13，2025/06/30，2025/07/09，2025/07/27，2025/08/23，2025/09/03，2025/09/11，2025/10/11，2025/10/17，2025/12/24，2026/01/16，2026/02/07，2026/03/28，2026/08/16，2026/09/16</t>
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -6986,7 +6986,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/08，2025/12/26，2026/01/05，2026/01/24，2026/02/05，2026/02/14，2026/03/09，2026/03/28，2026/04/26，2026/05/05，2026/05/23，2026/06/12，2026/08/27，2026/09/11</t>
+          <t>2025/03/20，2025/03/29，2025/05/09，2025/05/18，2025/05/22，2025/05/26，2025/06/13，2025/06/23，2025/07/07，2025/07/14，2025/07/18，2025/08/07，2025/08/19，2025/08/28，2025/09/12，2025/09/28，2025/10/09，2025/12/08，2025/12/26，2026/01/05，2026/01/24，2026/02/05，2026/02/14，2026/03/09，2026/03/28，2026/04/26，2026/05/05，2026/05/23，2026/06/12，2026/08/27，2026/09/11，2026/09/26</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -7331,7 +7331,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/06，2026/02/07，2026/03/24，2026/04/26，2026/05/04，2026/05/23，2026/07/09，2026/07/27，2026/09/02，2026/09/08</t>
+          <t>2025/03/21，2025/04/13，2025/06/07，2025/06/16，2025/09/14，2025/10/05，2025/10/31，2025/11/12，2025/12/06，2026/02/07，2026/03/24，2026/04/26，2026/05/04，2026/05/23，2026/07/09，2026/07/27，2026/09/02，2026/09/08，2026/09/22</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -7342,7 +7342,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/14，2025/05/12，2025/06/07，2025/07/06，2025/07/21，2025/09/14，2025/10/31，2025/11/09，2026/01/09，2026/05/04，2026/07/27，2026/9/14</t>
+          <t>2025/03/21，2025/04/14，2025/05/12，2025/06/07，2025/07/06，2025/07/21，2025/09/14，2025/10/31，2025/11/09，2026/01/09，2026/05/04，2026/07/27，2026/09/14，2026/09/14，2026/09/22</t>
         </is>
       </c>
       <c r="F171" t="inlineStr"/>
@@ -7382,7 +7382,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -7527,7 +7527,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11，2026/08/28，2026/9/14</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11，2026/08/28，2026/09/14，2026/09/22</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7538,7 +7538,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/01/19，2026/03/09，2026/04/18，2026/04/20，2026/05/10，2026/06/19，2026/06/26，2026/07/27，2026/08/28</t>
+          <t>2025/03/21，2025/05/01，2025/05/24，2025/06/05，2025/06/26，2025/07/24，2025/09/11，2025/10/17，2025/10/23，2025/11/19，2026/01/19，2026/03/09，2026/04/18，2026/04/20，2026/05/10，2026/06/19，2026/06/26，2026/07/27，2026/08/28，2026/09/17</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -7746,7 +7746,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/07，2025/04/18，2025/05/08，2025/10/24，2025/12/12，2026/04/26，2026/09/06</t>
+          <t>2025/03/21，2025/04/07，2025/04/18，2025/05/08，2025/10/24，2025/12/12，2026/04/26，2026/09/06，2026/09/23</t>
         </is>
       </c>
       <c r="F181" t="inlineStr"/>
@@ -7786,7 +7786,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/05，2025/05/18，2025/06/12，2025/07/14，2025/07/15，2025/08/02，2025/08/30，2025/10/03，2025/11/01，2025/11/26，2025/12/02，2026/02/14，2026/07/09，2026/08/25</t>
+          <t>2025/03/21，2025/04/05，2025/05/18，2025/06/12，2025/07/14，2025/07/15，2025/08/02，2025/08/30，2025/10/03，2025/11/01，2025/11/26，2025/12/02，2026/02/14，2026/07/09，2026/08/25，2026/09/14</t>
         </is>
       </c>
       <c r="F183" t="inlineStr"/>
@@ -7866,7 +7866,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -8135,7 +8135,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>2025/03/23，2025/04/10，2025/05/01，2025/05/19，2025/06/08，2025/07/14，2025/09/11，2025/09/12，2025/10/31，2026/01/09，2026/07/05，2026/09/04，2026/09/11</t>
+          <t>2025/03/23，2025/04/10，2025/05/01，2025/05/19，2025/06/08，2025/07/14，2025/09/11，2025/09/12，2025/10/31，2026/01/09，2026/07/05，2026/09/04，2026/09/11，2026/09/16</t>
         </is>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -8255,7 +8255,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/06，2025/04/21，2025/04/26，2025/05/18，2025/08/24，2025/12/30</t>
+          <t>2025/03/24，2025/04/06，2025/04/21，2025/04/26，2025/05/18，2025/08/24，2025/12/30，2026/09/16</t>
         </is>
       </c>
       <c r="F193" t="inlineStr"/>
@@ -8266,7 +8266,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/07，2026/01/17，2026/02/14，2026/04/09，2026/05/20，2026/06/19，2026/06/28，2026/07/31，2026/09/04</t>
+          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/07，2026/01/17，2026/02/14，2026/04/09，2026/05/20，2026/06/19，2026/06/28，2026/07/31，2026/09/04，2026/09/21</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -8306,7 +8306,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/09，2026/01/01，2026/02/07，2026/03/25，2026/04/26，2026/06/23，2026/07/31，2026/07/31</t>
+          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/09，2026/01/01，2026/02/07，2026/03/25，2026/04/26，2026/06/23，2026/07/31，2026/07/31，2026/09/14</t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
@@ -8426,7 +8426,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -8575,7 +8575,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/03/25，2026/06/23，2026/08/21，2026/9/14</t>
+          <t>2025/03/25，2025/05/13，2025/05/29，2025/06/17，2025/08/22，2025/09/04，2026/03/25，2026/06/23，2026/08/21，2026/09/14</t>
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
@@ -8815,7 +8815,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/06，2025/05/01，2025/06/23，2025/07/09，2025/09/05，2025/09/15，2025/10/16，2025/11/19，2025/12/17，2026/04/09，2026/07/16</t>
+          <t>2025/03/25，2025/04/06，2025/05/01，2025/06/23，2025/07/09，2025/09/05，2025/09/15，2025/10/16，2025/11/19，2025/12/17，2026/04/09，2026/07/16，2026/09/21</t>
         </is>
       </c>
       <c r="F207" t="inlineStr"/>
@@ -8826,7 +8826,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/17，2025/05/15，2025/05/27，2025/11/27，2025/12/24，2026/01/14，2026/06/28，2026/08/18，2026/09/08</t>
+          <t>2025/03/27，2025/04/17，2025/05/15，2025/05/27，2025/11/27，2025/12/24，2026/01/14，2026/06/28，2026/08/18，2026/09/08，2026/09/16</t>
         </is>
       </c>
       <c r="F209" t="inlineStr"/>
@@ -8906,7 +8906,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -9263,7 +9263,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/01/16，2026/06/06，2026/07/09，2026/08/08，2026/09/02</t>
+          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/01/16，2026/06/06，2026/07/09，2026/08/08，2026/09/02，2026/09/17</t>
         </is>
       </c>
       <c r="F218" t="inlineStr"/>
@@ -9274,7 +9274,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -9463,7 +9463,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/09，2026/01/09，2026/02/19，2026/05/10，2026/07/10，2026/07/15，2026/07/31，2026/08/28</t>
+          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/09，2026/01/09，2026/02/19，2026/05/10，2026/07/10，2026/07/15，2026/07/31，2026/08/28，2026/09/16</t>
         </is>
       </c>
       <c r="F223" t="inlineStr"/>
@@ -9474,7 +9474,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -9579,7 +9579,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/08/28，2025/09/18，2025/11/21，2025/12/04，2026/03/21，2026/06/27</t>
+          <t>2025/03/28，2025/04/04，2025/08/28，2025/09/18，2025/11/21，2025/12/04，2026/03/21，2026/06/27，2026/09/16</t>
         </is>
       </c>
       <c r="F226" t="inlineStr"/>
@@ -9590,7 +9590,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/08/16，2026/09/02</t>
+          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/08/16，2026/09/02，2026/09/16</t>
         </is>
       </c>
       <c r="F228" t="inlineStr"/>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/17，2025/06/13，2025/07/05，2025/09/15，2025/10/23</t>
+          <t>2025/03/28，2025/05/17，2025/06/13，2025/07/05，2025/09/15，2025/10/23，2026/09/16</t>
         </is>
       </c>
       <c r="F231" t="inlineStr"/>
@@ -9790,7 +9790,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -9859,7 +9859,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/08，2025/12/12，2026/01/28，2026/03/07，2026/03/28，2026/04/19，2026/05/15，2026/07/27</t>
+          <t>2025/03/29，2025/04/01，2025/04/12，2025/04/14，2025/04/17，2025/04/18，2025/04/20，2025/04/29，2025/05/08，2025/05/20，2025/05/25，2025/06/03，2025/06/08，2025/06/14，2025/06/20，2025/07/05，2025/07/08，2025/07/17，2025/07/28，2025/08/07，2025/08/19，2025/08/28，2025/09/03，2025/09/20，2025/10/03，2025/10/26，2025/12/08，2025/12/12，2026/01/28，2026/03/07，2026/03/28，2026/04/19，2026/05/15，2026/07/27，2026/09/17</t>
         </is>
       </c>
       <c r="F233" t="inlineStr"/>
@@ -9870,7 +9870,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -9903,7 +9903,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/05/29，2025/06/17，2025/07/24，2025/08/16，2025/09/21，2025/10/30，2026/02/09</t>
+          <t>2025/03/29，2025/05/29，2025/06/17，2025/07/24，2025/08/16，2025/09/21，2025/10/30，2026/02/09，2026/09/26</t>
         </is>
       </c>
       <c r="F234" t="inlineStr"/>
@@ -9914,7 +9914,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -9978,7 +9978,7 @@
       <c r="C236" t="inlineStr"/>
       <c r="D236" t="inlineStr">
         <is>
-          <t>K/DA/Madison Beer/(G)I-DLE ((여자)아이들)/刘柏辛Lexie</t>
+          <t>K/DA/Madison Beer/(G)I-DLE/刘柏辛Lexie</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -10023,7 +10023,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/25，2025/05/03，2025/06/23，2025/09/28，2025/11/28，2025/12/26，2026/06/28，2026/08/27，2026/9/14</t>
+          <t>2025/03/29，2025/04/25，2025/05/03，2025/06/23，2025/09/28，2025/11/28，2025/12/26，2026/06/28，2026/08/27，2026/09/14</t>
         </is>
       </c>
       <c r="F237" t="inlineStr"/>
@@ -10067,7 +10067,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/08/22，2025/09/21，2025/10/20，2025/12/02，2026/02/09，2026/06/03</t>
+          <t>2025/03/29，2025/08/22，2025/09/21，2025/10/20，2025/12/02，2026/02/09，2026/06/03，2026/09/26</t>
         </is>
       </c>
       <c r="F238" t="inlineStr"/>
@@ -10078,7 +10078,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -10231,7 +10231,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/14，2025/05/26，2025/06/15，2025/07/09，2025/10/25，2025/11/24，2025/12/30，2026/01/16，2026/03/25，2026/05/23，2026/07/17，2026/08/25</t>
+          <t>2025/03/30，2025/04/14，2025/05/26，2025/06/15，2025/07/09，2025/10/25，2025/11/24，2025/12/30，2026/01/16，2026/03/25，2026/05/23，2026/07/17，2026/08/25，2026/09/26</t>
         </is>
       </c>
       <c r="F242" t="inlineStr"/>
@@ -10242,7 +10242,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -10351,7 +10351,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/01/09，2026/03/07，2026/04/19，2026/05/23，2026/07/16，2026/08/27</t>
+          <t>2025/03/30，2025/05/10，2025/06/01，2025/06/10，2025/06/13，2025/07/21，2025/07/22，2025/08/03，2025/09/24，2025/10/05，2026/01/09，2026/03/07，2026/04/19，2026/05/23，2026/07/16，2026/08/27，2026/09/23，2026/09/26</t>
         </is>
       </c>
       <c r="F245" t="inlineStr"/>
@@ -10362,7 +10362,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -10471,7 +10471,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/01/01，2026/01/25，2026/03/08，2026/04/27，2026/06/13，2026/07/28，2026/08/28</t>
+          <t>2025/03/30，2025/04/15，2025/05/09，2025/06/13，2025/06/27，2025/07/11，2025/08/29，2025/09/12，2025/11/27，2026/01/01，2026/01/25，2026/03/08，2026/04/27，2026/06/13，2026/07/28，2026/08/28，2026/09/14</t>
         </is>
       </c>
       <c r="F248" t="inlineStr"/>
@@ -10482,7 +10482,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/02，2026/04/08，2026/05/01，2026/06/10，2026/06/20，2026/08/02，2026/08/21</t>
+          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/02，2026/04/08，2026/05/01，2026/06/10，2026/06/20，2026/08/02，2026/08/21，2026/09/23</t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
@@ -10842,7 +10842,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -11191,7 +11191,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/04，2025/05/20，2025/06/23，2025/07/24，2025/09/12，2025/10/17，2025/12/09，2026/02/14，2026/03/25，2026/06/13，2026/07/28</t>
+          <t>2025/04/02，2025/05/04，2025/05/20，2025/06/23，2025/07/24，2025/09/12，2025/10/17，2025/12/09，2026/02/14，2026/03/25，2026/06/13，2026/07/28，2026/09/16</t>
         </is>
       </c>
       <c r="F266" t="inlineStr"/>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -11471,7 +11471,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08，2026/08/28，2026/9/14，2026/9/14</t>
+          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08，2026/08/28，2026/09/14，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
@@ -11482,7 +11482,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -11675,7 +11675,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/06，2026/01/09，2026/01/29，2026/03/25，2026/04/24，2026/05/23，2026/06/15，2026/07/09，2026/07/22，2026/08/25，2026/08/28</t>
+          <t>2025/04/03，2025/04/15，2025/05/22，2025/05/29，2025/06/02，2025/06/07，2025/06/12，2025/06/21，2025/06/23，2025/07/08，2025/07/13，2025/07/21，2025/08/01，2025/08/03，2025/09/02，2025/09/19，2025/10/10，2025/11/12，2025/11/26，2025/12/06，2026/01/09，2026/01/29，2026/03/25，2026/04/24，2026/05/23，2026/06/15，2026/07/09，2026/07/22，2026/08/25，2026/08/28，2026/09/22</t>
         </is>
       </c>
       <c r="F278" t="inlineStr"/>
@@ -11686,7 +11686,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/27，2026/08/16</t>
+          <t>2025/04/03，2025/04/27，2026/08/16，2026/09/16</t>
         </is>
       </c>
       <c r="F279" t="inlineStr"/>
@@ -11726,7 +11726,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -11795,7 +11795,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/24，2025/09/12，2026/01/10，2026/06/03，2026/09/04</t>
+          <t>2025/04/03，2025/04/24，2025/09/12，2026/01/10，2026/06/03，2026/09/04，2026/09/16</t>
         </is>
       </c>
       <c r="F281" t="inlineStr"/>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -11929,7 +11929,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I284" t="inlineStr"/>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>BV1r8Yt6wEGn</t>
+        </is>
+      </c>
       <c r="J284" t="inlineStr"/>
     </row>
     <row r="285">
@@ -11951,7 +11955,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/07/11</t>
+          <t>2025/04/04，2025/07/11，2026/09/16</t>
         </is>
       </c>
       <c r="F285" t="inlineStr"/>
@@ -11962,7 +11966,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -12307,7 +12311,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/02/14，2026/03/05，2026/04/02，2026/05/20，2026/08/28，2026/9/14</t>
+          <t>2025/04/05，2025/04/11，2025/04/19，2025/05/04，2025/05/09，2025/05/23，2025/05/30，2025/06/27，2025/08/16，2025/09/30，2026/02/14，2026/03/05，2026/04/02，2026/05/20，2026/08/28，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -12318,7 +12322,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -12347,7 +12351,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>2025/04/05，2025/04/19，2025/05/20，2025/07/11，2025/09/12，2025/12/09，2025/12/16，2026/02/27，2026/06/13，2026/9/14</t>
+          <t>2025/04/05，2025/04/19，2025/05/20，2025/07/11，2025/09/12，2025/12/09，2025/12/16，2026/02/27，2026/06/13，2026/09/14，2026/09/16</t>
         </is>
       </c>
       <c r="F295" t="inlineStr"/>
@@ -12358,7 +12362,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -12751,7 +12755,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23，2026/08/30，2026/09/11，2026/9/14，2026/9/14</t>
+          <t>2025/04/07，2025/04/24，2025/05/03，2025/05/23，2025/06/07，2025/06/12，2025/06/23，2025/06/29，2025/07/15，2025/07/25，2025/09/24，2025/10/18，2025/11/12，2025/11/24，2025/12/23，2026/01/29，2026/03/20，2026/04/22，2026/07/09，2026/08/23，2026/08/30，2026/09/11，2026/09/14，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F305" t="inlineStr"/>
@@ -12762,7 +12766,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -12831,7 +12835,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/01/03，2026/01/22，2026/02/14，2026/05/20，2026/08/08，2026/08/19，2026/08/25，2026/09/06</t>
+          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/01/03，2026/01/22，2026/02/14，2026/05/20，2026/08/08，2026/08/19，2026/08/25，2026/09/06，2026/09/22</t>
         </is>
       </c>
       <c r="F307" t="inlineStr"/>
@@ -12842,7 +12846,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -12911,7 +12915,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/03，2025/11/09，2025/11/26，2025/12/09，2026/01/23，2026/03/13，2026/03/25，2026/04/08，2026/05/23，2026/06/20，2026/08/02，2026/08/28，2026/09/11</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/03，2025/11/09，2025/11/26，2025/12/09，2026/01/23，2026/03/13，2026/03/25，2026/04/08，2026/05/23，2026/06/20，2026/08/02，2026/08/28，2026/09/11，2026/09/16</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12922,7 +12926,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -12951,7 +12955,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/09，2026/01/24，2026/03/31，2026/04/02，2026/06/15，2026/07/27，2026/09/02</t>
+          <t>2025/04/08，2025/04/18，2025/04/19，2025/04/26，2025/05/04，2025/05/08，2025/05/19，2025/05/29，2025/06/07，2025/06/23，2025/07/05，2025/07/13，2025/08/21，2025/09/21，2025/10/25，2025/10/26，2025/11/19，2025/12/09，2026/01/24，2026/03/31，2026/04/02，2026/06/15，2026/07/27，2026/09/02，2026/09/14</t>
         </is>
       </c>
       <c r="F310" t="inlineStr"/>
@@ -12962,7 +12966,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -13391,7 +13395,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/09，2025/12/08，2026/01/05，2026/02/14，2026/05/23，2026/06/20，2026/07/18，2026/08/25，2026/08/30</t>
+          <t>2025/04/11，2025/04/28，2025/05/26，2025/06/17，2025/07/15，2025/07/26，2025/08/13，2025/09/03，2025/09/12，2025/10/07，2025/11/09，2025/12/08，2026/01/05，2026/02/14，2026/05/23，2026/06/20，2026/07/18，2026/08/25，2026/08/30，2026/09/14</t>
         </is>
       </c>
       <c r="F321" t="inlineStr"/>
@@ -13402,7 +13406,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -13743,7 +13747,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/18，2025/09/08，2025/12/05，2026/01/28，2026/04/19</t>
+          <t>2025/04/11，2025/05/18，2025/09/08，2025/12/05，2026/01/28，2026/04/19，2026/09/21</t>
         </is>
       </c>
       <c r="F330" t="inlineStr"/>
@@ -13754,7 +13758,7 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -13823,7 +13827,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/06/02，2025/06/12，2025/09/27，2025/11/09，2025/12/19，2026/01/01，2026/02/17，2026/07/09，2026/07/27，2026/08/21</t>
+          <t>2025/04/11，2025/06/02，2025/06/12，2025/09/27，2025/11/09，2025/12/19，2026/01/01，2026/02/17，2026/07/09，2026/07/27，2026/08/21，2026/09/21</t>
         </is>
       </c>
       <c r="F332" t="inlineStr"/>
@@ -13834,7 +13838,7 @@
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I332" t="inlineStr">
@@ -13943,7 +13947,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>2025/04/12，2026/08/30，2026/09/04</t>
+          <t>2025/04/12，2026/08/30，2026/09/04，2026/09/21</t>
         </is>
       </c>
       <c r="F335" t="inlineStr"/>
@@ -13954,7 +13958,7 @@
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I335" t="inlineStr">
@@ -14159,7 +14163,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>2025/04/13，2025/07/13，2025/07/18，2025/08/02，2025/09/04，2025/09/12，2025/10/17，2025/11/28，2026/01/22，2026/02/23，2026/09/04</t>
+          <t>2025/04/13，2025/07/13，2025/07/18，2025/08/02，2025/09/04，2025/09/12，2025/10/17，2025/11/28，2026/01/22，2026/02/23，2026/09/04，2026/09/16</t>
         </is>
       </c>
       <c r="F340" t="inlineStr"/>
@@ -14170,7 +14174,7 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
@@ -14243,7 +14247,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>2025/04/14，2025/10/31，2026/08/11</t>
+          <t>2025/04/14，2025/10/31，2026/08/11，2026/09/23</t>
         </is>
       </c>
       <c r="F342" t="inlineStr"/>
@@ -14254,7 +14258,7 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
@@ -14443,7 +14447,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/01/16，2026/03/25，2026/04/24，2026/05/23，2026/07/17，2026/08/21，2026/09/11</t>
+          <t>2025/04/15，2025/04/18，2025/05/12，2025/06/17，2025/09/03，2025/10/07，2025/11/24，2026/01/16，2026/03/25，2026/04/24，2026/05/23，2026/07/17，2026/08/21，2026/09/11，2026/09/26</t>
         </is>
       </c>
       <c r="F347" t="inlineStr"/>
@@ -14454,7 +14458,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -14483,7 +14487,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/25，2025/05/30，2025/06/17，2025/09/26，2025/10/03，2025/11/03，2025/12/23，2026/04/09，2026/9/14</t>
+          <t>2025/04/15，2025/04/25，2025/05/30，2025/06/17，2025/09/26，2025/10/03，2025/11/03，2025/12/23，2026/04/09，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F348" t="inlineStr"/>
@@ -14494,7 +14498,7 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
@@ -14523,7 +14527,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>2025/04/15，2025/04/18，2025/04/20，2025/05/18，2025/05/20，2025/05/25，2025/06/28，2025/06/30，2025/08/24，2025/09/26，2026/01/09，2026/04/17</t>
+          <t>2025/04/15，2025/04/18，2025/04/20，2025/05/18，2025/05/20，2025/05/25，2025/06/28，2025/06/30，2025/08/24，2025/09/26，2026/01/09，2026/04/17，2026/09/17</t>
         </is>
       </c>
       <c r="F349" t="inlineStr"/>
@@ -14534,7 +14538,7 @@
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I349" t="inlineStr">
@@ -14603,7 +14607,7 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/05/13，2025/06/13，2025/07/07，2025/09/30</t>
+          <t>2025/04/17，2025/05/13，2025/06/13，2025/07/07，2025/09/30，2026/09/16</t>
         </is>
       </c>
       <c r="F351" t="inlineStr"/>
@@ -14614,7 +14618,7 @@
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I351" t="inlineStr">
@@ -14683,7 +14687,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/04/18，2025/07/03，2025/10/17，2025/10/30，2026/01/09</t>
+          <t>2025/04/17，2025/04/18，2025/07/03，2025/10/17，2025/10/30，2026/01/09，2026/09/23</t>
         </is>
       </c>
       <c r="F353" t="inlineStr"/>
@@ -14694,7 +14698,7 @@
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
@@ -14851,7 +14855,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/04/29，2025/05/22，2025/05/25，2025/05/31，2025/08/29，2025/09/20，2025/10/09，2025/10/30，2025/12/11，2026/02/18，2026/05/20，2026/07/05，2026/07/31，2026/09/06</t>
+          <t>2025/04/17，2025/04/29，2025/05/22，2025/05/25，2025/05/31，2025/08/29，2025/09/20，2025/10/09，2025/10/30，2025/12/11，2026/02/18，2026/05/20，2026/07/05，2026/07/31，2026/09/06，2026/09/22</t>
         </is>
       </c>
       <c r="F357" t="inlineStr"/>
@@ -14862,7 +14866,7 @@
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
@@ -15411,7 +15415,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/09，2025/11/26，2025/12/05，2025/12/06，2026/01/01，2026/01/29，2026/03/01，2026/04/09，2026/05/20，2026/07/27，2026/09/11</t>
+          <t>2025/04/20，2025/04/27，2025/05/05，2025/05/09，2025/05/18，2025/06/07，2025/06/13，2025/06/21，2025/07/05，2025/07/15，2025/07/25，2025/08/08，2025/08/26，2025/08/28，2025/09/14，2025/09/30，2025/10/03，2025/10/24，2025/10/31，2025/11/09，2025/11/26，2025/12/05，2025/12/06，2026/01/01，2026/01/29，2026/03/01，2026/04/09，2026/05/20，2026/07/27，2026/09/11，2026/09/22</t>
         </is>
       </c>
       <c r="F371" t="inlineStr"/>
@@ -15422,7 +15426,7 @@
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I371" t="inlineStr">
@@ -15451,7 +15455,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>2025/04/20，2025/12/23</t>
+          <t>2025/04/20，2025/12/23，2026/09/21</t>
         </is>
       </c>
       <c r="F372" t="inlineStr"/>
@@ -15462,7 +15466,7 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I372" t="inlineStr">
@@ -16471,7 +16475,7 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/23，2025/10/09，2026/01/22，2026/03/09，2026/9/14</t>
+          <t>2025/04/25，2025/06/23，2025/10/09，2026/01/22，2026/03/09，2026/09/14</t>
         </is>
       </c>
       <c r="F398" t="inlineStr"/>
@@ -16551,7 +16555,7 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>2025/04/27，2025/06/02，2025/06/09，2025/07/09，2025/07/14，2025/08/26，2025/11/21，2025/12/17，2026/01/09，2026/04/09，2026/9/14</t>
+          <t>2025/04/27，2025/06/02，2025/06/09，2025/07/09，2025/07/14，2025/08/26，2025/11/21，2025/12/17，2026/01/09，2026/04/09，2026/09/14</t>
         </is>
       </c>
       <c r="F400" t="inlineStr"/>
@@ -16795,7 +16799,7 @@
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/05/06，2025/07/27，2025/09/17，2025/10/16，2025/11/09，2026/02/12，2026/07/10，2026/07/15</t>
+          <t>2025/04/28，2025/05/06，2025/07/27，2025/09/17，2025/10/16，2025/11/09，2026/02/12，2026/07/10，2026/07/15，2026/09/16</t>
         </is>
       </c>
       <c r="F406" t="inlineStr"/>
@@ -16806,7 +16810,7 @@
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I406" t="inlineStr">
@@ -17191,7 +17195,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/08/28，2025/09/11，2025/10/20，2025/12/09，2026/08/16</t>
+          <t>2025/05/03，2025/08/28，2025/09/11，2025/10/20，2025/12/09，2026/08/16，2026/09/16</t>
         </is>
       </c>
       <c r="F416" t="inlineStr"/>
@@ -17202,7 +17206,7 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I416" t="inlineStr">
@@ -17351,7 +17355,7 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>2025/05/03，2026/08/27，2026/9/14，2026/9/14</t>
+          <t>2025/05/03，2026/08/27，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F420" t="inlineStr"/>
@@ -17827,7 +17831,7 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/04/29，2026/08/07，2026/09/02</t>
+          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/04/29，2026/08/07，2026/09/02，2026/09/22</t>
         </is>
       </c>
       <c r="F432" t="inlineStr"/>
@@ -17838,7 +17842,7 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I432" t="inlineStr">
@@ -18187,7 +18191,7 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/01/01，2026/02/10，2026/02/22，2026/03/12，2026/04/05，2026/05/03，2026/05/24，2026/07/03，2026/08/07，2026/08/23</t>
+          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/01/01，2026/02/10，2026/02/22，2026/03/12，2026/04/05，2026/05/03，2026/05/24，2026/07/03，2026/08/07，2026/08/23，2026/09/16</t>
         </is>
       </c>
       <c r="F441" t="inlineStr"/>
@@ -18198,7 +18202,7 @@
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
@@ -18711,7 +18715,7 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/06/17，2025/06/23，2025/07/06，2025/07/15，2025/09/10，2025/10/18，2025/11/13，2026/05/04，2026/07/09，2026/08/30</t>
+          <t>2025/05/22，2025/06/17，2025/06/23，2025/07/06，2025/07/15，2025/09/10，2025/10/18，2025/11/13，2026/05/04，2026/07/09，2026/08/30，2026/09/22</t>
         </is>
       </c>
       <c r="F454" t="inlineStr"/>
@@ -18722,7 +18726,7 @@
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I454" t="inlineStr">
@@ -18835,7 +18839,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/07/21，2026/04/14，2026/06/19，2026/9/14，2026/9/14</t>
+          <t>2025/05/22，2025/07/21，2026/04/14，2026/06/19，2026/09/14，2026/09/14，2026/09/22</t>
         </is>
       </c>
       <c r="F457" t="inlineStr"/>
@@ -18846,7 +18850,7 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">
@@ -18959,7 +18963,7 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/09/12，2025/10/03，2025/10/11，2026/01/15，2026/04/29，2026/06/18</t>
+          <t>2025/05/22，2025/09/12，2025/10/03，2025/10/11，2026/01/15，2026/04/29，2026/06/18，2026/09/26</t>
         </is>
       </c>
       <c r="F460" t="inlineStr"/>
@@ -18970,7 +18974,7 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I460" t="inlineStr">
@@ -19443,7 +19447,7 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/07，2025/12/07，2025/12/23，2026/01/09，2026/01/24，2026/02/09，2026/02/25，2026/03/13，2026/03/21，2026/04/18，2026/05/04，2026/05/23，2026/06/14，2026/06/19，2026/07/16，2026/08/23</t>
+          <t>2025/05/27，2025/05/29，2025/05/30，2025/05/31，2025/06/02，2025/06/03，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/11，2025/07/22，2025/08/21，2025/09/10，2025/09/26，2025/10/03，2025/10/11，2025/10/26，2025/11/07，2025/12/07，2025/12/23，2026/01/09，2026/01/24，2026/02/09，2026/02/25，2026/03/13，2026/03/21，2026/04/18，2026/05/04，2026/05/23，2026/06/14，2026/06/19，2026/07/16，2026/08/23，2026/09/22，2026/09/23</t>
         </is>
       </c>
       <c r="F472" t="inlineStr"/>
@@ -19454,7 +19458,7 @@
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>38</t>
         </is>
       </c>
       <c r="I472" t="inlineStr">
@@ -19883,7 +19887,7 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>2025/05/31，2025/12/09</t>
+          <t>2025/05/31，2025/12/09，2026/09/26</t>
         </is>
       </c>
       <c r="F483" t="inlineStr"/>
@@ -19894,7 +19898,7 @@
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I483" t="inlineStr">
@@ -20927,7 +20931,7 @@
       </c>
       <c r="E509" t="inlineStr">
         <is>
-          <t>2025/06/08，2025/06/13，2025/06/16，2025/06/28，2025/07/18，2025/07/29，2025/08/18，2025/09/03，2025/09/11，2025/09/30，2025/10/05，2025/10/30，2025/11/17，2025/12/24，2026/02/02，2026/03/25</t>
+          <t>2025/06/08，2025/06/13，2025/06/16，2025/06/28，2025/07/18，2025/07/29，2025/08/18，2025/09/03，2025/09/11，2025/09/30，2025/10/05，2025/10/30，2025/11/17，2025/12/24，2026/02/02，2026/03/25，2026/09/21</t>
         </is>
       </c>
       <c r="F509" t="inlineStr"/>
@@ -20938,7 +20942,7 @@
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I509" t="inlineStr">
@@ -21127,7 +21131,7 @@
       </c>
       <c r="E514" t="inlineStr">
         <is>
-          <t>2025/06/12，2025/07/13，2025/07/18，2025/09/28，2025/10/20，2026/01/19，2026/04/17，2026/06/15</t>
+          <t>2025/06/12，2025/07/13，2025/07/18，2025/09/28，2025/10/20，2026/01/19，2026/04/17，2026/06/15，2026/09/21</t>
         </is>
       </c>
       <c r="F514" t="inlineStr"/>
@@ -21138,7 +21142,7 @@
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I514" t="inlineStr">
@@ -21931,7 +21935,7 @@
       </c>
       <c r="E534" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/23，2025/09/29，2026/01/09，2026/02/10</t>
+          <t>2025/06/20，2025/06/23，2025/09/29，2026/01/09，2026/02/10，2026/09/21</t>
         </is>
       </c>
       <c r="F534" t="inlineStr"/>
@@ -21942,7 +21946,7 @@
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I534" t="inlineStr">
@@ -22135,7 +22139,7 @@
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>2025/06/23</t>
+          <t>2025/06/23，2026/09/21</t>
         </is>
       </c>
       <c r="F539" t="inlineStr"/>
@@ -22146,7 +22150,7 @@
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I539" t="inlineStr">
@@ -22511,7 +22515,7 @@
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>2025/06/27，2025/07/21，2025/08/18，2025/08/21，2025/09/17，2025/09/22，2025/10/16，2025/11/26，2026/01/19，2026/05/20</t>
+          <t>2025/06/27，2025/07/21，2025/08/18，2025/08/21，2025/09/17，2025/09/22，2025/10/16，2025/11/26，2026/01/19，2026/05/20，2026/09/22</t>
         </is>
       </c>
       <c r="F548" t="inlineStr"/>
@@ -22522,7 +22526,7 @@
       </c>
       <c r="H548" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I548" t="inlineStr">
@@ -23823,7 +23827,7 @@
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>2025/07/11</t>
+          <t>2025/07/11，2026/09/23</t>
         </is>
       </c>
       <c r="F581" t="inlineStr"/>
@@ -23834,7 +23838,7 @@
       </c>
       <c r="H581" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I581" t="inlineStr">
@@ -23863,7 +23867,7 @@
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>2025/07/13，2025/08/26，2025/12/17</t>
+          <t>2025/07/13，2025/08/26，2025/12/17，2026/09/16</t>
         </is>
       </c>
       <c r="F582" t="inlineStr"/>
@@ -23874,7 +23878,7 @@
       </c>
       <c r="H582" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I582" t="inlineStr">
@@ -24103,7 +24107,7 @@
       </c>
       <c r="E588" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/01/09，2026/04/02，2026/04/24，2026/05/22，2026/06/12，2026/06/17，2026/08/11</t>
+          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/01/09，2026/04/02，2026/04/24，2026/05/22，2026/06/12，2026/06/17，2026/08/11，2026/09/19</t>
         </is>
       </c>
       <c r="F588" t="inlineStr"/>
@@ -24114,7 +24118,7 @@
       </c>
       <c r="H588" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I588" t="inlineStr">
@@ -24331,7 +24335,7 @@
       </c>
       <c r="E594" t="inlineStr">
         <is>
-          <t>2025/07/21，2025/09/08</t>
+          <t>2025/07/21，2025/09/08，2026/09/21</t>
         </is>
       </c>
       <c r="F594" t="inlineStr"/>
@@ -24342,7 +24346,7 @@
       </c>
       <c r="H594" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I594" t="inlineStr">
@@ -24615,7 +24619,7 @@
       </c>
       <c r="E601" t="inlineStr">
         <is>
-          <t>2025/07/26，2026/07/17</t>
+          <t>2025/07/26，2026/07/17，2026/09/26</t>
         </is>
       </c>
       <c r="F601" t="inlineStr"/>
@@ -24626,7 +24630,7 @@
       </c>
       <c r="H601" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I601" t="inlineStr">
@@ -24655,7 +24659,7 @@
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>2025/07/26，2025/08/08，2026/07/22，2026/9/14，2026/9/14</t>
+          <t>2025/07/26，2025/08/08，2026/07/22，2026/09/14，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F602" t="inlineStr"/>
@@ -24666,7 +24670,7 @@
       </c>
       <c r="H602" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I602" t="inlineStr">
@@ -24775,7 +24779,7 @@
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>2025/07/31，2025/09/12</t>
+          <t>2025/07/31，2025/09/12，2026/09/21</t>
         </is>
       </c>
       <c r="F605" t="inlineStr"/>
@@ -24786,7 +24790,7 @@
       </c>
       <c r="H605" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I605" t="inlineStr">
@@ -25687,7 +25691,7 @@
       </c>
       <c r="E628" t="inlineStr">
         <is>
-          <t>2025/09/10，2025/09/22，2025/09/24，2025/10/23，2025/12/06，2026/01/24，2026/02/05，2026/02/23，2026/05/05，2026/05/23，2026/07/09</t>
+          <t>2025/09/10，2025/09/22，2025/09/24，2025/10/23，2025/12/06，2026/01/24，2026/02/05，2026/02/23，2026/05/05，2026/05/23，2026/07/09，2026/09/21</t>
         </is>
       </c>
       <c r="F628" t="inlineStr"/>
@@ -25698,7 +25702,7 @@
       </c>
       <c r="H628" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I628" t="inlineStr">
@@ -26071,7 +26075,7 @@
       </c>
       <c r="E638" t="inlineStr">
         <is>
-          <t>2025/09/12，2025/10/17</t>
+          <t>2025/09/12，2025/10/17，2026/09/16</t>
         </is>
       </c>
       <c r="F638" t="inlineStr"/>
@@ -26082,7 +26086,7 @@
       </c>
       <c r="H638" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I638" t="inlineStr">
@@ -26311,7 +26315,7 @@
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/03，2025/11/13，2025/11/24，2025/12/05，2025/12/12，2025/12/17，2026/01/06，2026/01/15，2026/01/24，2026/02/27，2026/04/19，2026/06/06，2026/07/17，2026/07/28，2026/08/28，2026/08/30</t>
+          <t>2025/09/13，2025/09/13，2025/09/13，2025/09/17，2025/09/18，2025/09/20，2025/09/21，2025/09/24，2025/09/29，2025/10/10，2025/10/13，2025/10/22，2025/10/30，2025/11/03，2025/11/13，2025/11/24，2025/12/05，2025/12/12，2025/12/17，2026/01/06，2026/01/15，2026/01/24，2026/02/27，2026/04/19，2026/06/06，2026/07/17，2026/07/28，2026/08/28，2026/08/30，2026/09/16</t>
         </is>
       </c>
       <c r="F644" t="inlineStr"/>
@@ -26322,7 +26326,7 @@
       </c>
       <c r="H644" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I644" t="inlineStr">
@@ -26895,7 +26899,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31，2026/08/23，2026/09/04</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31，2026/08/23，2026/09/04，2026/09/17</t>
         </is>
       </c>
       <c r="F659" t="inlineStr"/>
@@ -26906,7 +26910,7 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
@@ -27087,7 +27091,7 @@
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>2025/09/22，2025/10/09，2025/12/05，2026/08/16</t>
+          <t>2025/09/22，2025/10/09，2025/12/05，2026/08/16，2026/09/16</t>
         </is>
       </c>
       <c r="F664" t="inlineStr"/>
@@ -27098,7 +27102,7 @@
       </c>
       <c r="H664" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I664" t="inlineStr">
@@ -27671,7 +27675,7 @@
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>2025/09/30，2025/10/01，2025/10/11，2025/10/17，2025/10/26，2026/08/16</t>
+          <t>2025/09/30，2025/10/01，2025/10/11，2025/10/17，2025/10/26，2026/08/16，2026/09/16</t>
         </is>
       </c>
       <c r="F679" t="inlineStr"/>
@@ -27682,7 +27686,7 @@
       </c>
       <c r="H679" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I679" t="inlineStr">
@@ -27831,7 +27835,7 @@
       </c>
       <c r="E683" t="inlineStr">
         <is>
-          <t>2025/10/01，2025/10/07，2025/10/10，2025/10/13，2025/10/17，2025/10/20，2025/11/03，2025/11/27</t>
+          <t>2025/10/01，2025/10/07，2025/10/10，2025/10/13，2025/10/17，2025/10/20，2025/11/03，2025/11/27，2026/09/16</t>
         </is>
       </c>
       <c r="F683" t="inlineStr"/>
@@ -27842,7 +27846,7 @@
       </c>
       <c r="H683" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I683" t="inlineStr">
@@ -27943,7 +27947,7 @@
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>2025/10/05</t>
+          <t>2025/10/05，2026/09/26</t>
         </is>
       </c>
       <c r="F686" t="inlineStr"/>
@@ -27954,7 +27958,7 @@
       </c>
       <c r="H686" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I686" t="inlineStr">
@@ -28279,7 +28283,7 @@
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>2025/10/17，2025/10/18，2025/10/23，2025/12/30，2026/01/12，2026/03/29</t>
+          <t>2025/10/17，2025/10/18，2025/10/23，2025/12/30，2026/01/12，2026/03/29，2026/09/16</t>
         </is>
       </c>
       <c r="F694" t="inlineStr"/>
@@ -28290,7 +28294,7 @@
       </c>
       <c r="H694" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I694" t="inlineStr">
@@ -28319,7 +28323,7 @@
       </c>
       <c r="E695" t="inlineStr">
         <is>
-          <t>2025/10/17，2025/10/18，2025/10/23，2025/10/28，2025/12/05，2025/12/12，2025/12/30</t>
+          <t>2025/10/17，2025/10/18，2025/10/23，2025/10/28，2025/12/05，2025/12/12，2025/12/30，2026/09/16</t>
         </is>
       </c>
       <c r="F695" t="inlineStr"/>
@@ -28330,7 +28334,7 @@
       </c>
       <c r="H695" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I695" t="inlineStr">
@@ -28519,7 +28523,7 @@
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>2025/10/19，2025/10/20，2025/11/18，2025/12/08，2025/12/16，2026/01/10，2026/06/17</t>
+          <t>2025/10/19，2025/10/20，2025/11/18，2025/12/08，2025/12/16，2026/01/10，2026/06/17，2026/09/21</t>
         </is>
       </c>
       <c r="F700" t="inlineStr"/>
@@ -28530,7 +28534,7 @@
       </c>
       <c r="H700" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I700" t="inlineStr">
@@ -28979,7 +28983,7 @@
       </c>
       <c r="E712" t="inlineStr">
         <is>
-          <t>2025/10/24，2025/10/25，2025/10/28，2025/11/01，2025/11/12，2025/11/26，2025/12/08，2026/01/02，2026/01/05，2026/01/09，2026/02/23，2026/03/14，2026/03/29，2026/04/24，2026/07/09，2026/08/11</t>
+          <t>2025/10/24，2025/10/25，2025/10/28，2025/11/01，2025/11/12，2025/11/26，2025/12/08，2026/01/02，2026/01/05，2026/01/09，2026/02/23，2026/03/14，2026/03/29，2026/04/24，2026/07/09，2026/08/11，2026/09/21</t>
         </is>
       </c>
       <c r="F712" t="inlineStr"/>
@@ -28990,7 +28994,7 @@
       </c>
       <c r="H712" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I712" t="inlineStr">
@@ -29487,7 +29491,7 @@
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/06，2025/12/12，2025/12/26，2026/01/05，2026/01/30，2026/02/09，2026/03/25，2026/05/01，2026/06/17，2026/07/25，2026/09/02</t>
+          <t>2025/11/12，2025/11/14，2025/11/24，2025/12/06，2025/12/12，2025/12/26，2026/01/05，2026/01/30，2026/02/09，2026/03/25，2026/05/01，2026/06/17，2026/07/25，2026/09/02，2026/09/22</t>
         </is>
       </c>
       <c r="F725" t="inlineStr"/>
@@ -29498,7 +29502,7 @@
       </c>
       <c r="H725" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I725" t="inlineStr">
@@ -29643,7 +29647,7 @@
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>2025/11/14</t>
+          <t>2025/11/14，2026/09/16</t>
         </is>
       </c>
       <c r="F729" t="inlineStr"/>
@@ -29654,10 +29658,14 @@
       </c>
       <c r="H729" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I729" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>BV1zueg62Eh7</t>
+        </is>
+      </c>
       <c r="J729" t="inlineStr"/>
     </row>
     <row r="730">
@@ -30067,7 +30075,7 @@
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/06，2025/12/13，2026/01/10，2026/01/24，2026/02/14，2026/03/14，2026/04/01，2026/04/08，2026/05/01，2026/05/06，2026/05/23，2026/06/20，2026/07/18，2026/08/07，2026/09/02</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/06，2025/12/13，2026/01/10，2026/01/24，2026/02/14，2026/03/14，2026/04/01，2026/04/08，2026/05/01，2026/05/06，2026/05/23，2026/06/20，2026/07/18，2026/08/07，2026/09/02，2026/09/22</t>
         </is>
       </c>
       <c r="F740" t="inlineStr"/>
@@ -30078,7 +30086,7 @@
       </c>
       <c r="H740" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I740" t="inlineStr">
@@ -30811,7 +30819,7 @@
       </c>
       <c r="E759" t="inlineStr">
         <is>
-          <t>2025/12/19，2026/02/08，2026/05/01，2026/05/25</t>
+          <t>2025/12/19，2026/02/08，2026/05/01，2026/05/25，2026/09/23</t>
         </is>
       </c>
       <c r="F759" t="inlineStr"/>
@@ -30822,7 +30830,7 @@
       </c>
       <c r="H759" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I759" t="inlineStr">
@@ -30891,7 +30899,7 @@
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/01/02，2026/01/05，2026/01/11，2026/01/25，2026/02/09，2026/02/23，2026/03/20，2026/04/02，2026/04/16，2026/04/29，2026/05/10，2026/06/06，2026/06/14，2026/06/20，2026/07/16，2026/08/02，2026/08/07，2026/08/23，2026/08/28，2026/09/11</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/01/02，2026/01/05，2026/01/11，2026/01/25，2026/02/09，2026/02/23，2026/03/20，2026/04/02，2026/04/16，2026/04/29，2026/05/10，2026/06/06，2026/06/14，2026/06/20，2026/07/16，2026/08/02，2026/08/07，2026/08/23，2026/08/28，2026/09/11，2026/09/26</t>
         </is>
       </c>
       <c r="F761" t="inlineStr"/>
@@ -30902,7 +30910,7 @@
       </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I761" t="inlineStr">
@@ -30931,7 +30939,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08，2026/08/19，2026/09/02</t>
+          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08，2026/08/19，2026/09/02，2026/09/17</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -30942,7 +30950,7 @@
       </c>
       <c r="H762" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I762" t="inlineStr">
@@ -31055,7 +31063,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/01/10，2026/01/22，2026/01/23，2026/01/31，2026/02/10，2026/02/23，2026/03/09，2026/03/12，2026/03/14，2026/03/17，2026/03/27，2026/04/24，2026/05/01，2026/06/14，2026/08/01，2026/08/28</t>
+          <t>2025/12/26，2026/01/10，2026/01/22，2026/01/23，2026/01/31，2026/02/10，2026/02/23，2026/03/09，2026/03/12，2026/03/14，2026/03/17，2026/03/27，2026/04/24，2026/05/01，2026/06/14，2026/08/01，2026/08/28，2026/09/16</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -31066,7 +31074,7 @@
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I765" t="inlineStr">
@@ -31242,7 +31250,7 @@
       <c r="C770" t="inlineStr"/>
       <c r="D770" t="inlineStr">
         <is>
-          <t>三理Mit3uri</t>
+          <t>龙奔</t>
         </is>
       </c>
       <c r="E770" t="inlineStr">
@@ -31443,7 +31451,7 @@
       </c>
       <c r="E775" t="inlineStr">
         <is>
-          <t>2026/01/23，2026/03/29，2026/07/26，2026/07/27，2026/09/11</t>
+          <t>2026/01/23，2026/03/29，2026/07/26，2026/07/27，2026/09/11，2026/09/21</t>
         </is>
       </c>
       <c r="F775" t="inlineStr"/>
@@ -31454,7 +31462,7 @@
       </c>
       <c r="H775" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I775" t="inlineStr">
@@ -31483,7 +31491,7 @@
       </c>
       <c r="E776" t="inlineStr">
         <is>
-          <t>2026/01/24，2026/01/25，2026/01/26，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/03/04，2026/03/12，2026/03/31，2026/04/01，2026/04/14，2026/04/18，2026/05/10，2026/05/23，2026/06/12，2026/07/03，2026/07/21，2026/08/07，2026/08/23</t>
+          <t>2026/01/24，2026/01/25，2026/01/26，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/03/04，2026/03/12，2026/03/31，2026/04/01，2026/04/14，2026/04/18，2026/05/10，2026/05/23，2026/06/12，2026/07/03，2026/07/21，2026/08/07，2026/08/23，2026/09/21</t>
         </is>
       </c>
       <c r="F776" t="inlineStr"/>
@@ -31494,7 +31502,7 @@
       </c>
       <c r="H776" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I776" t="inlineStr">
@@ -31931,7 +31939,7 @@
       </c>
       <c r="E787" t="inlineStr">
         <is>
-          <t>2026/02/08，2026/02/09，2026/02/14，2026/02/20，2026/02/28，2026/05/25，2026/06/13，2026/07/05，2026/07/18，2026/08/08，2026/08/23，2026/9/14，2026/9/14</t>
+          <t>2026/02/08，2026/02/09，2026/02/14，2026/02/20，2026/02/28，2026/05/25，2026/06/13，2026/07/05，2026/07/18，2026/08/08，2026/08/23，2026/09/14，2026/09/14，2026/09/26</t>
         </is>
       </c>
       <c r="F787" t="inlineStr"/>
@@ -31942,7 +31950,7 @@
       </c>
       <c r="H787" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I787" t="inlineStr">
@@ -32015,7 +32023,7 @@
       </c>
       <c r="E789" t="inlineStr">
         <is>
-          <t>2026/02/09，2026/02/27，2026/03/09，2026/04/14，2026/05/25，2026/07/25</t>
+          <t>2026/02/09，2026/02/27，2026/03/09，2026/04/14，2026/05/25，2026/07/25，2026/09/22</t>
         </is>
       </c>
       <c r="F789" t="inlineStr"/>
@@ -32026,7 +32034,7 @@
       </c>
       <c r="H789" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I789" t="inlineStr">
@@ -32219,7 +32227,7 @@
       </c>
       <c r="E794" t="inlineStr">
         <is>
-          <t>2026/02/19</t>
+          <t>2026/02/19，2026/09/21</t>
         </is>
       </c>
       <c r="F794" t="inlineStr"/>
@@ -32230,7 +32238,7 @@
       </c>
       <c r="H794" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I794" t="inlineStr">
@@ -32379,7 +32387,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>2026/02/22，2026/02/23，2026/02/24，2026/02/25，2026/03/14，2026/04/20，2026/06/16，2026/08/01，2026/08/27</t>
+          <t>2026/02/22，2026/02/23，2026/02/24，2026/02/25，2026/03/14，2026/04/20，2026/06/16，2026/08/01，2026/08/27，2026/09/26</t>
         </is>
       </c>
       <c r="F798" t="inlineStr"/>
@@ -32390,7 +32398,7 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I798" t="inlineStr">
@@ -32587,7 +32595,7 @@
       </c>
       <c r="E803" t="inlineStr">
         <is>
-          <t>2026/03/01，2026/03/01，2026/03/01，2026/03/01，2026/03/01，2026/03/04，2026/03/05，2026/03/05，2026/03/06，2026/03/12，2026/03/21，2026/03/31，2026/04/20，2026/05/02，2026/05/06，2026/05/21，2026/05/26，2026/06/14，2026/07/16，2026/9/14，2026/9/14</t>
+          <t>2026/03/01，2026/03/01，2026/03/01，2026/03/01，2026/03/01，2026/03/04，2026/03/05，2026/03/05，2026/03/06，2026/03/12，2026/03/21，2026/03/31，2026/04/20，2026/05/02，2026/05/06，2026/05/21，2026/05/26，2026/06/14，2026/07/16，2026/09/14，2026/09/14</t>
         </is>
       </c>
       <c r="F803" t="inlineStr"/>
@@ -32963,7 +32971,7 @@
       </c>
       <c r="E812" t="inlineStr">
         <is>
-          <t>2026/03/13，2026/03/25，2026/03/28，2026/04/11，2026/04/20，2026/05/26，2026/07/05，2026/07/22</t>
+          <t>2026/03/13，2026/03/25，2026/03/28，2026/04/11，2026/04/20，2026/05/26，2026/07/05，2026/07/22，2026/09/23</t>
         </is>
       </c>
       <c r="F812" t="inlineStr"/>
@@ -32974,7 +32982,7 @@
       </c>
       <c r="H812" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I812" t="inlineStr">
@@ -33323,7 +33331,7 @@
       </c>
       <c r="E821" t="inlineStr">
         <is>
-          <t>2026/03/17，2026/06/17</t>
+          <t>2026/03/17，2026/06/17，2026/09/21</t>
         </is>
       </c>
       <c r="F821" t="inlineStr"/>
@@ -33334,7 +33342,7 @@
       </c>
       <c r="H821" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I821" t="inlineStr">
@@ -34907,7 +34915,7 @@
       </c>
       <c r="E859" t="inlineStr">
         <is>
-          <t>2026/05/25，2026/05/25，2026/05/25，2026/05/26，2026/05/26，2026/06/25，2026/06/26，2026/07/09，2026/07/16，2026/08/23，2026/08/23，2026/09/11</t>
+          <t>2026/05/25，2026/05/25，2026/05/25，2026/05/26，2026/05/26，2026/06/25，2026/06/26，2026/07/09，2026/07/16，2026/08/23，2026/08/23，2026/09/11，2026/09/23</t>
         </is>
       </c>
       <c r="F859" t="inlineStr"/>
@@ -34918,7 +34926,7 @@
       </c>
       <c r="H859" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I859" t="inlineStr">
@@ -34951,7 +34959,7 @@
       </c>
       <c r="E860" t="inlineStr">
         <is>
-          <t>2026/05/25，2026/05/26，2026/06/15，2026/08/02</t>
+          <t>2026/05/25，2026/05/26，2026/06/15，2026/08/02，2026/09/22</t>
         </is>
       </c>
       <c r="F860" t="inlineStr"/>
@@ -34962,7 +34970,7 @@
       </c>
       <c r="H860" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I860" t="inlineStr">
@@ -35275,7 +35283,7 @@
       </c>
       <c r="E868" t="inlineStr">
         <is>
-          <t>2026/06/16，2026/06/17，2026/06/25</t>
+          <t>2026/06/16，2026/06/17，2026/06/25，2026/09/21</t>
         </is>
       </c>
       <c r="F868" t="inlineStr"/>
@@ -35286,7 +35294,7 @@
       </c>
       <c r="H868" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I868" t="inlineStr">
@@ -35603,7 +35611,7 @@
       </c>
       <c r="E876" t="inlineStr">
         <is>
-          <t>2026/07/05，2026/07/07，2026/07/17</t>
+          <t>2026/07/05，2026/07/07，2026/07/17，2026/09/23</t>
         </is>
       </c>
       <c r="F876" t="inlineStr"/>
@@ -35614,7 +35622,7 @@
       </c>
       <c r="H876" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I876" t="inlineStr">
@@ -35767,7 +35775,7 @@
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08，2026/08/28，2026/9/14</t>
+          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08，2026/08/28，2026/09/14</t>
         </is>
       </c>
       <c r="F880" t="inlineStr"/>
@@ -35971,7 +35979,7 @@
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>2026/08/03，2026/08/08，2026/08/09，2026/08/11，2026/08/18，2026/08/25，2026/09/08</t>
+          <t>2026/08/03，2026/08/08，2026/08/09，2026/08/11，2026/08/18，2026/08/25，2026/09/08，2026/09/22</t>
         </is>
       </c>
       <c r="F885" t="inlineStr"/>
@@ -35982,7 +35990,7 @@
       </c>
       <c r="H885" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I885" t="inlineStr">
@@ -36091,7 +36099,7 @@
       </c>
       <c r="E888" t="inlineStr">
         <is>
-          <t>2026/08/11，2026/08/11，2026/08/18，2026/08/25，2026/09/06，2026/09/11，2026/9/14</t>
+          <t>2026/08/11，2026/08/11，2026/08/18，2026/08/25，2026/09/06，2026/09/11，2026/09/14，2026/09/21</t>
         </is>
       </c>
       <c r="F888" t="inlineStr"/>
@@ -36102,7 +36110,7 @@
       </c>
       <c r="H888" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I888" t="inlineStr">
@@ -36415,7 +36423,7 @@
       </c>
       <c r="E896" t="inlineStr">
         <is>
-          <t>2026/08/23，2026/08/25，2026/09/02，2026/09/11</t>
+          <t>2026/08/23，2026/08/25，2026/09/02，2026/09/11，2026/09/21</t>
         </is>
       </c>
       <c r="F896" t="inlineStr"/>
@@ -36426,7 +36434,7 @@
       </c>
       <c r="H896" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I896" t="inlineStr">
@@ -36495,7 +36503,7 @@
       </c>
       <c r="E898" t="inlineStr">
         <is>
-          <t>2026/08/23</t>
+          <t>2026/08/23，2026/09/21，2026/09/26</t>
         </is>
       </c>
       <c r="F898" t="inlineStr"/>
@@ -36506,7 +36514,7 @@
       </c>
       <c r="H898" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I898" t="inlineStr">
@@ -36859,7 +36867,7 @@
       </c>
       <c r="E907" t="inlineStr">
         <is>
-          <t>2026/09/06，2026/09/11</t>
+          <t>2026/09/06，2026/09/11，2026/09/16</t>
         </is>
       </c>
       <c r="F907" t="inlineStr"/>
@@ -36870,7 +36878,7 @@
       </c>
       <c r="H907" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I907" t="inlineStr">
@@ -36903,7 +36911,7 @@
       </c>
       <c r="E908" t="inlineStr">
         <is>
-          <t>2026/09/13</t>
+          <t>2026/09/13，2026/09/21</t>
         </is>
       </c>
       <c r="F908" t="inlineStr"/>
@@ -36914,7 +36922,7 @@
       </c>
       <c r="H908" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I908" t="inlineStr">
@@ -36943,7 +36951,7 @@
       </c>
       <c r="E909" t="inlineStr">
         <is>
-          <t>2026/09/04</t>
+          <t>2026/09/04，2026/09/16，2026/09/22</t>
         </is>
       </c>
       <c r="F909" t="inlineStr"/>
@@ -36954,7 +36962,7 @@
       </c>
       <c r="H909" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I909" t="inlineStr">
@@ -36975,7 +36983,11 @@
           <t>Better Dig Two</t>
         </is>
       </c>
-      <c r="C910" t="inlineStr"/>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>最好挖两座坟</t>
+        </is>
+      </c>
       <c r="D910" t="inlineStr">
         <is>
           <t>The Band Perry</t>
@@ -37003,6 +37015,202 @@
         </is>
       </c>
       <c r="J910" t="inlineStr"/>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>910</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Let Her Go</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr"/>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr"/>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I911" t="inlineStr">
+        <is>
+          <t>BV1MBeA6CEhH</t>
+        </is>
+      </c>
+      <c r="J911" t="inlineStr"/>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>911</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Say Something</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr"/>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>A Great Big World</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>2026/09/16</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr"/>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I912" t="inlineStr">
+        <is>
+          <t>BV1d7eg6gEGu</t>
+        </is>
+      </c>
+      <c r="J912" t="inlineStr"/>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>912</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>U&amp;I</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr"/>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>放課後ティータイム</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>2026/09/21</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr"/>
+      <c r="G913" t="inlineStr">
+        <is>
+          <t>日语</t>
+        </is>
+      </c>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I913" t="inlineStr">
+        <is>
+          <t>BV1mzht6MEds</t>
+        </is>
+      </c>
+      <c r="J913" t="inlineStr"/>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>913</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>天天</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr"/>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>陶喆</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>2026/09/21</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr"/>
+      <c r="G914" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H914" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I914" t="inlineStr">
+        <is>
+          <t>BV1kThz6fEeg</t>
+        </is>
+      </c>
+      <c r="J914" t="inlineStr"/>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>914</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>荷塘月色</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr"/>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>凤凰传奇</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>2026/09/26</t>
+        </is>
+      </c>
+      <c r="F915" t="inlineStr"/>
+      <c r="G915" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I915" t="inlineStr"/>
+      <c r="J915" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>